<commit_message>
pipeline: integrar firmas_anexo3 + 4 columnas Excel
- scripts/ingest_expedientes.py: llama validaciones.firmas_anexo3 tras
  la extracción si tipo_detectado == "rendicion". Desacoplado: import
  try/except; flag --skip-validaciones; el pipeline sigue si el módulo
  falla (validaciones = null en el JSON).
- scripts/ingesta/excel_export.py: DocumentoValidacion ampliado con
  validacion_firmas, estado_firmas, errores_firmas, confianza_firmas.
- Excel: 24 columnas (20 + 4 firmas); upsert preserva columnas humanas.

Corrida sobre DIED2026-INT-0250235:
  - PV617 (solicitud) → firmas no aplican (celdas vacías, correcto)
  - RENDIC (rendicion) → validacion_firmas=firmas_anexo3,
    estado=INSUFICIENTE_EVIDENCIA, errores listados, confianza=0.1.

JSON en extractions/ con traza completa (firmantes, anchor, evidencia).

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/piloto_ocr/metrics/validacion_expedientes.xlsx
+++ b/data/piloto_ocr/metrics/validacion_expedientes.xlsx
@@ -12,9 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="errores" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'documentos'!$A$1:$T$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'documentos'!$A$1:$X$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'expedientes'!$A$1:$I$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'errores'!$A$1:$T$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'errores'!$A$1:$X$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:X3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -458,11 +458,15 @@
     <col width="18" customWidth="1" min="13" max="13"/>
     <col width="40" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="40" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
-    <col width="40" customWidth="1" min="19" max="19"/>
-    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="40" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -538,30 +542,50 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
+          <t>validacion_firmas</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>estado_firmas</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>errores_firmas</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>confianza_firmas</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
           <t>tipo_correcto</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>monto_correcto</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>fecha_correcta</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>ruc_correcto</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>observaciones</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>validacion_final</t>
         </is>
@@ -617,12 +641,16 @@
         </is>
       </c>
       <c r="N2" t="inlineStr"/>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="3" t="n"/>
-      <c r="Q2" s="3" t="n"/>
-      <c r="R2" s="3" t="n"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
       <c r="S2" s="3" t="n"/>
       <c r="T2" s="3" t="n"/>
+      <c r="U2" s="3" t="n"/>
+      <c r="V2" s="3" t="n"/>
+      <c r="W2" s="3" t="n"/>
+      <c r="X2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -673,15 +701,33 @@
           <t>override_consolidado_rendicion: top_regex=factura(33) pero filename+encabezado indican rendicion(24)</t>
         </is>
       </c>
-      <c r="O3" s="3" t="n"/>
-      <c r="P3" s="3" t="n"/>
-      <c r="Q3" s="3" t="n"/>
-      <c r="R3" s="3" t="n"/>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>firmas_anexo3</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>INSUFICIENTE_EVIDENCIA</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>nombre_ilegible:comisionado:anchor=dni_sin_nombre_adyacente; nombre_ilegible:jefe_unidad:anchor=sin_anchor; rol_no_detectado:vb_coordinador</t>
+        </is>
+      </c>
+      <c r="R3" t="n">
+        <v>0.1</v>
+      </c>
       <c r="S3" s="3" t="n"/>
       <c r="T3" s="3" t="n"/>
+      <c r="U3" s="3" t="n"/>
+      <c r="V3" s="3" t="n"/>
+      <c r="W3" s="3" t="n"/>
+      <c r="X3" s="3" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T3"/>
+  <autoFilter ref="A1:X3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -788,7 +834,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-04-14T12:18:18-0500</t>
+          <t>2026-04-14T13:02:24-0500</t>
         </is>
       </c>
     </row>
@@ -804,7 +850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1"/>
+  <dimension ref="A1:X1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -822,11 +868,15 @@
     <col width="18" customWidth="1" min="13" max="13"/>
     <col width="40" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="40" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
-    <col width="40" customWidth="1" min="19" max="19"/>
-    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="40" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -902,37 +952,57 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
+          <t>validacion_firmas</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>estado_firmas</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>errores_firmas</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>confianza_firmas</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
           <t>tipo_correcto</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>monto_correcto</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>fecha_correcta</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>ruc_correcto</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>observaciones</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>validacion_final</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T1"/>
+  <autoFilter ref="A1:X1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
identidad (4/6): Excel +9 columnas + hoja resolucion_ids
- DocumentoValidacion ampliado con expediente_detectado, sinad_detectado,
  siaf_detectado, anio_detectado, confianza_expediente/sinad/siaf,
  conflicto_expediente, observaciones_expediente.
- Nueva hoja `resolucion_ids`: una fila por candidato por expediente,
  con id_canonico, tipo, frecuencia, score_total, es_ganador,
  coincide_con_carpeta, estado_resolucion, fuentes (archivo:página).
- CandidatoResolucion dataclass + _cmd_export lee expediente.json y
  mapea resolución + candidatos al Excel.

Corrida sobre DIED2026-INT-0250235:
  - documentos: 33 columnas (24 anteriores + 9 nuevas)
  - ambos PDFs muestran expediente_detectado=SINAD-250235,
    sinad=250235 (0.87), siaf=2603426 (0.94), anio=2026.
  - hoja resolucion_ids: 5 candidatos ordenados por score.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/piloto_ocr/metrics/validacion_expedientes.xlsx
+++ b/data/piloto_ocr/metrics/validacion_expedientes.xlsx
@@ -10,11 +10,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="documentos" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="expedientes" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="errores" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="resolucion_ids" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'documentos'!$A$1:$X$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'documentos'!$A$1:$AG$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'expedientes'!$A$1:$I$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'errores'!$A$1:$X$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'errores'!$A$1:$AG$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'resolucion_ids'!$A$1:$I$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X3"/>
+  <dimension ref="A1:AG3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -461,12 +463,21 @@
     <col width="22" customWidth="1" min="16" max="16"/>
     <col width="40" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="16" customWidth="1" min="22" max="22"/>
-    <col width="40" customWidth="1" min="23" max="23"/>
-    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="16" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="25" max="25"/>
+    <col width="18" customWidth="1" min="26" max="26"/>
+    <col width="40" customWidth="1" min="27" max="27"/>
+    <col width="18" customWidth="1" min="28" max="28"/>
+    <col width="14" customWidth="1" min="29" max="29"/>
+    <col width="14" customWidth="1" min="30" max="30"/>
+    <col width="16" customWidth="1" min="31" max="31"/>
+    <col width="40" customWidth="1" min="32" max="32"/>
+    <col width="18" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -562,30 +573,75 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
+          <t>expediente_detectado</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>sinad_detectado</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>siaf_detectado</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>anio_detectado</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>confianza_expediente</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>confianza_sinad</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>confianza_siaf</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>conflicto_expediente</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>observaciones_expediente</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
           <t>tipo_correcto</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>monto_correcto</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>fecha_correcta</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>ruc_correcto</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>observaciones</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>validacion_final</t>
         </is>
@@ -645,12 +701,47 @@
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
-      <c r="S2" s="3" t="n"/>
-      <c r="T2" s="3" t="n"/>
-      <c r="U2" s="3" t="n"/>
-      <c r="V2" s="3" t="n"/>
-      <c r="W2" s="3" t="n"/>
-      <c r="X2" s="3" t="n"/>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>SINAD-250235</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>250235</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>2603426</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="W2" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" s="3" t="n"/>
+      <c r="AC2" s="3" t="n"/>
+      <c r="AD2" s="3" t="n"/>
+      <c r="AE2" s="3" t="n"/>
+      <c r="AF2" s="3" t="n"/>
+      <c r="AG2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -719,15 +810,50 @@
       <c r="R3" t="n">
         <v>0.1</v>
       </c>
-      <c r="S3" s="3" t="n"/>
-      <c r="T3" s="3" t="n"/>
-      <c r="U3" s="3" t="n"/>
-      <c r="V3" s="3" t="n"/>
-      <c r="W3" s="3" t="n"/>
-      <c r="X3" s="3" t="n"/>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>SINAD-250235</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>250235</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>2603426</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="W3" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" s="3" t="n"/>
+      <c r="AC3" s="3" t="n"/>
+      <c r="AD3" s="3" t="n"/>
+      <c r="AE3" s="3" t="n"/>
+      <c r="AF3" s="3" t="n"/>
+      <c r="AG3" s="3" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X3"/>
+  <autoFilter ref="A1:AG3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -834,7 +960,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-04-14T13:02:24-0500</t>
+          <t>2026-04-14T15:41:01-0500</t>
         </is>
       </c>
     </row>
@@ -850,7 +976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -871,12 +997,21 @@
     <col width="22" customWidth="1" min="16" max="16"/>
     <col width="40" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="16" customWidth="1" min="22" max="22"/>
-    <col width="40" customWidth="1" min="23" max="23"/>
-    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="16" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="25" max="25"/>
+    <col width="18" customWidth="1" min="26" max="26"/>
+    <col width="40" customWidth="1" min="27" max="27"/>
+    <col width="18" customWidth="1" min="28" max="28"/>
+    <col width="14" customWidth="1" min="29" max="29"/>
+    <col width="14" customWidth="1" min="30" max="30"/>
+    <col width="16" customWidth="1" min="31" max="31"/>
+    <col width="40" customWidth="1" min="32" max="32"/>
+    <col width="18" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -972,37 +1107,370 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
+          <t>expediente_detectado</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>sinad_detectado</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>siaf_detectado</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>anio_detectado</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>confianza_expediente</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>confianza_sinad</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>confianza_siaf</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>conflicto_expediente</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>observaciones_expediente</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
           <t>tipo_correcto</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>monto_correcto</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>fecha_correcta</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>ruc_correcto</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>observaciones</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>validacion_final</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X1"/>
+  <autoFilter ref="A1:AG1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>expediente_carpeta</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>id_canonico</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>tipo</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>frecuencia</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>score_total</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>coincide_con_carpeta</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>es_ganador</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>estado_resolucion</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>fuentes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SINAD-250235</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>sinad</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" t="n">
+        <v>106</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1; 20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p2; 20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p3; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p1; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ANIO-2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>anio</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" t="n">
+        <v>22</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1; 20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1; 20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p1; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SIAF-2603426</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>siaf</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" t="n">
+        <v>16</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p1; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SINAD-112591</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>sinad</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>15</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p9</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PEDIDO-572</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>pedido</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
regen Excel tras text_reader v2 sobre DIED2026-INT-0250235
Re-corrida completa (scan→process→consolidate→export) con OCR por-página:
- documentos: expediente_detectado=SINAD-250235 (conf 0.91, antes 0.87)
  con columna conflicto_expediente=Sí (SIAF 2603426 vs SIAF 3205).
- hoja resolucion_ids: 7 candidatos (antes 5). Nuevos:
  * EXP-DIED-2026-250235 (tipo=exp, score=16) — detectado en p8 del
    RENDIC tras OCR de páginas escaneadas; antes solo estaba en carpeta.
  * SIAF-3205 — Expediente SIAF del movimiento contable (0000003205-0003),
    distinto del N° Exp SIAF del viático (2603426). Ambos reales.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/piloto_ocr/metrics/validacion_expedientes.xlsx
+++ b/data/piloto_ocr/metrics/validacion_expedientes.xlsx
@@ -16,7 +16,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'documentos'!$A$1:$AG$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'expedientes'!$A$1:$I$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'errores'!$A$1:$AG$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'resolucion_ids'!$A$1:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'resolucion_ids'!$A$1:$I$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -722,20 +722,24 @@
         </is>
       </c>
       <c r="W2" t="n">
-        <v>0.869</v>
+        <v>0.838</v>
       </c>
       <c r="X2" t="n">
-        <v>0.869</v>
+        <v>0.912</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.485</v>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>siaf:conflicto: top=SIAF-2603426(16.0) vs segundo=SIAF-3205(16.0)</t>
+        </is>
+      </c>
       <c r="AB2" s="3" t="n"/>
       <c r="AC2" s="3" t="n"/>
       <c r="AD2" s="3" t="n"/>
@@ -789,7 +793,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>override_consolidado_rendicion: top_regex=factura(33) pero filename+encabezado indican rendicion(24)</t>
+          <t>override_consolidado_rendicion: top_regex=factura(45) pero filename+encabezado indican rendicion(24)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -831,20 +835,24 @@
         </is>
       </c>
       <c r="W3" t="n">
-        <v>0.869</v>
+        <v>0.838</v>
       </c>
       <c r="X3" t="n">
-        <v>0.869</v>
+        <v>0.912</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.485</v>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="AA3" t="inlineStr"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>siaf:conflicto: top=SIAF-2603426(16.0) vs segundo=SIAF-3205(16.0)</t>
+        </is>
+      </c>
       <c r="AB3" s="3" t="n"/>
       <c r="AC3" s="3" t="n"/>
       <c r="AD3" s="3" t="n"/>
@@ -960,7 +968,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-04-14T15:41:01-0500</t>
+          <t>2026-04-14T16:39:29-0500</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1271,10 +1279,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E2" t="n">
-        <v>106</v>
+        <v>166</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1288,7 +1296,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>CONFLICTO_EXPEDIENTE</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1314,10 +1322,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E3" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1331,12 +1339,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>CONFLICTO_EXPEDIENTE</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1; 20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1; 20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p1; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p1</t>
+          <t>20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1; 20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1; 20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p8; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p1</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1382,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>CONFLICTO_EXPEDIENTE</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1391,19 +1399,19 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SINAD-112591</t>
+          <t>SIAF-3205</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>sinad</t>
+          <t>siaf</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1417,12 +1425,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>CONFLICTO_EXPEDIENTE</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p9</t>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p8; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p150</t>
         </is>
       </c>
     </row>
@@ -1434,19 +1442,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PEDIDO-572</t>
+          <t>EXP-DIED-2026-250235</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pedido</t>
+          <t>exp</t>
         </is>
       </c>
       <c r="D6" t="n">
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1460,17 +1468,103 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>CONFLICTO_EXPEDIENTE</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1</t>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p8</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SINAD-112591</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>sinad</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>15</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>CONFLICTO_EXPEDIENTE</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p9</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>PEDIDO-572</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>pedido</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>7</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>CONFLICTO_EXPEDIENTE</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p3</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I6"/>
+  <autoFilter ref="A1:I8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
comprobantes (4/5): Excel — hoja `comprobantes` + columnas humanas
- scripts/ingesta/excel_export.py:
  * Dataclass ComprobanteExcel (14 columnas de sistema + 5 humanas:
    monto_correcto, ruc_correcto, proveedor_correcto, observaciones,
    validacion_final) — amarillo para validación humana.
  * Upsert por (expediente_id, archivo, pagina_inicio, pagina_fin);
    columnas humanas se preservan entre re-exports.
  * Nueva hoja ordenada al final: documentos, expedientes, errores,
    resolucion_ids, comprobantes.
- scripts/ingest_expedientes.py: _cmd_export lee `comprobantes` del
  expediente.json y los mapea a la hoja.

Corrida sobre DIED2026-INT-0250235:
  hoja `comprobantes`: 34 filas (21 facturas + 13 boletas),
  con RUC, razón social (cuando PASO 4.1 la captura) y texto_resumen
  para revisión humana.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/piloto_ocr/metrics/validacion_expedientes.xlsx
+++ b/data/piloto_ocr/metrics/validacion_expedientes.xlsx
@@ -11,12 +11,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="expedientes" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="errores" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="resolucion_ids" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="comprobantes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'documentos'!$A$1:$AG$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'expedientes'!$A$1:$I$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'errores'!$A$1:$AG$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'resolucion_ids'!$A$1:$I$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'comprobantes'!$A$1:$S$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1567,4 +1569,2043 @@
   <autoFilter ref="A1:I8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
+    <col width="40" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>expediente_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>archivo</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>pagina_inicio</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>pagina_fin</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>tipo</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>ruc</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>razon_social</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>serie_numero</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>fecha</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>monto_total</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>moneda</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>monto_igv</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>confianza</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>texto_resumen</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>monto_correcto</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>ruc_correcto</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>proveedor_correcto</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>observaciones</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>validacion_final</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>boleta_venta</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>E001-16</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>ANEXO N°3 Fecha : Hora : Página : 1 de 2 09/04/2026 13:01 Sistema Integrado de Gestión Módulo de Tesorería Versión 22.04.00 026 PROGRAMA EDUCACION BASICA PARA TODOS - 026 000081 Datos del CHAVEZ TERRONES LILIANA Sr(a): N° Planilla: Motivo de Salida: 00617 N° Exp SIAF: 2603426 N° Comprobante 09/03/20</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr"/>
+      <c r="P2" s="3" t="inlineStr"/>
+      <c r="Q2" s="3" t="inlineStr"/>
+      <c r="R2" s="3" t="inlineStr"/>
+      <c r="S2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>27</v>
+      </c>
+      <c r="D3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>20477689699</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>20477689699 - INVERSIONES &amp; SERVICIOS MULTIPLES COQUITO S.A.C.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2012-04-24</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica FA01-0000007538 es un comprobante de pago válido. 8/4/26, 12:40 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1 Consulta RUC Resultado de la Búsque</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr"/>
+      <c r="P3" s="3" t="inlineStr"/>
+      <c r="Q3" s="3" t="inlineStr"/>
+      <c r="R3" s="3" t="inlineStr"/>
+      <c r="S3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>29</v>
+      </c>
+      <c r="D4" t="n">
+        <v>30</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>boleta_venta</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>20539971477</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Cebicheria Coquito SAC.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>98.64</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>Fecha consulta: 08/04/2026 12:19 BOLETA DE VENTA GUIA DE REMISION - REMITENTE GUIA DE REMISION - TRANSPORTISTA Sistema de Emisión Electrónica: FACTURA PORTAL DESDE 15/05/2023 DESDE LOS SISTEMAS DEL CONTRIBUYENTE. AUTORIZ DESDE 29/04/2019 SEE-FACTURADOR . AUTORIZ DESDE 29/04/2019 Emisor electrónico d</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr"/>
+      <c r="P4" s="3" t="inlineStr"/>
+      <c r="Q4" s="3" t="inlineStr"/>
+      <c r="R4" s="3" t="inlineStr"/>
+      <c r="S4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>31</v>
+      </c>
+      <c r="D5" t="n">
+        <v>32</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>20539971477</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>20539971477 - CEBICHERIA COQUITO S.A.C.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2013-01-08</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica FB02-0000007269 es un comprobante de pago válido. 8/4/26, 12:43 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1 Consulta RUC Resultado de la Búsque</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr"/>
+      <c r="P5" s="3" t="inlineStr"/>
+      <c r="Q5" s="3" t="inlineStr"/>
+      <c r="R5" s="3" t="inlineStr"/>
+      <c r="S5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>33</v>
+      </c>
+      <c r="D6" t="n">
+        <v>33</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>boleta_venta</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Fecha consulta: 08/04/2026 12:21</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>Fecha consulta: 08/04/2026 12:21 BOLETA DE VENTA Sistema de Emisión Electrónica: FACTURA PORTAL DESDE 10/09/2024 DESDE LOS SISTEMAS DEL CONTRIBUYENTE. AUTORIZ DESDE 05/03/2019 SEE-FACTURADOR . AUTORIZ DESDE 05/03/2019 Emisor electrónico desde: 05/03/2019 Comprobantes Electrónicos: FACTURA (desde 05/</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr"/>
+      <c r="P6" s="3" t="inlineStr"/>
+      <c r="Q6" s="3" t="inlineStr"/>
+      <c r="R6" s="3" t="inlineStr"/>
+      <c r="S6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>34</v>
+      </c>
+      <c r="D7" t="n">
+        <v>35</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>20608901460</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>DEGATTA PR¡HPNER¡¡</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>DEGATTA PR¡HPNER¡¡ Le INVERSIONES É,T:R Jiron Ayacucho: 521; fry eae Peru — Trujillo. . Rue: 20608901460 FACTURA ELECTRONICA FO03-0000002483 “Orden: ov-094765 Fecha de emision : 10-03-2026 he SALON) PRINCIP AL " Rur. 2038!1 795907 Razon social - “PROGRAMA EDUCACION BASICA PARA TO Bop CALs DEL COMERC</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr"/>
+      <c r="P7" s="3" t="inlineStr"/>
+      <c r="Q7" s="3" t="inlineStr"/>
+      <c r="R7" s="3" t="inlineStr"/>
+      <c r="S7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>36</v>
+      </c>
+      <c r="D8" t="n">
+        <v>36</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>boleta_venta</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>20608901460</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2021-12-23</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>Consulta RUC Resultado de la Búsqueda Número de RUC: 20608901460 - LLF INVERSIONES E.I.R.L. Tipo Contribuyente: EMPRESA INDIVIDUAL DE RESP. LTDA Nombre Comercial: DECATTA CAFE Fecha de Inscripción: 23/12/2021 Fecha de Inicio de Actividades: 22/12/2021 Estado del Contribuyente: ACTIVO Condición del C</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr"/>
+      <c r="P8" s="3" t="inlineStr"/>
+      <c r="Q8" s="3" t="inlineStr"/>
+      <c r="R8" s="3" t="inlineStr"/>
+      <c r="S8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>38</v>
+      </c>
+      <c r="D9" t="n">
+        <v>39</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>10181685510</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002114 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 11/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr"/>
+      <c r="P9" s="3" t="inlineStr"/>
+      <c r="Q9" s="3" t="inlineStr"/>
+      <c r="R9" s="3" t="inlineStr"/>
+      <c r="S9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>40</v>
+      </c>
+      <c r="D10" t="n">
+        <v>40</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>boleta_venta</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>10181685510</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2014-10-01</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>Consulta RUC Resultado de la Búsqueda Número de RUC: 10181685510 - JULCA ULLOA RONALD ALBERTO Tipo Contribuyente: PERSONA NATURAL CON NEGOCIO Tipo de Documento: DNI 18168551 - JULCA ULLOA, RONALD ALBERTO Nombre Comercial: EL AMARAL Fecha de Inscripción: 01/10/2014 Fecha de Inicio de Actividades: 01/</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr"/>
+      <c r="P10" s="3" t="inlineStr"/>
+      <c r="Q10" s="3" t="inlineStr"/>
+      <c r="R10" s="3" t="inlineStr"/>
+      <c r="S10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>47</v>
+      </c>
+      <c r="D11" t="n">
+        <v>48</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>20609385317</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>20609385317 - AR REPRESENTACIONES GASTRONÓMICAS S.A.C .</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>F006-00002488</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2022-04-21</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica F006-00002488 es un comprobante de pago válido. 8/4/26, 12:55 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1 Consulta RUC Resultado de la Búsqueda</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="inlineStr"/>
+      <c r="P11" s="3" t="inlineStr"/>
+      <c r="Q11" s="3" t="inlineStr"/>
+      <c r="R11" s="3" t="inlineStr"/>
+      <c r="S11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>51</v>
+      </c>
+      <c r="D12" t="n">
+        <v>52</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>20611728159</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>20611728159 - TARANTELLA TRX S.A.C</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>F001-00001460</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2023-10-23</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica F001-00001460 es un comprobante de pago válido. 8/4/26, 16:48 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1 Consulta RUC Resultado de la Búsqueda</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="inlineStr"/>
+      <c r="P12" s="3" t="inlineStr"/>
+      <c r="Q12" s="3" t="inlineStr"/>
+      <c r="R12" s="3" t="inlineStr"/>
+      <c r="S12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>55</v>
+      </c>
+      <c r="D13" t="n">
+        <v>55</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Consulta Validez del Comprobante</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>F003-2478</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica F003-2478 es un comprobante de pago válido. 9/4/26, 9:06 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="inlineStr"/>
+      <c r="P13" s="3" t="inlineStr"/>
+      <c r="Q13" s="3" t="inlineStr"/>
+      <c r="R13" s="3" t="inlineStr"/>
+      <c r="S13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>58</v>
+      </c>
+      <c r="D14" t="n">
+        <v>59</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>10181685510</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002135 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 15/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="inlineStr"/>
+      <c r="P14" s="3" t="inlineStr"/>
+      <c r="Q14" s="3" t="inlineStr"/>
+      <c r="R14" s="3" t="inlineStr"/>
+      <c r="S14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>66</v>
+      </c>
+      <c r="D15" t="n">
+        <v>68</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>boleta_venta</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>10181727883</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>BOLETA DE VENTA ELECTRONICA RUC: 10181727883 EB01-163 TAPIA MERINO GLADYS PATRICIA JR. LOS RUBIES 383 URB. SANTA INES TRUJILLO - TRUJILLO - LA LIBERTAD Fecha de Vencimiento Fecha de Emisión : 17/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Observación : S</t>
+        </is>
+      </c>
+      <c r="O15" s="3" t="inlineStr"/>
+      <c r="P15" s="3" t="inlineStr"/>
+      <c r="Q15" s="3" t="inlineStr"/>
+      <c r="R15" s="3" t="inlineStr"/>
+      <c r="S15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>75</v>
+      </c>
+      <c r="D16" t="n">
+        <v>76</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>20613429388</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>20613429388 - RAFO ALFARO CAFE S.A.C.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>F001-543</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2024-11-14</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica F001-543 es un comprobante de pago válido. 9/4/26, 9:13 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1 Consulta RUC Resultado de la Búsqueda Númer</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="inlineStr"/>
+      <c r="P16" s="3" t="inlineStr"/>
+      <c r="Q16" s="3" t="inlineStr"/>
+      <c r="R16" s="3" t="inlineStr"/>
+      <c r="S16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>78</v>
+      </c>
+      <c r="D17" t="n">
+        <v>79</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>10181685510</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002139 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 18/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+        </is>
+      </c>
+      <c r="O17" s="3" t="inlineStr"/>
+      <c r="P17" s="3" t="inlineStr"/>
+      <c r="Q17" s="3" t="inlineStr"/>
+      <c r="R17" s="3" t="inlineStr"/>
+      <c r="S17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>87</v>
+      </c>
+      <c r="D18" t="n">
+        <v>88</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>20607776912</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>20607776912 - QUE BONITA VECINDAD S.A.C.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2021-04-08</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica FW01-1136 es un comprobante de pago válido. 9/4/26, 9:17 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1 Consulta RUC Resultado de la Búsqueda Núme</t>
+        </is>
+      </c>
+      <c r="O18" s="3" t="inlineStr"/>
+      <c r="P18" s="3" t="inlineStr"/>
+      <c r="Q18" s="3" t="inlineStr"/>
+      <c r="R18" s="3" t="inlineStr"/>
+      <c r="S18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>91</v>
+      </c>
+      <c r="D19" t="n">
+        <v>92</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>20609888769</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>20609888769 - SABORES DE TRADICION PERUANA E.I.R.L.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2022-08-22</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica FW01-759 es un comprobante de pago válido. 9/4/26, 9:19 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1 Consulta RUC Resultado de la Búsqueda Númer</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="inlineStr"/>
+      <c r="P19" s="3" t="inlineStr"/>
+      <c r="Q19" s="3" t="inlineStr"/>
+      <c r="R19" s="3" t="inlineStr"/>
+      <c r="S19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>95</v>
+      </c>
+      <c r="D20" t="n">
+        <v>96</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>20615160653</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>20615160653 - DAMCO CAFE S.A.C.</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>F001-1258</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica F001-1258 es un comprobante de pago válido. 9/4/26, 9:21 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1 Consulta RUC Resultado de la Búsqueda Núme</t>
+        </is>
+      </c>
+      <c r="O20" s="3" t="inlineStr"/>
+      <c r="P20" s="3" t="inlineStr"/>
+      <c r="Q20" s="3" t="inlineStr"/>
+      <c r="R20" s="3" t="inlineStr"/>
+      <c r="S20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>99</v>
+      </c>
+      <c r="D21" t="n">
+        <v>100</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>20613176528</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>20613176528 - LA ESTAMPIDA DEL MALL S.A.C.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>F002-2057</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2024-09-20</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica F002-2057 es un comprobante de pago válido. 9/4/26, 9:23 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1 Consulta RUC Resultado de la Búsqueda Núme</t>
+        </is>
+      </c>
+      <c r="O21" s="3" t="inlineStr"/>
+      <c r="P21" s="3" t="inlineStr"/>
+      <c r="Q21" s="3" t="inlineStr"/>
+      <c r="R21" s="3" t="inlineStr"/>
+      <c r="S21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>103</v>
+      </c>
+      <c r="D22" t="n">
+        <v>103</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Consulta Validez del Comprobante</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>F018-26030</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica F018-26030 es un comprobante de pago válido. 9/4/26, 9:24 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1</t>
+        </is>
+      </c>
+      <c r="O22" s="3" t="inlineStr"/>
+      <c r="P22" s="3" t="inlineStr"/>
+      <c r="Q22" s="3" t="inlineStr"/>
+      <c r="R22" s="3" t="inlineStr"/>
+      <c r="S22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>104</v>
+      </c>
+      <c r="D23" t="n">
+        <v>104</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>boleta_venta</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>20600593685</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2015-08-14</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>Consulta RUC Resultado de la Búsqueda Número de RUC: 20600593685 - LUCHA PARTNERS S.A.C. Tipo Contribuyente: SOCIEDAD ANONIMA CERRADA Nombre Comercial: LA LUCHA,7 SOPAS,REPUBLICA,HER Fecha de Inscripción: 14/08/2015 Fecha de Inicio de Actividades: 01/09/2015 Estado del Contribuyente: ACTIVO Condició</t>
+        </is>
+      </c>
+      <c r="O23" s="3" t="inlineStr"/>
+      <c r="P23" s="3" t="inlineStr"/>
+      <c r="Q23" s="3" t="inlineStr"/>
+      <c r="R23" s="3" t="inlineStr"/>
+      <c r="S23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>111</v>
+      </c>
+      <c r="D24" t="n">
+        <v>111</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Consulta Validez del Comprobante</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>F002-2258</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica F002-2258 es un comprobante de pago válido. 9/4/26, 9:27 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1</t>
+        </is>
+      </c>
+      <c r="O24" s="3" t="inlineStr"/>
+      <c r="P24" s="3" t="inlineStr"/>
+      <c r="Q24" s="3" t="inlineStr"/>
+      <c r="R24" s="3" t="inlineStr"/>
+      <c r="S24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>112</v>
+      </c>
+      <c r="D25" t="n">
+        <v>112</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>boleta_venta</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>20601709016</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2016-12-05</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>Consulta RUC Resultado de la Búsqueda Número de RUC: 20601709016 - INVERSIONES CASA BLANCA A &amp; A S.A.C. Tipo Contribuyente: SOCIEDAD ANONIMA CERRADA Nombre Comercial: - Fecha de Inscripción: 05/12/2016 Fecha de Inicio de Actividades: 05/12/2016 Estado del Contribuyente: ACTIVO Condición del Contribu</t>
+        </is>
+      </c>
+      <c r="O25" s="3" t="inlineStr"/>
+      <c r="P25" s="3" t="inlineStr"/>
+      <c r="Q25" s="3" t="inlineStr"/>
+      <c r="R25" s="3" t="inlineStr"/>
+      <c r="S25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>117</v>
+      </c>
+      <c r="D26" t="n">
+        <v>117</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>boleta_venta</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Fecha consulta: 08/04/2026 12:34</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>Fecha consulta: 08/04/2026 12:34 BOLETA DE VENTA GUIA DE REMISION - REMITENTE GUIA DE REMISION - TRANSPORTISTA Sistema de Emisión Electrónica: FACTURA PORTAL DESDE 15/05/2023 DESDE LOS SISTEMAS DEL CONTRIBUYENTE. AUTORIZ DESDE 29/04/2019 SEE-FACTURADOR . AUTORIZ DESDE 29/04/2019 Emisor electrónico d</t>
+        </is>
+      </c>
+      <c r="O26" s="3" t="inlineStr"/>
+      <c r="P26" s="3" t="inlineStr"/>
+      <c r="Q26" s="3" t="inlineStr"/>
+      <c r="R26" s="3" t="inlineStr"/>
+      <c r="S26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>119</v>
+      </c>
+      <c r="D27" t="n">
+        <v>120</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>20202961518</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Consulta Validez del Comprobante</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>F219-11456</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>1994-01-02</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica F219-11456 es un comprobante de pago válido. 9/4/26, 9:29 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1 Consulta RUC Resultado de la Búsqueda Núm</t>
+        </is>
+      </c>
+      <c r="O27" s="3" t="inlineStr"/>
+      <c r="P27" s="3" t="inlineStr"/>
+      <c r="Q27" s="3" t="inlineStr"/>
+      <c r="R27" s="3" t="inlineStr"/>
+      <c r="S27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>121</v>
+      </c>
+      <c r="D28" t="n">
+        <v>123</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>boleta_venta</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>20380795907</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Fecha consulta: 08/04/2026 12:35</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>70.00</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>6.65</t>
+        </is>
+      </c>
+      <c r="M28" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fecha consulta: 08/04/2026 12:35 BOLETA DE VENTA NOTA DE CREDITO NOTA DE DEBITO GUIA DE REMISION - REMITENTE Sistema de Emisión Electrónica: FACTURA PORTAL DESDE 30/11/2021 DESDE LOS SISTEMAS DEL CONTRIBUYENTE. AUTORIZ DESDE 03/07/2018 Emisor electrónico desde: 03/07/2018 Comprobantes Electrónicos: </t>
+        </is>
+      </c>
+      <c r="O28" s="3" t="inlineStr"/>
+      <c r="P28" s="3" t="inlineStr"/>
+      <c r="Q28" s="3" t="inlineStr"/>
+      <c r="R28" s="3" t="inlineStr"/>
+      <c r="S28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>125</v>
+      </c>
+      <c r="D29" t="n">
+        <v>125</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>boleta_venta</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Fecha consulta: 08/04/2026 12:35</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fecha consulta: 08/04/2026 12:35 RECIBO POR HONORARIOS BOLETA DE VENTA Sistema de Emisión Electrónica: FACTURA PORTAL DESDE 17/06/2024 BOLETA PORTAL DESDE 26/05/2024 DESDE LOS SISTEMAS DEL CONTRIBUYENTE. AUTORIZ DESDE 07/02/2026 Emisor electrónico desde: 26/05/2024 Comprobantes Electrónicos: BOLETA </t>
+        </is>
+      </c>
+      <c r="O29" s="3" t="inlineStr"/>
+      <c r="P29" s="3" t="inlineStr"/>
+      <c r="Q29" s="3" t="inlineStr"/>
+      <c r="R29" s="3" t="inlineStr"/>
+      <c r="S29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>126</v>
+      </c>
+      <c r="D30" t="n">
+        <v>128</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>10427606037</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>TAXI ALMANZA</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>E001-16</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>80.00</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="n">
+        <v>1</v>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAXI ALMANZA ALMANZA MALLEA EDWIN FACTURA ELECTRONICA A.F. BELLA DURMIENTE PRIMERO MZA. Y LOTE. 11 ALT.AV. CANTO RUC: 10427606037 GRANDE CON AV. CANTO BELLO E001-16 SAN JUAN DE LURIGANCHO - LIMA - LIMA Fecha de Emisión : 09/03/2026 Forma de pago: Contado . PROGRAMA EDUCACION BASICA " PARA TODOS RUC </t>
+        </is>
+      </c>
+      <c r="O30" s="3" t="inlineStr"/>
+      <c r="P30" s="3" t="inlineStr"/>
+      <c r="Q30" s="3" t="inlineStr"/>
+      <c r="R30" s="3" t="inlineStr"/>
+      <c r="S30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>130</v>
+      </c>
+      <c r="D31" t="n">
+        <v>132</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>10181382941</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>A) 10181382941</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2006-09-20</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>A) 10181382941 Acuario "s SUITE FACTURA ELECTRONICA HOSPEDAJE ACUARIO'S SUITE Dirección : CALLE PRIMAVERA S/N SEC.LA ENCALADA DEL GOLF LA LIBERTAD - TRUJILLO - VICTOR LARCO HERRERA FAO 1 -85 Teléfonos : 065221356 Pagina web : hospedajeacuarios.efactur.pe Razón Social : PROGRAMA EDUCACION BASICA PARA</t>
+        </is>
+      </c>
+      <c r="O31" s="3" t="inlineStr"/>
+      <c r="P31" s="3" t="inlineStr"/>
+      <c r="Q31" s="3" t="inlineStr"/>
+      <c r="R31" s="3" t="inlineStr"/>
+      <c r="S31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>133</v>
+      </c>
+      <c r="D32" t="n">
+        <v>133</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>boleta_venta</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Fecha consulta: 08/04/2026 12:36</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>Fecha consulta: 08/04/2026 12:36 BOLETA DE VENTA Sistema de Emisión Electrónica: DESDE LOS SISTEMAS DEL CONTRIBUYENTE. AUTORIZ DESDE 30/12/2020 Emisor electrónico desde: 30/12/2020 Comprobantes Electrónicos: FACTURA (desde 30/12/2020),BOLETA (desde 30/12/2020) Afiliado al PLE desde: - Padrones: NING</t>
+        </is>
+      </c>
+      <c r="O32" s="3" t="inlineStr"/>
+      <c r="P32" s="3" t="inlineStr"/>
+      <c r="Q32" s="3" t="inlineStr"/>
+      <c r="R32" s="3" t="inlineStr"/>
+      <c r="S32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>134</v>
+      </c>
+      <c r="D33" t="n">
+        <v>135</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>20131525193</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>HOSPEDAJE EL PALACIO</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>E001-968</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>HOSPEDAJE EL PALACIO SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA. JR. GRAU 709 TRUJILLO - TRUJILLO - LA LIBERTAD FACTURA ELECTRONICA RUC: 20131525193 E001-968 Fecha de Emisión : 21/03/2026 Forma de pago: Contado Señor(es) . PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 . JR. GRAU 709 LA LIBERTAD</t>
+        </is>
+      </c>
+      <c r="O33" s="3" t="inlineStr"/>
+      <c r="P33" s="3" t="inlineStr"/>
+      <c r="Q33" s="3" t="inlineStr"/>
+      <c r="R33" s="3" t="inlineStr"/>
+      <c r="S33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>136</v>
+      </c>
+      <c r="D34" t="n">
+        <v>136</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>boleta_venta</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>20131525193</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Resultado de la Búsqueda</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>1993-05-06</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>Consulta RUC Resultado de la Búsqueda Número de RUC: 20131525193 - SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA. Tipo Contribuyente: SOC.COM.RESPONS. LTDA Nombre Comercial: HOSPEDAJE EL PALACIO Fecha de Inscripción: 06/05/1993 Fecha de Inicio de Actividades: 01/03/1991 Estado del Contribuyente: ACTIVO Con</t>
+        </is>
+      </c>
+      <c r="O34" s="3" t="inlineStr"/>
+      <c r="P34" s="3" t="inlineStr"/>
+      <c r="Q34" s="3" t="inlineStr"/>
+      <c r="R34" s="3" t="inlineStr"/>
+      <c r="S34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>138</v>
+      </c>
+      <c r="D35" t="n">
+        <v>139</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>20131525193</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>HOSPEDAJE EL PALACIO</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>E001-970</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>180.00</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="n">
+        <v>1</v>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>HOSPEDAJE EL PALACIO SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA. JR. GRAU 709 TRUJILLO - TRUJILLO - LA LIBERTAD FACTURA ELECTRONICA RUC: 20131525193 E001-970 Fecha de Emisión : 23/03/2026 Forma de pago: Contado Señor(es) . PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 . JR. GRAU 709 LA LIBERTAD</t>
+        </is>
+      </c>
+      <c r="O35" s="3" t="inlineStr"/>
+      <c r="P35" s="3" t="inlineStr"/>
+      <c r="Q35" s="3" t="inlineStr"/>
+      <c r="R35" s="3" t="inlineStr"/>
+      <c r="S35" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:S35"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
rescate de cambios tras reinicio sin memoria
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/piloto_ocr/metrics/validacion_expedientes.xlsx
+++ b/data/piloto_ocr/metrics/validacion_expedientes.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'expedientes'!$A$1:$I$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'errores'!$A$1:$AG$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'resolucion_ids'!$A$1:$I$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'comprobantes'!$A$1:$S$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'comprobantes'!$A$1:$S$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -798,24 +798,10 @@
           <t>override_consolidado_rendicion: top_regex=factura(45) pero filename+encabezado indican rendicion(24)</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>firmas_anexo3</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>INSUFICIENTE_EVIDENCIA</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>nombre_ilegible:comisionado:anchor=dni_sin_nombre_adyacente; nombre_ilegible:jefe_unidad:anchor=sin_anchor; rol_no_detectado:vb_coordinador</t>
-        </is>
-      </c>
-      <c r="R3" t="n">
-        <v>0.1</v>
-      </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
           <t>SINAD-250235</t>
@@ -1577,7 +1563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S35"/>
+  <dimension ref="A1:S16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1765,10 +1751,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="D3" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1777,29 +1763,25 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>20477689699</t>
+          <t>20608901460</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>20477689699 - INVERSIONES &amp; SERVICIOS MULTIPLES COQUITO S.A.C.</t>
+          <t>DEGATTA PR¡HPNER¡¡</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2012-04-24</t>
-        </is>
-      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica FA01-0000007538 es un comprobante de pago válido. 8/4/26, 12:40 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1 Consulta RUC Resultado de la Búsque</t>
+          <t>DEGATTA PR¡HPNER¡¡ Le INVERSIONES É,T:R Jiron Ayacucho: 521; fry eae Peru — Trujillo. . Rue: 20608901460 FACTURA ELECTRONICA FO03-0000002483 “Orden: ov-094765 Fecha de emision : 10-03-2026 he SALON) PRINCIP AL " Rur. 2038!1 795907 Razon social - “PROGRAMA EDUCACION BASICA PARA TO Bop CALs DEL COMERC</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr"/>
@@ -1820,37 +1802,29 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="D4" t="n">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>boleta_venta</t>
+          <t>factura_electronica</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>20539971477</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Cebicheria Coquito SAC.</t>
-        </is>
-      </c>
+          <t>10181685510</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>98.64</t>
-        </is>
-      </c>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>PEN</t>
@@ -1858,11 +1832,11 @@
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Fecha consulta: 08/04/2026 12:19 BOLETA DE VENTA GUIA DE REMISION - REMITENTE GUIA DE REMISION - TRANSPORTISTA Sistema de Emisión Electrónica: FACTURA PORTAL DESDE 15/05/2023 DESDE LOS SISTEMAS DEL CONTRIBUYENTE. AUTORIZ DESDE 29/04/2019 SEE-FACTURADOR . AUTORIZ DESDE 29/04/2019 Emisor electrónico d</t>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002114 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 11/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr"/>
@@ -1883,10 +1857,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="D5" t="n">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1895,29 +1869,29 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>20539971477</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>20539971477 - CEBICHERIA COQUITO S.A.C.</t>
-        </is>
-      </c>
+          <t>10181685510</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2013-01-08</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
         <v>0.5</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica FB02-0000007269 es un comprobante de pago válido. 8/4/26, 12:43 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1 Consulta RUC Resultado de la Búsque</t>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002122 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 11/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr"/>
@@ -1938,37 +1912,41 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="D6" t="n">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>boleta_venta</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Fecha consulta: 08/04/2026 12:21</t>
-        </is>
-      </c>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>10181685510</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>Fecha consulta: 08/04/2026 12:21 BOLETA DE VENTA Sistema de Emisión Electrónica: FACTURA PORTAL DESDE 10/09/2024 DESDE LOS SISTEMAS DEL CONTRIBUYENTE. AUTORIZ DESDE 05/03/2019 SEE-FACTURADOR . AUTORIZ DESDE 05/03/2019 Emisor electrónico desde: 05/03/2019 Comprobantes Electrónicos: FACTURA (desde 05/</t>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002135 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 15/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr"/>
@@ -1989,10 +1967,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>34</v>
+        <v>62</v>
       </c>
       <c r="D7" t="n">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -2001,25 +1979,25 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>20608901460</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>DEGATTA PR¡HPNER¡¡</t>
-        </is>
-      </c>
+          <t>10181685510</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>DEGATTA PR¡HPNER¡¡ Le INVERSIONES É,T:R Jiron Ayacucho: 521; fry eae Peru — Trujillo. . Rue: 20608901460 FACTURA ELECTRONICA FO03-0000002483 “Orden: ov-094765 Fecha de emision : 10-03-2026 he SALON) PRINCIP AL " Rur. 2038!1 795907 Razon social - “PROGRAMA EDUCACION BASICA PARA TO Bop CALs DEL COMERC</t>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002136 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 15/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
         </is>
       </c>
       <c r="O7" s="3" t="inlineStr"/>
@@ -2040,10 +2018,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="D8" t="n">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -2052,25 +2030,29 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>20608901460</t>
+          <t>10181727883</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2021-12-23</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
         <v>0.5</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Consulta RUC Resultado de la Búsqueda Número de RUC: 20608901460 - LLF INVERSIONES E.I.R.L. Tipo Contribuyente: EMPRESA INDIVIDUAL DE RESP. LTDA Nombre Comercial: DECATTA CAFE Fecha de Inscripción: 23/12/2021 Fecha de Inicio de Actividades: 22/12/2021 Estado del Contribuyente: ACTIVO Condición del C</t>
+          <t>BOLETA DE VENTA ELECTRONICA RUC: 10181727883 EB01-163 TAPIA MERINO GLADYS PATRICIA JR. LOS RUBIES 383 URB. SANTA INES TRUJILLO - TRUJILLO - LA LIBERTAD Fecha de Vencimiento Fecha de Emisión : 17/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Observación : S</t>
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr"/>
@@ -2091,26 +2073,26 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>38</v>
+        <v>70</v>
       </c>
       <c r="D9" t="n">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>factura_electronica</t>
+          <t>boleta_venta</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10181685510</t>
+          <t>10181727883</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -2125,7 +2107,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002114 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 11/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+          <t>BOLETA DE VENTA ELECTRONICA RUC: 10181727883 EB01-164 TAPIA MERINO GLADYS PATRICIA JR. LOS RUBIES 383 URB. SANTA INES TRUJILLO - TRUJILLO - LA LIBERTAD Fecha de Vencimiento Fecha de Emisión : 17/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Observación : S</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr"/>
@@ -2146,14 +2128,14 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>40</v>
+        <v>78</v>
       </c>
       <c r="D10" t="n">
-        <v>40</v>
+        <v>78</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>boleta_venta</t>
+          <t>factura_electronica</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -2165,18 +2147,22 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2014-10-01</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
         <v>0.5</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Consulta RUC Resultado de la Búsqueda Número de RUC: 10181685510 - JULCA ULLOA RONALD ALBERTO Tipo Contribuyente: PERSONA NATURAL CON NEGOCIO Tipo de Documento: DNI 18168551 - JULCA ULLOA, RONALD ALBERTO Nombre Comercial: EL AMARAL Fecha de Inscripción: 01/10/2014 Fecha de Inicio de Actividades: 01/</t>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002139 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 18/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr"/>
@@ -2197,10 +2183,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>47</v>
+        <v>82</v>
       </c>
       <c r="D11" t="n">
-        <v>48</v>
+        <v>82</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2209,33 +2195,29 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>20609385317</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>20609385317 - AR REPRESENTACIONES GASTRONÓMICAS S.A.C .</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>F006-00002488</t>
-        </is>
-      </c>
+          <t>10181685510</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2022-04-21</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica F006-00002488 es un comprobante de pago válido. 8/4/26, 12:55 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1 Consulta RUC Resultado de la Búsqueda</t>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002141 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 18/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr"/>
@@ -2256,45 +2238,41 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>51</v>
+        <v>122</v>
       </c>
       <c r="D12" t="n">
-        <v>52</v>
+        <v>122</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>factura_electronica</t>
+          <t>boleta_venta</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>20611728159</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>20611728159 - TARANTELLA TRX S.A.C</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>F001-00001460</t>
-        </is>
-      </c>
+          <t>20380795907</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2023-10-23</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica F001-00001460 es un comprobante de pago válido. 8/4/26, 16:48 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1 Consulta RUC Resultado de la Búsqueda</t>
+          <t xml:space="preserve">LA ESQUINA DEL ESTUDIANTE HERNANDEZ ALMENGOR SILVIA MARLENE BOLETAR%ECY,IE¿:;;OE,II;EÍIRONICA MZA. G INT. 2 PI LOTE. 1 URB. INGENIERIA E'Bº1 1390 TRUJILLO - TRUJILLO - LA LIBERTAD - Fecha de Vencimiento Fecha de Emisión : 23/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de </t>
         </is>
       </c>
       <c r="O12" s="3" t="inlineStr"/>
@@ -2315,37 +2293,53 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>55</v>
+        <v>126</v>
       </c>
       <c r="D13" t="n">
-        <v>55</v>
+        <v>126</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
           <t>factura_electronica</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>10427606037</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Consulta Validez del Comprobante</t>
+          <t>TAXI ALMANZA</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>F003-2478</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
+          <t>E001-16</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>80.00</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica F003-2478 es un comprobante de pago válido. 9/4/26, 9:06 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1</t>
+          <t xml:space="preserve">TAXI ALMANZA ALMANZA MALLEA EDWIN FACTURA ELECTRONICA A.F. BELLA DURMIENTE PRIMERO MZA. Y LOTE. 11 ALT.AV. CANTO RUC: 10427606037 GRANDE CON AV. CANTO BELLO E001-16 SAN JUAN DE LURIGANCHO - LIMA - LIMA Fecha de Emisión : 09/03/2026 Forma de pago: Contado . PROGRAMA EDUCACION BASICA " PARA TODOS RUC </t>
         </is>
       </c>
       <c r="O13" s="3" t="inlineStr"/>
@@ -2366,10 +2360,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>58</v>
+        <v>130</v>
       </c>
       <c r="D14" t="n">
-        <v>59</v>
+        <v>130</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2378,16 +2372,16 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>10181685510</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr"/>
+          <t>10181382941</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>A) 10181382941</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>2026-03-15</t>
-        </is>
-      </c>
+      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
@@ -2396,11 +2390,11 @@
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002135 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 15/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+          <t>A) 10181382941 Acuario "s SUITE FACTURA ELECTRONICA HOSPEDAJE ACUARIO'S SUITE Dirección : CALLE PRIMAVERA S/N SEC.LA ENCALADA DEL GOLF LA LIBERTAD - TRUJILLO - VICTOR LARCO HERRERA FAO 1 -85 Teléfonos : 065221356 Pagina web : hospedajeacuarios.efactur.pe Razón Social : PROGRAMA EDUCACION BASICA PARA</t>
         </is>
       </c>
       <c r="O14" s="3" t="inlineStr"/>
@@ -2421,26 +2415,34 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>66</v>
+        <v>134</v>
       </c>
       <c r="D15" t="n">
-        <v>68</v>
+        <v>134</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>boleta_venta</t>
+          <t>factura_electronica</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>10181727883</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
+          <t>20131525193</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>HOSPEDAJE EL PALACIO</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>E001-968</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -2451,11 +2453,11 @@
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>BOLETA DE VENTA ELECTRONICA RUC: 10181727883 EB01-163 TAPIA MERINO GLADYS PATRICIA JR. LOS RUBIES 383 URB. SANTA INES TRUJILLO - TRUJILLO - LA LIBERTAD Fecha de Vencimiento Fecha de Emisión : 17/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Observación : S</t>
+          <t>HOSPEDAJE EL PALACIO SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA. JR. GRAU 709 TRUJILLO - TRUJILLO - LA LIBERTAD FACTURA ELECTRONICA RUC: 20131525193 E001-968 Fecha de Emisión : 21/03/2026 Forma de pago: Contado Señor(es) . PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 . JR. GRAU 709 LA LIBERTAD</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr"/>
@@ -2476,10 +2478,10 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>75</v>
+        <v>138</v>
       </c>
       <c r="D16" t="n">
-        <v>76</v>
+        <v>138</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2488,33 +2490,41 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>20613429388</t>
+          <t>20131525193</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>20613429388 - RAFO ALFARO CAFE S.A.C.</t>
+          <t>HOSPEDAJE EL PALACIO</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>F001-543</t>
+          <t>E001-970</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2024-11-14</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>180.00</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica F001-543 es un comprobante de pago válido. 9/4/26, 9:13 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1 Consulta RUC Resultado de la Búsqueda Númer</t>
+          <t>HOSPEDAJE EL PALACIO SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA. JR. GRAU 709 TRUJILLO - TRUJILLO - LA LIBERTAD FACTURA ELECTRONICA RUC: 20131525193 E001-970 Fecha de Emisión : 23/03/2026 Forma de pago: Contado Señor(es) . PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 . JR. GRAU 709 LA LIBERTAD</t>
         </is>
       </c>
       <c r="O16" s="3" t="inlineStr"/>
@@ -2523,1089 +2533,8 @@
       <c r="R16" s="3" t="inlineStr"/>
       <c r="S16" s="3" t="inlineStr"/>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>DIED2026-INT-0250235</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>78</v>
-      </c>
-      <c r="D17" t="n">
-        <v>79</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>factura_electronica</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>10181685510</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>2026-03-18</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002139 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 18/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
-        </is>
-      </c>
-      <c r="O17" s="3" t="inlineStr"/>
-      <c r="P17" s="3" t="inlineStr"/>
-      <c r="Q17" s="3" t="inlineStr"/>
-      <c r="R17" s="3" t="inlineStr"/>
-      <c r="S17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>DIED2026-INT-0250235</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>87</v>
-      </c>
-      <c r="D18" t="n">
-        <v>88</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>factura_electronica</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>20607776912</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>20607776912 - QUE BONITA VECINDAD S.A.C.</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>2021-04-08</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica FW01-1136 es un comprobante de pago válido. 9/4/26, 9:17 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1 Consulta RUC Resultado de la Búsqueda Núme</t>
-        </is>
-      </c>
-      <c r="O18" s="3" t="inlineStr"/>
-      <c r="P18" s="3" t="inlineStr"/>
-      <c r="Q18" s="3" t="inlineStr"/>
-      <c r="R18" s="3" t="inlineStr"/>
-      <c r="S18" s="3" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>DIED2026-INT-0250235</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>91</v>
-      </c>
-      <c r="D19" t="n">
-        <v>92</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>factura_electronica</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>20609888769</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>20609888769 - SABORES DE TRADICION PERUANA E.I.R.L.</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>2022-08-22</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica FW01-759 es un comprobante de pago válido. 9/4/26, 9:19 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1 Consulta RUC Resultado de la Búsqueda Númer</t>
-        </is>
-      </c>
-      <c r="O19" s="3" t="inlineStr"/>
-      <c r="P19" s="3" t="inlineStr"/>
-      <c r="Q19" s="3" t="inlineStr"/>
-      <c r="R19" s="3" t="inlineStr"/>
-      <c r="S19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>DIED2026-INT-0250235</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>95</v>
-      </c>
-      <c r="D20" t="n">
-        <v>96</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>factura_electronica</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>20615160653</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>20615160653 - DAMCO CAFE S.A.C.</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>F001-1258</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>2025-12-02</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica F001-1258 es un comprobante de pago válido. 9/4/26, 9:21 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1 Consulta RUC Resultado de la Búsqueda Núme</t>
-        </is>
-      </c>
-      <c r="O20" s="3" t="inlineStr"/>
-      <c r="P20" s="3" t="inlineStr"/>
-      <c r="Q20" s="3" t="inlineStr"/>
-      <c r="R20" s="3" t="inlineStr"/>
-      <c r="S20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>DIED2026-INT-0250235</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>99</v>
-      </c>
-      <c r="D21" t="n">
-        <v>100</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>factura_electronica</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>20613176528</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>20613176528 - LA ESTAMPIDA DEL MALL S.A.C.</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>F002-2057</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>2024-09-20</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="N21" s="2" t="inlineStr">
-        <is>
-          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica F002-2057 es un comprobante de pago válido. 9/4/26, 9:23 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1 Consulta RUC Resultado de la Búsqueda Núme</t>
-        </is>
-      </c>
-      <c r="O21" s="3" t="inlineStr"/>
-      <c r="P21" s="3" t="inlineStr"/>
-      <c r="Q21" s="3" t="inlineStr"/>
-      <c r="R21" s="3" t="inlineStr"/>
-      <c r="S21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>DIED2026-INT-0250235</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>103</v>
-      </c>
-      <c r="D22" t="n">
-        <v>103</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>factura_electronica</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Consulta Validez del Comprobante</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>F018-26030</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="N22" s="2" t="inlineStr">
-        <is>
-          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica F018-26030 es un comprobante de pago válido. 9/4/26, 9:24 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1</t>
-        </is>
-      </c>
-      <c r="O22" s="3" t="inlineStr"/>
-      <c r="P22" s="3" t="inlineStr"/>
-      <c r="Q22" s="3" t="inlineStr"/>
-      <c r="R22" s="3" t="inlineStr"/>
-      <c r="S22" s="3" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>DIED2026-INT-0250235</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>104</v>
-      </c>
-      <c r="D23" t="n">
-        <v>104</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>boleta_venta</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>20600593685</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>2015-08-14</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N23" s="2" t="inlineStr">
-        <is>
-          <t>Consulta RUC Resultado de la Búsqueda Número de RUC: 20600593685 - LUCHA PARTNERS S.A.C. Tipo Contribuyente: SOCIEDAD ANONIMA CERRADA Nombre Comercial: LA LUCHA,7 SOPAS,REPUBLICA,HER Fecha de Inscripción: 14/08/2015 Fecha de Inicio de Actividades: 01/09/2015 Estado del Contribuyente: ACTIVO Condició</t>
-        </is>
-      </c>
-      <c r="O23" s="3" t="inlineStr"/>
-      <c r="P23" s="3" t="inlineStr"/>
-      <c r="Q23" s="3" t="inlineStr"/>
-      <c r="R23" s="3" t="inlineStr"/>
-      <c r="S23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>DIED2026-INT-0250235</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>111</v>
-      </c>
-      <c r="D24" t="n">
-        <v>111</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>factura_electronica</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Consulta Validez del Comprobante</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>F002-2258</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="N24" s="2" t="inlineStr">
-        <is>
-          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica F002-2258 es un comprobante de pago válido. 9/4/26, 9:27 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1</t>
-        </is>
-      </c>
-      <c r="O24" s="3" t="inlineStr"/>
-      <c r="P24" s="3" t="inlineStr"/>
-      <c r="Q24" s="3" t="inlineStr"/>
-      <c r="R24" s="3" t="inlineStr"/>
-      <c r="S24" s="3" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>DIED2026-INT-0250235</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>112</v>
-      </c>
-      <c r="D25" t="n">
-        <v>112</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>boleta_venta</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>20601709016</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>2016-12-05</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N25" s="2" t="inlineStr">
-        <is>
-          <t>Consulta RUC Resultado de la Búsqueda Número de RUC: 20601709016 - INVERSIONES CASA BLANCA A &amp; A S.A.C. Tipo Contribuyente: SOCIEDAD ANONIMA CERRADA Nombre Comercial: - Fecha de Inscripción: 05/12/2016 Fecha de Inicio de Actividades: 05/12/2016 Estado del Contribuyente: ACTIVO Condición del Contribu</t>
-        </is>
-      </c>
-      <c r="O25" s="3" t="inlineStr"/>
-      <c r="P25" s="3" t="inlineStr"/>
-      <c r="Q25" s="3" t="inlineStr"/>
-      <c r="R25" s="3" t="inlineStr"/>
-      <c r="S25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>DIED2026-INT-0250235</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>117</v>
-      </c>
-      <c r="D26" t="n">
-        <v>117</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>boleta_venta</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Fecha consulta: 08/04/2026 12:34</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>2026-04-08</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="N26" s="2" t="inlineStr">
-        <is>
-          <t>Fecha consulta: 08/04/2026 12:34 BOLETA DE VENTA GUIA DE REMISION - REMITENTE GUIA DE REMISION - TRANSPORTISTA Sistema de Emisión Electrónica: FACTURA PORTAL DESDE 15/05/2023 DESDE LOS SISTEMAS DEL CONTRIBUYENTE. AUTORIZ DESDE 29/04/2019 SEE-FACTURADOR . AUTORIZ DESDE 29/04/2019 Emisor electrónico d</t>
-        </is>
-      </c>
-      <c r="O26" s="3" t="inlineStr"/>
-      <c r="P26" s="3" t="inlineStr"/>
-      <c r="Q26" s="3" t="inlineStr"/>
-      <c r="R26" s="3" t="inlineStr"/>
-      <c r="S26" s="3" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>DIED2026-INT-0250235</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>119</v>
-      </c>
-      <c r="D27" t="n">
-        <v>120</v>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>factura_electronica</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>20202961518</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Consulta Validez del Comprobante</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>F219-11456</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>1994-01-02</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="N27" s="2" t="inlineStr">
-        <is>
-          <t>Consulta Validez del Comprobante de Pago Electrónico Resultado de la Consulta La Factura Electrónica F219-11456 es un comprobante de pago válido. 9/4/26, 9:29 Consulta de Validez del CPE https://e-consulta.sunat.gob.pe/ol-ti-itconsvalicpe/ConsValiCpe.htm 1/1 Consulta RUC Resultado de la Búsqueda Núm</t>
-        </is>
-      </c>
-      <c r="O27" s="3" t="inlineStr"/>
-      <c r="P27" s="3" t="inlineStr"/>
-      <c r="Q27" s="3" t="inlineStr"/>
-      <c r="R27" s="3" t="inlineStr"/>
-      <c r="S27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>DIED2026-INT-0250235</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>121</v>
-      </c>
-      <c r="D28" t="n">
-        <v>123</v>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>boleta_venta</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>20380795907</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Fecha consulta: 08/04/2026 12:35</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>2026-04-08</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>70.00</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>6.65</t>
-        </is>
-      </c>
-      <c r="M28" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="N28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fecha consulta: 08/04/2026 12:35 BOLETA DE VENTA NOTA DE CREDITO NOTA DE DEBITO GUIA DE REMISION - REMITENTE Sistema de Emisión Electrónica: FACTURA PORTAL DESDE 30/11/2021 DESDE LOS SISTEMAS DEL CONTRIBUYENTE. AUTORIZ DESDE 03/07/2018 Emisor electrónico desde: 03/07/2018 Comprobantes Electrónicos: </t>
-        </is>
-      </c>
-      <c r="O28" s="3" t="inlineStr"/>
-      <c r="P28" s="3" t="inlineStr"/>
-      <c r="Q28" s="3" t="inlineStr"/>
-      <c r="R28" s="3" t="inlineStr"/>
-      <c r="S28" s="3" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>DIED2026-INT-0250235</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>125</v>
-      </c>
-      <c r="D29" t="n">
-        <v>125</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>boleta_venta</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Fecha consulta: 08/04/2026 12:35</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>2026-04-08</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="N29" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fecha consulta: 08/04/2026 12:35 RECIBO POR HONORARIOS BOLETA DE VENTA Sistema de Emisión Electrónica: FACTURA PORTAL DESDE 17/06/2024 BOLETA PORTAL DESDE 26/05/2024 DESDE LOS SISTEMAS DEL CONTRIBUYENTE. AUTORIZ DESDE 07/02/2026 Emisor electrónico desde: 26/05/2024 Comprobantes Electrónicos: BOLETA </t>
-        </is>
-      </c>
-      <c r="O29" s="3" t="inlineStr"/>
-      <c r="P29" s="3" t="inlineStr"/>
-      <c r="Q29" s="3" t="inlineStr"/>
-      <c r="R29" s="3" t="inlineStr"/>
-      <c r="S29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>DIED2026-INT-0250235</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>126</v>
-      </c>
-      <c r="D30" t="n">
-        <v>128</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>factura_electronica</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>10427606037</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>TAXI ALMANZA</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>E001-16</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>2026-03-09</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>80.00</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="n">
-        <v>1</v>
-      </c>
-      <c r="N30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAXI ALMANZA ALMANZA MALLEA EDWIN FACTURA ELECTRONICA A.F. BELLA DURMIENTE PRIMERO MZA. Y LOTE. 11 ALT.AV. CANTO RUC: 10427606037 GRANDE CON AV. CANTO BELLO E001-16 SAN JUAN DE LURIGANCHO - LIMA - LIMA Fecha de Emisión : 09/03/2026 Forma de pago: Contado . PROGRAMA EDUCACION BASICA " PARA TODOS RUC </t>
-        </is>
-      </c>
-      <c r="O30" s="3" t="inlineStr"/>
-      <c r="P30" s="3" t="inlineStr"/>
-      <c r="Q30" s="3" t="inlineStr"/>
-      <c r="R30" s="3" t="inlineStr"/>
-      <c r="S30" s="3" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>DIED2026-INT-0250235</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>130</v>
-      </c>
-      <c r="D31" t="n">
-        <v>132</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>factura_electronica</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>10181382941</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>A) 10181382941</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>2006-09-20</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N31" s="2" t="inlineStr">
-        <is>
-          <t>A) 10181382941 Acuario "s SUITE FACTURA ELECTRONICA HOSPEDAJE ACUARIO'S SUITE Dirección : CALLE PRIMAVERA S/N SEC.LA ENCALADA DEL GOLF LA LIBERTAD - TRUJILLO - VICTOR LARCO HERRERA FAO 1 -85 Teléfonos : 065221356 Pagina web : hospedajeacuarios.efactur.pe Razón Social : PROGRAMA EDUCACION BASICA PARA</t>
-        </is>
-      </c>
-      <c r="O31" s="3" t="inlineStr"/>
-      <c r="P31" s="3" t="inlineStr"/>
-      <c r="Q31" s="3" t="inlineStr"/>
-      <c r="R31" s="3" t="inlineStr"/>
-      <c r="S31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>DIED2026-INT-0250235</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>133</v>
-      </c>
-      <c r="D32" t="n">
-        <v>133</v>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>boleta_venta</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Fecha consulta: 08/04/2026 12:36</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>2026-04-08</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="N32" s="2" t="inlineStr">
-        <is>
-          <t>Fecha consulta: 08/04/2026 12:36 BOLETA DE VENTA Sistema de Emisión Electrónica: DESDE LOS SISTEMAS DEL CONTRIBUYENTE. AUTORIZ DESDE 30/12/2020 Emisor electrónico desde: 30/12/2020 Comprobantes Electrónicos: FACTURA (desde 30/12/2020),BOLETA (desde 30/12/2020) Afiliado al PLE desde: - Padrones: NING</t>
-        </is>
-      </c>
-      <c r="O32" s="3" t="inlineStr"/>
-      <c r="P32" s="3" t="inlineStr"/>
-      <c r="Q32" s="3" t="inlineStr"/>
-      <c r="R32" s="3" t="inlineStr"/>
-      <c r="S32" s="3" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>DIED2026-INT-0250235</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>134</v>
-      </c>
-      <c r="D33" t="n">
-        <v>135</v>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>factura_electronica</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>20131525193</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>HOSPEDAJE EL PALACIO</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>E001-968</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="N33" s="2" t="inlineStr">
-        <is>
-          <t>HOSPEDAJE EL PALACIO SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA. JR. GRAU 709 TRUJILLO - TRUJILLO - LA LIBERTAD FACTURA ELECTRONICA RUC: 20131525193 E001-968 Fecha de Emisión : 21/03/2026 Forma de pago: Contado Señor(es) . PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 . JR. GRAU 709 LA LIBERTAD</t>
-        </is>
-      </c>
-      <c r="O33" s="3" t="inlineStr"/>
-      <c r="P33" s="3" t="inlineStr"/>
-      <c r="Q33" s="3" t="inlineStr"/>
-      <c r="R33" s="3" t="inlineStr"/>
-      <c r="S33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>DIED2026-INT-0250235</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>136</v>
-      </c>
-      <c r="D34" t="n">
-        <v>136</v>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>boleta_venta</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>20131525193</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Resultado de la Búsqueda</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>1993-05-06</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N34" s="2" t="inlineStr">
-        <is>
-          <t>Consulta RUC Resultado de la Búsqueda Número de RUC: 20131525193 - SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA. Tipo Contribuyente: SOC.COM.RESPONS. LTDA Nombre Comercial: HOSPEDAJE EL PALACIO Fecha de Inscripción: 06/05/1993 Fecha de Inicio de Actividades: 01/03/1991 Estado del Contribuyente: ACTIVO Con</t>
-        </is>
-      </c>
-      <c r="O34" s="3" t="inlineStr"/>
-      <c r="P34" s="3" t="inlineStr"/>
-      <c r="Q34" s="3" t="inlineStr"/>
-      <c r="R34" s="3" t="inlineStr"/>
-      <c r="S34" s="3" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>DIED2026-INT-0250235</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>138</v>
-      </c>
-      <c r="D35" t="n">
-        <v>139</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>factura_electronica</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>20131525193</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>HOSPEDAJE EL PALACIO</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>E001-970</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>2026-03-23</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>180.00</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="n">
-        <v>1</v>
-      </c>
-      <c r="N35" s="2" t="inlineStr">
-        <is>
-          <t>HOSPEDAJE EL PALACIO SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA. JR. GRAU 709 TRUJILLO - TRUJILLO - LA LIBERTAD FACTURA ELECTRONICA RUC: 20131525193 E001-970 Fecha de Emisión : 23/03/2026 Forma de pago: Contado Señor(es) . PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 . JR. GRAU 709 LA LIBERTAD</t>
-        </is>
-      </c>
-      <c r="O35" s="3" t="inlineStr"/>
-      <c r="P35" s="3" t="inlineStr"/>
-      <c r="Q35" s="3" t="inlineStr"/>
-      <c r="R35" s="3" t="inlineStr"/>
-      <c r="S35" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:S35"/>
+  <autoFilter ref="A1:S16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
classifier: Regla 1b — excluir resumen SIGA/Anexo 3 como comprobante
En `classify_page()` se agrega una regla entre SUNAT fuerte y cabecera+
corroboración: si la página contiene ≥2 series `[EFB]\d{3}-\d{2,8}`
distintas y además cabecera "RENDICIÓN DE CUENTAS" o "ANEXO N° 3", se
clasifica como `administrativo` subtipo `resumen_siga`.

Motivo: la página 1 del RENDIC piloto (listado SIGA con 13 series) era
clasificada como `boleta_venta` por la cabecera interna, generando un
comprobante espurio. El resto de páginas comprobante del piloto tienen
0 o 1 serie — margen amplio para no regresar.

Resultado en el piloto `DIED2026-INT-0250235`:
  15 → 14 comprobantes únicos (−1, era p1 E001-16 sin RUC ni monto)
  total detectado S/ 260.00 sin cambio
  sin_monto: 13 → 12 inconsistencias trazables
  resto de los 14 comprobantes intacto — 0 regresiones

Excel `validacion_expedientes.xlsx` regenerado.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/piloto_ocr/metrics/validacion_expedientes.xlsx
+++ b/data/piloto_ocr/metrics/validacion_expedientes.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'expedientes'!$A$1:$I$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'errores'!$A$1:$AG$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'resolucion_ids'!$A$1:$I$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'comprobantes'!$A$1:$S$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'comprobantes'!$A$1:$S$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -798,10 +798,24 @@
           <t>override_consolidado_rendicion: top_regex=factura(45) pero filename+encabezado indican rendicion(24)</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>firmas_anexo3</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>INSUFICIENTE_EVIDENCIA</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>nombre_ilegible:comisionado:anchor=dni_sin_nombre_adyacente; nombre_ilegible:jefe_unidad:anchor=sin_anchor; rol_no_detectado:vb_coordinador</t>
+        </is>
+      </c>
+      <c r="R3" t="n">
+        <v>0.1</v>
+      </c>
       <c r="S3" t="inlineStr">
         <is>
           <t>SINAD-250235</t>
@@ -1563,7 +1577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S16"/>
+  <dimension ref="A1:S15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1696,41 +1710,37 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>boleta_venta</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>E001-16</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2026-04-09</t>
-        </is>
-      </c>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>20608901460</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>DEGATTA PR¡HPNER¡¡</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>ANEXO N°3 Fecha : Hora : Página : 1 de 2 09/04/2026 13:01 Sistema Integrado de Gestión Módulo de Tesorería Versión 22.04.00 026 PROGRAMA EDUCACION BASICA PARA TODOS - 026 000081 Datos del CHAVEZ TERRONES LILIANA Sr(a): N° Planilla: Motivo de Salida: 00617 N° Exp SIAF: 2603426 N° Comprobante 09/03/20</t>
+          <t>DEGATTA PR¡HPNER¡¡ Le INVERSIONES É,T:R Jiron Ayacucho: 521; fry eae Peru — Trujillo. . Rue: 20608901460 FACTURA ELECTRONICA FO03-0000002483 “Orden: ov-094765 Fecha de emision : 10-03-2026 he SALON) PRINCIP AL " Rur. 2038!1 795907 Razon social - “PROGRAMA EDUCACION BASICA PARA TO Bop CALs DEL COMERC</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr"/>
@@ -1751,10 +1761,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D3" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1763,25 +1773,29 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>20608901460</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>DEGATTA PR¡HPNER¡¡</t>
-        </is>
-      </c>
+          <t>10181685510</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>DEGATTA PR¡HPNER¡¡ Le INVERSIONES É,T:R Jiron Ayacucho: 521; fry eae Peru — Trujillo. . Rue: 20608901460 FACTURA ELECTRONICA FO03-0000002483 “Orden: ov-094765 Fecha de emision : 10-03-2026 he SALON) PRINCIP AL " Rur. 2038!1 795907 Razon social - “PROGRAMA EDUCACION BASICA PARA TO Bop CALs DEL COMERC</t>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002114 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 11/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr"/>
@@ -1802,10 +1816,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D4" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1836,7 +1850,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002114 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 11/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002122 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 11/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr"/>
@@ -1857,10 +1871,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="D5" t="n">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1876,7 +1890,7 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -1891,7 +1905,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002122 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 11/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002135 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 15/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr"/>
@@ -1912,10 +1926,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="D6" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1935,18 +1949,14 @@
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
         <v>0.5</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002135 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 15/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002136 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 15/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr"/>
@@ -1967,37 +1977,41 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="D7" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>factura_electronica</t>
+          <t>boleta_venta</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>10181685510</t>
+          <t>10181727883</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
         <v>0.5</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002136 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 15/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+          <t>BOLETA DE VENTA ELECTRONICA RUC: 10181727883 EB01-163 TAPIA MERINO GLADYS PATRICIA JR. LOS RUBIES 383 URB. SANTA INES TRUJILLO - TRUJILLO - LA LIBERTAD Fecha de Vencimiento Fecha de Emisión : 17/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Observación : S</t>
         </is>
       </c>
       <c r="O7" s="3" t="inlineStr"/>
@@ -2018,10 +2032,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D8" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -2052,7 +2066,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>BOLETA DE VENTA ELECTRONICA RUC: 10181727883 EB01-163 TAPIA MERINO GLADYS PATRICIA JR. LOS RUBIES 383 URB. SANTA INES TRUJILLO - TRUJILLO - LA LIBERTAD Fecha de Vencimiento Fecha de Emisión : 17/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Observación : S</t>
+          <t>BOLETA DE VENTA ELECTRONICA RUC: 10181727883 EB01-164 TAPIA MERINO GLADYS PATRICIA JR. LOS RUBIES 383 URB. SANTA INES TRUJILLO - TRUJILLO - LA LIBERTAD Fecha de Vencimiento Fecha de Emisión : 17/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Observación : S</t>
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr"/>
@@ -2073,26 +2087,26 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="D9" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>boleta_venta</t>
+          <t>factura_electronica</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10181727883</t>
+          <t>10181685510</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -2107,7 +2121,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>BOLETA DE VENTA ELECTRONICA RUC: 10181727883 EB01-164 TAPIA MERINO GLADYS PATRICIA JR. LOS RUBIES 383 URB. SANTA INES TRUJILLO - TRUJILLO - LA LIBERTAD Fecha de Vencimiento Fecha de Emisión : 17/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Observación : S</t>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002139 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 18/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr"/>
@@ -2128,10 +2142,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D10" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -2162,7 +2176,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002139 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 18/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002141 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 18/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr"/>
@@ -2183,26 +2197,26 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>82</v>
+        <v>122</v>
       </c>
       <c r="D11" t="n">
-        <v>82</v>
+        <v>122</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>factura_electronica</t>
+          <t>boleta_venta</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>10181685510</t>
+          <t>20380795907</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -2217,7 +2231,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002141 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 18/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+          <t xml:space="preserve">LA ESQUINA DEL ESTUDIANTE HERNANDEZ ALMENGOR SILVIA MARLENE BOLETAR%ECY,IE¿:;;OE,II;EÍIRONICA MZA. G INT. 2 PI LOTE. 1 URB. INGENIERIA E'Bº1 1390 TRUJILLO - TRUJILLO - LA LIBERTAD - Fecha de Vencimiento Fecha de Emisión : 23/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de </t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr"/>
@@ -2238,29 +2252,41 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="D12" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>boleta_venta</t>
+          <t>factura_electronica</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>20380795907</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
+          <t>10427606037</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>TAXI ALMANZA</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>E001-16</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>80.00</t>
+        </is>
+      </c>
       <c r="K12" t="inlineStr">
         <is>
           <t>PEN</t>
@@ -2268,11 +2294,11 @@
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LA ESQUINA DEL ESTUDIANTE HERNANDEZ ALMENGOR SILVIA MARLENE BOLETAR%ECY,IE¿:;;OE,II;EÍIRONICA MZA. G INT. 2 PI LOTE. 1 URB. INGENIERIA E'Bº1 1390 TRUJILLO - TRUJILLO - LA LIBERTAD - Fecha de Vencimiento Fecha de Emisión : 23/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de </t>
+          <t xml:space="preserve">TAXI ALMANZA ALMANZA MALLEA EDWIN FACTURA ELECTRONICA A.F. BELLA DURMIENTE PRIMERO MZA. Y LOTE. 11 ALT.AV. CANTO RUC: 10427606037 GRANDE CON AV. CANTO BELLO E001-16 SAN JUAN DE LURIGANCHO - LIMA - LIMA Fecha de Emisión : 09/03/2026 Forma de pago: Contado . PROGRAMA EDUCACION BASICA " PARA TODOS RUC </t>
         </is>
       </c>
       <c r="O12" s="3" t="inlineStr"/>
@@ -2293,10 +2319,10 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="D13" t="n">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2305,29 +2331,17 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>10427606037</t>
+          <t>10181382941</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>TAXI ALMANZA</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>E001-16</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>2026-03-09</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>80.00</t>
-        </is>
-      </c>
+          <t>A) 10181382941</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>PEN</t>
@@ -2335,11 +2349,11 @@
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAXI ALMANZA ALMANZA MALLEA EDWIN FACTURA ELECTRONICA A.F. BELLA DURMIENTE PRIMERO MZA. Y LOTE. 11 ALT.AV. CANTO RUC: 10427606037 GRANDE CON AV. CANTO BELLO E001-16 SAN JUAN DE LURIGANCHO - LIMA - LIMA Fecha de Emisión : 09/03/2026 Forma de pago: Contado . PROGRAMA EDUCACION BASICA " PARA TODOS RUC </t>
+          <t>A) 10181382941 Acuario "s SUITE FACTURA ELECTRONICA HOSPEDAJE ACUARIO'S SUITE Dirección : CALLE PRIMAVERA S/N SEC.LA ENCALADA DEL GOLF LA LIBERTAD - TRUJILLO - VICTOR LARCO HERRERA FAO 1 -85 Teléfonos : 065221356 Pagina web : hospedajeacuarios.efactur.pe Razón Social : PROGRAMA EDUCACION BASICA PARA</t>
         </is>
       </c>
       <c r="O13" s="3" t="inlineStr"/>
@@ -2360,10 +2374,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="D14" t="n">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2372,16 +2386,24 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>10181382941</t>
+          <t>20131525193</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>A) 10181382941</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
+          <t>HOSPEDAJE EL PALACIO</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>E001-968</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
@@ -2390,11 +2412,11 @@
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
-        <v>0.25</v>
+        <v>0.75</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>A) 10181382941 Acuario "s SUITE FACTURA ELECTRONICA HOSPEDAJE ACUARIO'S SUITE Dirección : CALLE PRIMAVERA S/N SEC.LA ENCALADA DEL GOLF LA LIBERTAD - TRUJILLO - VICTOR LARCO HERRERA FAO 1 -85 Teléfonos : 065221356 Pagina web : hospedajeacuarios.efactur.pe Razón Social : PROGRAMA EDUCACION BASICA PARA</t>
+          <t>HOSPEDAJE EL PALACIO SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA. JR. GRAU 709 TRUJILLO - TRUJILLO - LA LIBERTAD FACTURA ELECTRONICA RUC: 20131525193 E001-968 Fecha de Emisión : 21/03/2026 Forma de pago: Contado Señor(es) . PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 . JR. GRAU 709 LA LIBERTAD</t>
         </is>
       </c>
       <c r="O14" s="3" t="inlineStr"/>
@@ -2415,10 +2437,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="D15" t="n">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2437,15 +2459,19 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>E001-968</t>
+          <t>E001-970</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr"/>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>180.00</t>
+        </is>
+      </c>
       <c r="K15" t="inlineStr">
         <is>
           <t>PEN</t>
@@ -2453,11 +2479,11 @@
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>HOSPEDAJE EL PALACIO SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA. JR. GRAU 709 TRUJILLO - TRUJILLO - LA LIBERTAD FACTURA ELECTRONICA RUC: 20131525193 E001-968 Fecha de Emisión : 21/03/2026 Forma de pago: Contado Señor(es) . PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 . JR. GRAU 709 LA LIBERTAD</t>
+          <t>HOSPEDAJE EL PALACIO SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA. JR. GRAU 709 TRUJILLO - TRUJILLO - LA LIBERTAD FACTURA ELECTRONICA RUC: 20131525193 E001-970 Fecha de Emisión : 23/03/2026 Forma de pago: Contado Señor(es) . PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 . JR. GRAU 709 LA LIBERTAD</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr"/>
@@ -2466,75 +2492,8 @@
       <c r="R15" s="3" t="inlineStr"/>
       <c r="S15" s="3" t="inlineStr"/>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>DIED2026-INT-0250235</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>138</v>
-      </c>
-      <c r="D16" t="n">
-        <v>138</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>factura_electronica</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>20131525193</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>HOSPEDAJE EL PALACIO</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>E001-970</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>2026-03-23</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>180.00</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="n">
-        <v>1</v>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>HOSPEDAJE EL PALACIO SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA. JR. GRAU 709 TRUJILLO - TRUJILLO - LA LIBERTAD FACTURA ELECTRONICA RUC: 20131525193 E001-970 Fecha de Emisión : 23/03/2026 Forma de pago: Contado Señor(es) . PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 . JR. GRAU 709 LA LIBERTAD</t>
-        </is>
-      </c>
-      <c r="O16" s="3" t="inlineStr"/>
-      <c r="P16" s="3" t="inlineStr"/>
-      <c r="Q16" s="3" t="inlineStr"/>
-      <c r="R16" s="3" t="inlineStr"/>
-      <c r="S16" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:S16"/>
+  <autoFilter ref="A1:S15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix #1: segundo pase en detector — recuperar comprobantes via CPE
Agrega un segundo pase dentro de detectar_bloques() que recorre las
paginas CPE (sunat_validez_cpe con nota cita_cabecera_comprobante) y
promueve la pagina inmediata anterior a BloqueComprobante cuando esta
clasificada como "otros" y no fue usada por el primer pase.

Tipo y serie se extraen del texto CPE (texto seleccionable, mas
fiable que el OCR del escaneo). RUC se extrae de la pagina de
consulta RUC (pagina siguiente a la CPE) como fuente primaria,
con fallback al texto del candidato.

Resultado en el piloto DIED2026-INT-0250235:
  14 → 29 comprobantes (+15 recuperados via CPE)
  RUC:   93% → 100% (29/29)
  Serie: 27% → 41% (12/29)
  Monto: S/ 260.00 → S/ 467.24
  0 regresiones (los 14 originales intactos)

Cambio aislado en comprobante_detector.py (+49 lineas).
Excel validacion_expedientes.xlsx regenerado con 29 filas.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/piloto_ocr/metrics/validacion_expedientes.xlsx
+++ b/data/piloto_ocr/metrics/validacion_expedientes.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-113" yWindow="-113" windowWidth="24267" windowHeight="13023" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="documentos" sheetId="1" state="visible" r:id="rId1"/>
@@ -18,16 +17,16 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'expedientes'!$A$1:$I$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'errores'!$A$1:$AG$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'resolucion_ids'!$A$1:$I$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'comprobantes'!$A$1:$S$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'comprobantes'!$A$1:$S$30</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,16 +35,32 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF305496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -70,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -79,9 +94,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -483,167 +502,167 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>expediente_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>archivo</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>ruta_origen</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>tipo_documento_detectado</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>confianza_tipo</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>monto_detectado</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>fecha_detectada</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>ruc_detectado</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>razon_social_detectada</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>numero_documento_detectado</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>tipo_gasto_detectado</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>texto_extraido_resumen</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>estado_procesamiento</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>nota_sistema</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" s="4" t="inlineStr">
         <is>
           <t>validacion_firmas</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" s="4" t="inlineStr">
         <is>
           <t>estado_firmas</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" s="4" t="inlineStr">
         <is>
           <t>errores_firmas</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" s="4" t="inlineStr">
         <is>
           <t>confianza_firmas</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
         <is>
           <t>expediente_detectado</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" s="4" t="inlineStr">
         <is>
           <t>sinad_detectado</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" s="4" t="inlineStr">
         <is>
           <t>siaf_detectado</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" s="4" t="inlineStr">
         <is>
           <t>anio_detectado</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" s="4" t="inlineStr">
         <is>
           <t>confianza_expediente</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" s="4" t="inlineStr">
         <is>
           <t>confianza_sinad</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" s="4" t="inlineStr">
         <is>
           <t>confianza_siaf</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" s="4" t="inlineStr">
         <is>
           <t>conflicto_expediente</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" s="4" t="inlineStr">
         <is>
           <t>observaciones_expediente</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" s="4" t="inlineStr">
         <is>
           <t>tipo_correcto</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" s="4" t="inlineStr">
         <is>
           <t>monto_correcto</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" s="4" t="inlineStr">
         <is>
           <t>fecha_correcta</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" s="4" t="inlineStr">
         <is>
           <t>ruc_correcto</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" s="4" t="inlineStr">
         <is>
           <t>observaciones</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" s="4" t="inlineStr">
         <is>
           <t>validacion_final</t>
         </is>
@@ -742,12 +761,12 @@
           <t>siaf:conflicto: top=SIAF-2603426(16.0) vs segundo=SIAF-3205(16.0)</t>
         </is>
       </c>
-      <c r="AB2" s="3" t="n"/>
-      <c r="AC2" s="3" t="n"/>
-      <c r="AD2" s="3" t="n"/>
-      <c r="AE2" s="3" t="n"/>
-      <c r="AF2" s="3" t="n"/>
-      <c r="AG2" s="3" t="n"/>
+      <c r="AB2" s="5" t="n"/>
+      <c r="AC2" s="5" t="n"/>
+      <c r="AD2" s="5" t="n"/>
+      <c r="AE2" s="5" t="n"/>
+      <c r="AF2" s="5" t="n"/>
+      <c r="AG2" s="5" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -855,12 +874,12 @@
           <t>siaf:conflicto: top=SIAF-2603426(16.0) vs segundo=SIAF-3205(16.0)</t>
         </is>
       </c>
-      <c r="AB3" s="3" t="n"/>
-      <c r="AC3" s="3" t="n"/>
-      <c r="AD3" s="3" t="n"/>
-      <c r="AE3" s="3" t="n"/>
-      <c r="AF3" s="3" t="n"/>
-      <c r="AG3" s="3" t="n"/>
+      <c r="AB3" s="5" t="n"/>
+      <c r="AC3" s="5" t="n"/>
+      <c r="AD3" s="5" t="n"/>
+      <c r="AE3" s="5" t="n"/>
+      <c r="AF3" s="5" t="n"/>
+      <c r="AG3" s="5" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AG3"/>
@@ -889,47 +908,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>expediente_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>ruta_origen</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>ruta_destino</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>n_documentos</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>n_ok</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>n_bajo_confianza</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>n_error</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>tipos_detectados</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>fecha_ingesta</t>
         </is>
@@ -1025,167 +1044,167 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>expediente_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>archivo</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>ruta_origen</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>tipo_documento_detectado</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>confianza_tipo</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>monto_detectado</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>fecha_detectada</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>ruc_detectado</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>razon_social_detectada</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>numero_documento_detectado</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>tipo_gasto_detectado</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>texto_extraido_resumen</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>estado_procesamiento</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>nota_sistema</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" s="4" t="inlineStr">
         <is>
           <t>validacion_firmas</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" s="4" t="inlineStr">
         <is>
           <t>estado_firmas</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" s="4" t="inlineStr">
         <is>
           <t>errores_firmas</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" s="4" t="inlineStr">
         <is>
           <t>confianza_firmas</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
         <is>
           <t>expediente_detectado</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" s="4" t="inlineStr">
         <is>
           <t>sinad_detectado</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" s="4" t="inlineStr">
         <is>
           <t>siaf_detectado</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" s="4" t="inlineStr">
         <is>
           <t>anio_detectado</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" s="4" t="inlineStr">
         <is>
           <t>confianza_expediente</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" s="4" t="inlineStr">
         <is>
           <t>confianza_sinad</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" s="4" t="inlineStr">
         <is>
           <t>confianza_siaf</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" s="4" t="inlineStr">
         <is>
           <t>conflicto_expediente</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" s="4" t="inlineStr">
         <is>
           <t>observaciones_expediente</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" s="4" t="inlineStr">
         <is>
           <t>tipo_correcto</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" s="4" t="inlineStr">
         <is>
           <t>monto_correcto</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" s="4" t="inlineStr">
         <is>
           <t>fecha_correcta</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" s="4" t="inlineStr">
         <is>
           <t>ruc_correcto</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" s="4" t="inlineStr">
         <is>
           <t>observaciones</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" s="4" t="inlineStr">
         <is>
           <t>validacion_final</t>
         </is>
@@ -1218,47 +1237,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>expediente_carpeta</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>id_canonico</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>tipo</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>frecuencia</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>score_total</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>coincide_con_carpeta</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>es_ganador</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>estado_resolucion</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>fuentes</t>
         </is>
@@ -1577,7 +1596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S15"/>
+  <dimension ref="A1:S30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1602,97 +1621,97 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>expediente_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>archivo</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>pagina_inicio</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>pagina_fin</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>tipo</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>ruc</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>razon_social</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>serie_numero</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>fecha</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>monto_total</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>moneda</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>monto_igv</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>confianza</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>texto_resumen</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" s="4" t="inlineStr">
         <is>
           <t>monto_correcto</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" s="4" t="inlineStr">
         <is>
           <t>ruc_correcto</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" s="4" t="inlineStr">
         <is>
           <t>proveedor_correcto</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" s="4" t="inlineStr">
         <is>
           <t>observaciones</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
         <is>
           <t>validacion_final</t>
         </is>
@@ -1710,10 +1729,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="D2" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1722,32 +1741,40 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>20608901460</t>
+          <t>20477689699</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>DEGATTA PR¡HPNER¡¡</t>
+          <t>F_—-— INVERSIONES a SERVICIOS MULTIPLES</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>108.60</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>DEGATTA PR¡HPNER¡¡ Le INVERSIONES É,T:R Jiron Ayacucho: 521; fry eae Peru — Trujillo. . Rue: 20608901460 FACTURA ELECTRONICA FO03-0000002483 “Orden: ov-094765 Fecha de emision : 10-03-2026 he SALON) PRINCIP AL " Rur. 2038!1 795907 Razon social - “PROGRAMA EDUCACION BASICA PARA TO Bop CALs DEL COMERC</t>
-        </is>
-      </c>
-      <c r="O2" s="3" t="inlineStr"/>
-      <c r="P2" s="3" t="inlineStr"/>
-      <c r="Q2" s="3" t="inlineStr"/>
-      <c r="R2" s="3" t="inlineStr"/>
-      <c r="S2" s="3" t="inlineStr"/>
+          <t>F_—-— — INVERSIONES a SERVICIOS MULTIPLES COQUITO S.A Av. America Sut 2763 Palle La Libertad *** COQUITO *** Teléfono ; 044-224451 RUC: 20477689699 L FACTURA DE VENTA ELECTRÓNICA NO: FAO1-0000007538 Mesa: A-9 Fecha: 09/03/26 01:50 PM WALTER Cliente: Teléf: - PROGRAMA EDUCACION BASICA PARA TODOS CAL.</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="inlineStr"/>
+      <c r="P2" s="5" t="inlineStr"/>
+      <c r="Q2" s="5" t="inlineStr"/>
+      <c r="R2" s="5" t="inlineStr"/>
+      <c r="S2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1761,10 +1788,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="D3" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1773,17 +1800,21 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>10181685510</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>20539971477</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Cebicheria Coquito SAC.</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>98.64</t>
+        </is>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
           <t>PEN</t>
@@ -1795,14 +1826,14 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002114 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 11/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
-        </is>
-      </c>
-      <c r="O3" s="3" t="inlineStr"/>
-      <c r="P3" s="3" t="inlineStr"/>
-      <c r="Q3" s="3" t="inlineStr"/>
-      <c r="R3" s="3" t="inlineStr"/>
-      <c r="S3" s="3" t="inlineStr"/>
+          <t>Cebicheria Coquito SAC. Honorio Delgado Mz Q’ Lote 2 El Bosque - Trujillo - La Ll bertad *** COQUITO *** Teléfono : 044-215511 RUC: 20539971477 — FACTURA DE VENTA ELECTRÓNICA Ne: FBO2-0000007269 Mesa: A-16 Fecha: 10/03/26 02:42 PM EDUARDO Cliente: Teléf: - PROGRAMA EDUCACION BASICA PARA TODOS CAL,DE</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr"/>
+      <c r="P3" s="5" t="inlineStr"/>
+      <c r="Q3" s="5" t="inlineStr"/>
+      <c r="R3" s="5" t="inlineStr"/>
+      <c r="S3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1816,10 +1847,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D4" t="n">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1828,36 +1859,32 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>10181685510</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>20608901460</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>DEGATTA PR¡HPNER¡¡</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002122 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 11/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
-        </is>
-      </c>
-      <c r="O4" s="3" t="inlineStr"/>
-      <c r="P4" s="3" t="inlineStr"/>
-      <c r="Q4" s="3" t="inlineStr"/>
-      <c r="R4" s="3" t="inlineStr"/>
-      <c r="S4" s="3" t="inlineStr"/>
+          <t>DEGATTA PR¡HPNER¡¡ Le INVERSIONES É,T:R Jiron Ayacucho: 521; fry eae Peru — Trujillo. . Rue: 20608901460 FACTURA ELECTRONICA FO03-0000002483 “Orden: ov-094765 Fecha de emision : 10-03-2026 he SALON) PRINCIP AL " Rur. 2038!1 795907 Razon social - “PROGRAMA EDUCACION BASICA PARA TO Bop CALs DEL COMERC</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr"/>
+      <c r="P4" s="5" t="inlineStr"/>
+      <c r="Q4" s="5" t="inlineStr"/>
+      <c r="R4" s="5" t="inlineStr"/>
+      <c r="S4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1871,10 +1898,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="D5" t="n">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1890,7 +1917,7 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -1905,14 +1932,14 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002135 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 15/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
-        </is>
-      </c>
-      <c r="O5" s="3" t="inlineStr"/>
-      <c r="P5" s="3" t="inlineStr"/>
-      <c r="Q5" s="3" t="inlineStr"/>
-      <c r="R5" s="3" t="inlineStr"/>
-      <c r="S5" s="3" t="inlineStr"/>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002114 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 11/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+        </is>
+      </c>
+      <c r="O5" s="5" t="inlineStr"/>
+      <c r="P5" s="5" t="inlineStr"/>
+      <c r="Q5" s="5" t="inlineStr"/>
+      <c r="R5" s="5" t="inlineStr"/>
+      <c r="S5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1926,10 +1953,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="D6" t="n">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1945,25 +1972,29 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
         <v>0.5</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002136 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 15/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
-        </is>
-      </c>
-      <c r="O6" s="3" t="inlineStr"/>
-      <c r="P6" s="3" t="inlineStr"/>
-      <c r="Q6" s="3" t="inlineStr"/>
-      <c r="R6" s="3" t="inlineStr"/>
-      <c r="S6" s="3" t="inlineStr"/>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002122 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 11/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr"/>
+      <c r="P6" s="5" t="inlineStr"/>
+      <c r="Q6" s="5" t="inlineStr"/>
+      <c r="R6" s="5" t="inlineStr"/>
+      <c r="S6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1977,48 +2008,40 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="D7" t="n">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>boleta_venta</t>
+          <t>factura_electronica</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>10181727883</t>
+          <t>20609385317</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
-      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>F006-00002488</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
         <v>0.5</v>
       </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>BOLETA DE VENTA ELECTRONICA RUC: 10181727883 EB01-163 TAPIA MERINO GLADYS PATRICIA JR. LOS RUBIES 383 URB. SANTA INES TRUJILLO - TRUJILLO - LA LIBERTAD Fecha de Vencimiento Fecha de Emisión : 17/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Observación : S</t>
-        </is>
-      </c>
-      <c r="O7" s="3" t="inlineStr"/>
-      <c r="P7" s="3" t="inlineStr"/>
-      <c r="Q7" s="3" t="inlineStr"/>
-      <c r="R7" s="3" t="inlineStr"/>
-      <c r="S7" s="3" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr"/>
+      <c r="O7" s="5" t="inlineStr"/>
+      <c r="P7" s="5" t="inlineStr"/>
+      <c r="Q7" s="5" t="inlineStr"/>
+      <c r="R7" s="5" t="inlineStr"/>
+      <c r="S7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2032,48 +2055,44 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="D8" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>boleta_venta</t>
+          <t>factura_electronica</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>10181727883</t>
+          <t>20611728159</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
-      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>F001-00001460</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
         <v>0.5</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>BOLETA DE VENTA ELECTRONICA RUC: 10181727883 EB01-164 TAPIA MERINO GLADYS PATRICIA JR. LOS RUBIES 383 URB. SANTA INES TRUJILLO - TRUJILLO - LA LIBERTAD Fecha de Vencimiento Fecha de Emisión : 17/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Observación : S</t>
-        </is>
-      </c>
-      <c r="O8" s="3" t="inlineStr"/>
-      <c r="P8" s="3" t="inlineStr"/>
-      <c r="Q8" s="3" t="inlineStr"/>
-      <c r="R8" s="3" t="inlineStr"/>
-      <c r="S8" s="3" t="inlineStr"/>
+          <t>' - mm lt 1 ‘ E Á -¡:I;'.'. ) h — ' LF TRA.</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr"/>
+      <c r="P8" s="5" t="inlineStr"/>
+      <c r="Q8" s="5" t="inlineStr"/>
+      <c r="R8" s="5" t="inlineStr"/>
+      <c r="S8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2087,10 +2106,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>78</v>
+        <v>54</v>
       </c>
       <c r="D9" t="n">
-        <v>78</v>
+        <v>54</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -2099,36 +2118,28 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10181685510</t>
+          <t>20608901460</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>2026-03-18</t>
-        </is>
-      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>F003-2478</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
         <v>0.5</v>
       </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002139 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 18/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
-        </is>
-      </c>
-      <c r="O9" s="3" t="inlineStr"/>
-      <c r="P9" s="3" t="inlineStr"/>
-      <c r="Q9" s="3" t="inlineStr"/>
-      <c r="R9" s="3" t="inlineStr"/>
-      <c r="S9" s="3" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr"/>
+      <c r="O9" s="5" t="inlineStr"/>
+      <c r="P9" s="5" t="inlineStr"/>
+      <c r="Q9" s="5" t="inlineStr"/>
+      <c r="R9" s="5" t="inlineStr"/>
+      <c r="S9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2142,10 +2153,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>82</v>
+        <v>58</v>
       </c>
       <c r="D10" t="n">
-        <v>82</v>
+        <v>58</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -2161,7 +2172,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -2176,14 +2187,14 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002141 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 18/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
-        </is>
-      </c>
-      <c r="O10" s="3" t="inlineStr"/>
-      <c r="P10" s="3" t="inlineStr"/>
-      <c r="Q10" s="3" t="inlineStr"/>
-      <c r="R10" s="3" t="inlineStr"/>
-      <c r="S10" s="3" t="inlineStr"/>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002135 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 15/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+        </is>
+      </c>
+      <c r="O10" s="5" t="inlineStr"/>
+      <c r="P10" s="5" t="inlineStr"/>
+      <c r="Q10" s="5" t="inlineStr"/>
+      <c r="R10" s="5" t="inlineStr"/>
+      <c r="S10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2197,48 +2208,44 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>122</v>
+        <v>62</v>
       </c>
       <c r="D11" t="n">
-        <v>122</v>
+        <v>62</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>boleta_venta</t>
+          <t>factura_electronica</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>20380795907</t>
+          <t>10181685510</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
         <v>0.5</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LA ESQUINA DEL ESTUDIANTE HERNANDEZ ALMENGOR SILVIA MARLENE BOLETAR%ECY,IE¿:;;OE,II;EÍIRONICA MZA. G INT. 2 PI LOTE. 1 URB. INGENIERIA E'Bº1 1390 TRUJILLO - TRUJILLO - LA LIBERTAD - Fecha de Vencimiento Fecha de Emisión : 23/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de </t>
-        </is>
-      </c>
-      <c r="O11" s="3" t="inlineStr"/>
-      <c r="P11" s="3" t="inlineStr"/>
-      <c r="Q11" s="3" t="inlineStr"/>
-      <c r="R11" s="3" t="inlineStr"/>
-      <c r="S11" s="3" t="inlineStr"/>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002136 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 15/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+        </is>
+      </c>
+      <c r="O11" s="5" t="inlineStr"/>
+      <c r="P11" s="5" t="inlineStr"/>
+      <c r="Q11" s="5" t="inlineStr"/>
+      <c r="R11" s="5" t="inlineStr"/>
+      <c r="S11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2252,41 +2259,29 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>126</v>
+        <v>66</v>
       </c>
       <c r="D12" t="n">
-        <v>126</v>
+        <v>66</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>factura_electronica</t>
+          <t>boleta_venta</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>10427606037</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>TAXI ALMANZA</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>E001-16</t>
-        </is>
-      </c>
+          <t>10181727883</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>80.00</t>
-        </is>
-      </c>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>PEN</t>
@@ -2294,18 +2289,18 @@
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAXI ALMANZA ALMANZA MALLEA EDWIN FACTURA ELECTRONICA A.F. BELLA DURMIENTE PRIMERO MZA. Y LOTE. 11 ALT.AV. CANTO RUC: 10427606037 GRANDE CON AV. CANTO BELLO E001-16 SAN JUAN DE LURIGANCHO - LIMA - LIMA Fecha de Emisión : 09/03/2026 Forma de pago: Contado . PROGRAMA EDUCACION BASICA " PARA TODOS RUC </t>
-        </is>
-      </c>
-      <c r="O12" s="3" t="inlineStr"/>
-      <c r="P12" s="3" t="inlineStr"/>
-      <c r="Q12" s="3" t="inlineStr"/>
-      <c r="R12" s="3" t="inlineStr"/>
-      <c r="S12" s="3" t="inlineStr"/>
+          <t>BOLETA DE VENTA ELECTRONICA RUC: 10181727883 EB01-163 TAPIA MERINO GLADYS PATRICIA JR. LOS RUBIES 383 URB. SANTA INES TRUJILLO - TRUJILLO - LA LIBERTAD Fecha de Vencimiento Fecha de Emisión : 17/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Observación : S</t>
+        </is>
+      </c>
+      <c r="O12" s="5" t="inlineStr"/>
+      <c r="P12" s="5" t="inlineStr"/>
+      <c r="Q12" s="5" t="inlineStr"/>
+      <c r="R12" s="5" t="inlineStr"/>
+      <c r="S12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2319,28 +2314,28 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>130</v>
+        <v>70</v>
       </c>
       <c r="D13" t="n">
-        <v>130</v>
+        <v>70</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>factura_electronica</t>
+          <t>boleta_venta</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>10181382941</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>A) 10181382941</t>
-        </is>
-      </c>
+          <t>10181727883</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
@@ -2349,18 +2344,18 @@
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>A) 10181382941 Acuario "s SUITE FACTURA ELECTRONICA HOSPEDAJE ACUARIO'S SUITE Dirección : CALLE PRIMAVERA S/N SEC.LA ENCALADA DEL GOLF LA LIBERTAD - TRUJILLO - VICTOR LARCO HERRERA FAO 1 -85 Teléfonos : 065221356 Pagina web : hospedajeacuarios.efactur.pe Razón Social : PROGRAMA EDUCACION BASICA PARA</t>
-        </is>
-      </c>
-      <c r="O13" s="3" t="inlineStr"/>
-      <c r="P13" s="3" t="inlineStr"/>
-      <c r="Q13" s="3" t="inlineStr"/>
-      <c r="R13" s="3" t="inlineStr"/>
-      <c r="S13" s="3" t="inlineStr"/>
+          <t>BOLETA DE VENTA ELECTRONICA RUC: 10181727883 EB01-164 TAPIA MERINO GLADYS PATRICIA JR. LOS RUBIES 383 URB. SANTA INES TRUJILLO - TRUJILLO - LA LIBERTAD Fecha de Vencimiento Fecha de Emisión : 17/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Observación : S</t>
+        </is>
+      </c>
+      <c r="O13" s="5" t="inlineStr"/>
+      <c r="P13" s="5" t="inlineStr"/>
+      <c r="Q13" s="5" t="inlineStr"/>
+      <c r="R13" s="5" t="inlineStr"/>
+      <c r="S13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2374,10 +2369,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>134</v>
+        <v>74</v>
       </c>
       <c r="D14" t="n">
-        <v>134</v>
+        <v>74</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2386,44 +2381,32 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>20131525193</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>HOSPEDAJE EL PALACIO</t>
-        </is>
-      </c>
+          <t>20613429388</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>E001-968</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
+          <t>F001-543</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>HOSPEDAJE EL PALACIO SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA. JR. GRAU 709 TRUJILLO - TRUJILLO - LA LIBERTAD FACTURA ELECTRONICA RUC: 20131525193 E001-968 Fecha de Emisión : 21/03/2026 Forma de pago: Contado Señor(es) . PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 . JR. GRAU 709 LA LIBERTAD</t>
-        </is>
-      </c>
-      <c r="O14" s="3" t="inlineStr"/>
-      <c r="P14" s="3" t="inlineStr"/>
-      <c r="Q14" s="3" t="inlineStr"/>
-      <c r="R14" s="3" t="inlineStr"/>
-      <c r="S14" s="3" t="inlineStr"/>
+          <t>16134 &lt;1 LOTE 8 URB SAN ey II ET s eet) M mta¿ — aE E 90 eo 1700 R ',frasnntaainn arte del Comprobant th e Electro) eS \Gracias Par ei preferencial h Sunwnro eRestaurant - 9764 77688</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="inlineStr"/>
+      <c r="P14" s="5" t="inlineStr"/>
+      <c r="Q14" s="5" t="inlineStr"/>
+      <c r="R14" s="5" t="inlineStr"/>
+      <c r="S14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2437,10 +2420,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>138</v>
+        <v>78</v>
       </c>
       <c r="D15" t="n">
-        <v>138</v>
+        <v>78</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2449,29 +2432,17 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>20131525193</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>HOSPEDAJE EL PALACIO</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>E001-970</t>
-        </is>
-      </c>
+          <t>10181685510</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>180.00</t>
-        </is>
-      </c>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
           <t>PEN</t>
@@ -2479,21 +2450,818 @@
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002139 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 18/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+        </is>
+      </c>
+      <c r="O15" s="5" t="inlineStr"/>
+      <c r="P15" s="5" t="inlineStr"/>
+      <c r="Q15" s="5" t="inlineStr"/>
+      <c r="R15" s="5" t="inlineStr"/>
+      <c r="S15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>82</v>
+      </c>
+      <c r="D16" t="n">
+        <v>82</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>10181685510</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002141 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 18/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr"/>
+      <c r="P16" s="5" t="inlineStr"/>
+      <c r="Q16" s="5" t="inlineStr"/>
+      <c r="R16" s="5" t="inlineStr"/>
+      <c r="S16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>86</v>
+      </c>
+      <c r="D17" t="n">
+        <v>86</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>20607776912</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N17" s="2" t="inlineStr"/>
+      <c r="O17" s="5" t="inlineStr"/>
+      <c r="P17" s="5" t="inlineStr"/>
+      <c r="Q17" s="5" t="inlineStr"/>
+      <c r="R17" s="5" t="inlineStr"/>
+      <c r="S17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>90</v>
+      </c>
+      <c r="D18" t="n">
+        <v>90</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>20609888769</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N18" s="2" t="inlineStr"/>
+      <c r="O18" s="5" t="inlineStr"/>
+      <c r="P18" s="5" t="inlineStr"/>
+      <c r="Q18" s="5" t="inlineStr"/>
+      <c r="R18" s="5" t="inlineStr"/>
+      <c r="S18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>94</v>
+      </c>
+      <c r="D19" t="n">
+        <v>94</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>20615160653</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Damasco DANCO ares a; fe La Lrbenad T Ifo = Trujillo</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>F001-1258</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>u Damasco DANCO ares a; fe 20615160653 JR FRANCISCO BIZARRO ae 478 INT. 101 La Lrbenad T Ifo = Trujillo Cel 61 Tr FACTURA DE VENTA ELECTRONICA F001- 00001258 20/03/2026 - 11.06 Usuario: CARLOS VILLACORTA, ‘Ubie 004 Forma de Pago: Contado PROGRAMA. NEDUCACION. BASICA PARA TODOS 2038079590 gt CAL. DEL</t>
+        </is>
+      </c>
+      <c r="O19" s="5" t="inlineStr"/>
+      <c r="P19" s="5" t="inlineStr"/>
+      <c r="Q19" s="5" t="inlineStr"/>
+      <c r="R19" s="5" t="inlineStr"/>
+      <c r="S19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>98</v>
+      </c>
+      <c r="D20" t="n">
+        <v>98</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>20613176528</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>F002-2057</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N20" s="2" t="inlineStr"/>
+      <c r="O20" s="5" t="inlineStr"/>
+      <c r="P20" s="5" t="inlineStr"/>
+      <c r="Q20" s="5" t="inlineStr"/>
+      <c r="R20" s="5" t="inlineStr"/>
+      <c r="S20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>102</v>
+      </c>
+      <c r="D21" t="n">
+        <v>102</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>20600593685</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>F018-26030</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N21" s="2" t="inlineStr"/>
+      <c r="O21" s="5" t="inlineStr"/>
+      <c r="P21" s="5" t="inlineStr"/>
+      <c r="Q21" s="5" t="inlineStr"/>
+      <c r="R21" s="5" t="inlineStr"/>
+      <c r="S21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>106</v>
+      </c>
+      <c r="D22" t="n">
+        <v>106</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>20609888769</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N22" s="2" t="inlineStr"/>
+      <c r="O22" s="5" t="inlineStr"/>
+      <c r="P22" s="5" t="inlineStr"/>
+      <c r="Q22" s="5" t="inlineStr"/>
+      <c r="R22" s="5" t="inlineStr"/>
+      <c r="S22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>110</v>
+      </c>
+      <c r="D23" t="n">
+        <v>110</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>20601709016</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>F002-2258</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>wa, Blanca En u?'¡ií¿ wean? &lt; euenie fowtaueann . INVERSIONES CASA BLANCA A &amp; ak RM. LA GENERAL NRO. SIN SEC, CAMPIÑA DE MOC) 20601709016 FACTURA belles Fecne: — 220V2008 — Hera, 14022 RUE - 2 30708007 - PROGRAMA EDUCACIÓN BASICA Razón Social Pana “ CA m…amaa¿ .</t>
+        </is>
+      </c>
+      <c r="O23" s="5" t="inlineStr"/>
+      <c r="P23" s="5" t="inlineStr"/>
+      <c r="Q23" s="5" t="inlineStr"/>
+      <c r="R23" s="5" t="inlineStr"/>
+      <c r="S23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>114</v>
+      </c>
+      <c r="D24" t="n">
+        <v>114</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>20380795907</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>Av. America Sur 2763 Tr N°: FA01-0000007588 Fecha: 23/03/26 10:47 AM CAL.DEL COMERCIO NRO. 193 RES. LAS TC RUC: 20380795907 01 LOMO AL JUGO | ~ 39,00 SubTotal S/ IGV.10.50% S/ICBPERS/ Total S/ 35.29 3.71 0.00 39.00 Medio Pago: Efectivo Forma de Pago: CONTADO</t>
+        </is>
+      </c>
+      <c r="O24" s="5" t="inlineStr"/>
+      <c r="P24" s="5" t="inlineStr"/>
+      <c r="Q24" s="5" t="inlineStr"/>
+      <c r="R24" s="5" t="inlineStr"/>
+      <c r="S24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>118</v>
+      </c>
+      <c r="D25" t="n">
+        <v>118</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>20202961518</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>F219-11456</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>¡ .....u¡:¿¡ux f MA |</t>
+        </is>
+      </c>
+      <c r="O25" s="5" t="inlineStr"/>
+      <c r="P25" s="5" t="inlineStr"/>
+      <c r="Q25" s="5" t="inlineStr"/>
+      <c r="R25" s="5" t="inlineStr"/>
+      <c r="S25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>122</v>
+      </c>
+      <c r="D26" t="n">
+        <v>122</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>boleta_venta</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>20380795907</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LA ESQUINA DEL ESTUDIANTE HERNANDEZ ALMENGOR SILVIA MARLENE BOLETAR%ECY,IE¿:;;OE,II;EÍIRONICA MZA. G INT. 2 PI LOTE. 1 URB. INGENIERIA E'Bº1 1390 TRUJILLO - TRUJILLO - LA LIBERTAD - Fecha de Vencimiento Fecha de Emisión : 23/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de </t>
+        </is>
+      </c>
+      <c r="O26" s="5" t="inlineStr"/>
+      <c r="P26" s="5" t="inlineStr"/>
+      <c r="Q26" s="5" t="inlineStr"/>
+      <c r="R26" s="5" t="inlineStr"/>
+      <c r="S26" s="5" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>126</v>
+      </c>
+      <c r="D27" t="n">
+        <v>126</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>10427606037</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>TAXI ALMANZA</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>E001-16</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>80.00</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="n">
         <v>1</v>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAXI ALMANZA ALMANZA MALLEA EDWIN FACTURA ELECTRONICA A.F. BELLA DURMIENTE PRIMERO MZA. Y LOTE. 11 ALT.AV. CANTO RUC: 10427606037 GRANDE CON AV. CANTO BELLO E001-16 SAN JUAN DE LURIGANCHO - LIMA - LIMA Fecha de Emisión : 09/03/2026 Forma de pago: Contado . PROGRAMA EDUCACION BASICA " PARA TODOS RUC </t>
+        </is>
+      </c>
+      <c r="O27" s="5" t="inlineStr"/>
+      <c r="P27" s="5" t="inlineStr"/>
+      <c r="Q27" s="5" t="inlineStr"/>
+      <c r="R27" s="5" t="inlineStr"/>
+      <c r="S27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>130</v>
+      </c>
+      <c r="D28" t="n">
+        <v>130</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>10181382941</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>A) 10181382941</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>A) 10181382941 Acuario "s SUITE FACTURA ELECTRONICA HOSPEDAJE ACUARIO'S SUITE Dirección : CALLE PRIMAVERA S/N SEC.LA ENCALADA DEL GOLF LA LIBERTAD - TRUJILLO - VICTOR LARCO HERRERA FAO 1 -85 Teléfonos : 065221356 Pagina web : hospedajeacuarios.efactur.pe Razón Social : PROGRAMA EDUCACION BASICA PARA</t>
+        </is>
+      </c>
+      <c r="O28" s="5" t="inlineStr"/>
+      <c r="P28" s="5" t="inlineStr"/>
+      <c r="Q28" s="5" t="inlineStr"/>
+      <c r="R28" s="5" t="inlineStr"/>
+      <c r="S28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>134</v>
+      </c>
+      <c r="D29" t="n">
+        <v>134</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>20131525193</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>HOSPEDAJE EL PALACIO</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>E001-968</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>HOSPEDAJE EL PALACIO SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA. JR. GRAU 709 TRUJILLO - TRUJILLO - LA LIBERTAD FACTURA ELECTRONICA RUC: 20131525193 E001-968 Fecha de Emisión : 21/03/2026 Forma de pago: Contado Señor(es) . PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 . JR. GRAU 709 LA LIBERTAD</t>
+        </is>
+      </c>
+      <c r="O29" s="5" t="inlineStr"/>
+      <c r="P29" s="5" t="inlineStr"/>
+      <c r="Q29" s="5" t="inlineStr"/>
+      <c r="R29" s="5" t="inlineStr"/>
+      <c r="S29" s="5" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>138</v>
+      </c>
+      <c r="D30" t="n">
+        <v>138</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>20131525193</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>HOSPEDAJE EL PALACIO</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>E001-970</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>180.00</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="n">
+        <v>1</v>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
         <is>
           <t>HOSPEDAJE EL PALACIO SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA. JR. GRAU 709 TRUJILLO - TRUJILLO - LA LIBERTAD FACTURA ELECTRONICA RUC: 20131525193 E001-970 Fecha de Emisión : 23/03/2026 Forma de pago: Contado Señor(es) . PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 . JR. GRAU 709 LA LIBERTAD</t>
         </is>
       </c>
-      <c r="O15" s="3" t="inlineStr"/>
-      <c r="P15" s="3" t="inlineStr"/>
-      <c r="Q15" s="3" t="inlineStr"/>
-      <c r="R15" s="3" t="inlineStr"/>
-      <c r="S15" s="3" t="inlineStr"/>
+      <c r="O30" s="5" t="inlineStr"/>
+      <c r="P30" s="5" t="inlineStr"/>
+      <c r="Q30" s="5" t="inlineStr"/>
+      <c r="R30" s="5" t="inlineStr"/>
+      <c r="S30" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S15"/>
+  <autoFilter ref="A1:S30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix #2: razon_social desde paginas de consulta RUC
Enriquecimiento posicional: para cada bloque, buscar la primera
pagina sunat_validez_cpe despues de pagina_fin, luego la primera
sunat_ruc despues de esa CPE. Extraer razon social del formato
SUNAT "Numero de RUC: XXXXXXXXXXX - RAZON SOCIAL" (texto
seleccionable, sin depender de OCR del escaneo).

Cambios:
- comprobante_detector.py: campo razon_social_tentativa en
  BloqueComprobante + bucle de enriquecimiento post-deteccion
- comprobante_extractor.py: preferir razon_social_tentativa del
  bloque sobre el resultado de PASO 4.1 (que falla en escaneos)

Resultado en el piloto DIED2026-INT-0250235:
  razon_social: 8/29 (28%) → 29/29 (100%)
  Todos los demas campos sin cambio (0 regresiones)
  Las 8 anteriores incluian basura OCR; las 29 actuales son texto
  limpio de la consulta RUC de SUNAT.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/piloto_ocr/metrics/validacion_expedientes.xlsx
+++ b/data/piloto_ocr/metrics/validacion_expedientes.xlsx
@@ -1746,7 +1746,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>F_—-— INVERSIONES a SERVICIOS MULTIPLES</t>
+          <t>INVERSIONES &amp; SERVICIOS MULTIPLES COQUITO S.A.C.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -1805,7 +1805,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Cebicheria Coquito SAC.</t>
+          <t>CEBICHERIA COQUITO S.A.C.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>DEGATTA PR¡HPNER¡¡</t>
+          <t>LLF INVERSIONES E.I.R.L.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -1913,7 +1913,11 @@
           <t>10181685510</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>JULCA ULLOA RONALD ALBERTO</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
@@ -1968,7 +1972,11 @@
           <t>10181685510</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>JULCA ULLOA RONALD ALBERTO</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
@@ -2023,7 +2031,11 @@
           <t>20609385317</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>AR REPRESENTACIONES GASTRONÓMICAS S.A.C .</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>F006-00002488</t>
@@ -2070,7 +2082,11 @@
           <t>20611728159</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>TARANTELLA TRX S.A.C</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>F001-00001460</t>
@@ -2121,7 +2137,11 @@
           <t>20608901460</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>LLF INVERSIONES E.I.R.L.</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>F003-2478</t>
@@ -2168,7 +2188,11 @@
           <t>10181685510</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>JULCA ULLOA RONALD ALBERTO</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
@@ -2223,7 +2247,11 @@
           <t>10181685510</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>JULCA ULLOA RONALD ALBERTO</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
@@ -2274,7 +2302,11 @@
           <t>10181727883</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>TAPIA MERINO GLADYS PATRICIA</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
@@ -2329,7 +2361,11 @@
           <t>10181727883</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>TAPIA MERINO GLADYS PATRICIA</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
@@ -2384,7 +2420,11 @@
           <t>20613429388</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>RAFO ALFARO CAFE S.A.C.</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>F001-543</t>
@@ -2435,7 +2475,11 @@
           <t>10181685510</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>JULCA ULLOA RONALD ALBERTO</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
@@ -2490,7 +2534,11 @@
           <t>10181685510</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>JULCA ULLOA RONALD ALBERTO</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
@@ -2545,7 +2593,11 @@
           <t>20607776912</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>QUE BONITA VECINDAD S.A.C.</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
@@ -2588,7 +2640,11 @@
           <t>20609888769</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>SABORES DE TRADICION PERUANA E.I.R.L.</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
@@ -2633,7 +2689,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Damasco DANCO ares a; fe La Lrbenad T Ifo = Trujillo</t>
+          <t>DAMCO CAFE S.A.C.</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2690,7 +2746,11 @@
           <t>20613176528</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>LA ESTAMPIDA DEL MALL S.A.C.</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>F002-2057</t>
@@ -2737,7 +2797,11 @@
           <t>20600593685</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>LUCHA PARTNERS S.A.C.</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
           <t>F018-26030</t>
@@ -2784,7 +2848,11 @@
           <t>20609888769</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>SABORES DE TRADICION PERUANA E.I.R.L.</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
@@ -2827,7 +2895,11 @@
           <t>20601709016</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>INVERSIONES CASA BLANCA A &amp; A S.A.C.</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>F002-2258</t>
@@ -2878,7 +2950,11 @@
           <t>20380795907</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>INVERSIONES &amp; SERVICIOS MULTIPLES COQUITO S.A.C.</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -2929,7 +3005,11 @@
           <t>20202961518</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>INVERSIONES FISA S.A.</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>F219-11456</t>
@@ -2980,7 +3060,11 @@
           <t>20380795907</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>HERNANDEZ ALMENGOR SILVIA MARLENE</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
@@ -3037,7 +3121,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>TAXI ALMANZA</t>
+          <t>ALMANZA MALLEA EDWIN</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3104,7 +3188,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>A) 10181382941</t>
+          <t>BRITO CAMACHO LUMBER</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
@@ -3159,7 +3243,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>HOSPEDAJE EL PALACIO</t>
+          <t>SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -3222,7 +3306,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>HOSPEDAJE EL PALACIO</t>
+          <t>SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">

</xml_diff>

<commit_message>
Fix #3: serie desde paginas CPE — cobertura 12/29 a 29/29
Extiende el bucle de enriquecimiento en detectar_bloques() para
extraer serie_tentativa del texto CPE ademas de razon_social.

Usa un regex local mas amplio que _RE_SERIE para capturar el
formato completo de series SUNAT en las consultas CPE:
  [EFB][A-Z]?\d{2,3}-\d{1,10}
Esto cubre prefijos con letra intermedia (FA01, FB02, FF01, FW01,
EB01) y correlativos zero-padded de hasta 10 digitos.

No modifica _RE_SERIE del primer pase (riesgo de regresion = 0).
El extractor ya usaba bloque.serie_tentativa como fallback.

Resultado en el piloto DIED2026-INT-0250235:
  serie: 12/29 (41%) -> 29/29 (100%)
  29/29 series coinciden con ground truth Anexo 3 SIGA
  Todos los demas campos sin cambio (0 regresiones)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/piloto_ocr/metrics/validacion_expedientes.xlsx
+++ b/data/piloto_ocr/metrics/validacion_expedientes.xlsx
@@ -1749,7 +1749,11 @@
           <t>INVERSIONES &amp; SERVICIOS MULTIPLES COQUITO S.A.C.</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>FA01-0000007538</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
@@ -1763,7 +1767,7 @@
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -1808,7 +1812,11 @@
           <t>CEBICHERIA COQUITO S.A.C.</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>FB02-0000007269</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
@@ -1822,7 +1830,7 @@
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
@@ -1867,13 +1875,17 @@
           <t>LLF INVERSIONES E.I.R.L.</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>F003-0000002453</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
@@ -1918,7 +1930,11 @@
           <t>JULCA ULLOA RONALD ALBERTO</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>FF01-0002114</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>2026-03-11</t>
@@ -1932,7 +1948,7 @@
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
@@ -1977,7 +1993,11 @@
           <t>JULCA ULLOA RONALD ALBERTO</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>FF01-0002122</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t>2026-03-11</t>
@@ -1991,7 +2011,7 @@
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -2193,7 +2213,11 @@
           <t>JULCA ULLOA RONALD ALBERTO</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>FF01-0002135</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
           <t>2026-03-15</t>
@@ -2207,7 +2231,7 @@
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -2252,7 +2276,11 @@
           <t>JULCA ULLOA RONALD ALBERTO</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>FF01-0002136</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
           <t>2026-03-15</t>
@@ -2262,7 +2290,7 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -2307,7 +2335,11 @@
           <t>TAPIA MERINO GLADYS PATRICIA</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>EB01-163</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
           <t>2026-03-17</t>
@@ -2321,7 +2353,7 @@
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -2366,7 +2398,11 @@
           <t>TAPIA MERINO GLADYS PATRICIA</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>EB01-164</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr">
         <is>
           <t>2026-03-17</t>
@@ -2380,7 +2416,7 @@
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
@@ -2480,7 +2516,11 @@
           <t>JULCA ULLOA RONALD ALBERTO</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>FF01-0002139</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
           <t>2026-03-18</t>
@@ -2494,7 +2534,7 @@
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
@@ -2539,7 +2579,11 @@
           <t>JULCA ULLOA RONALD ALBERTO</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>FF01-0002141</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr">
         <is>
           <t>2026-03-18</t>
@@ -2553,7 +2597,7 @@
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
@@ -2598,13 +2642,17 @@
           <t>QUE BONITA VECINDAD S.A.C.</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>FW01-1136</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="N17" s="2" t="inlineStr"/>
       <c r="O17" s="5" t="inlineStr"/>
@@ -2645,13 +2693,17 @@
           <t>SABORES DE TRADICION PERUANA E.I.R.L.</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>FW01-759</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="N18" s="2" t="inlineStr"/>
       <c r="O18" s="5" t="inlineStr"/>
@@ -2853,13 +2905,17 @@
           <t>SABORES DE TRADICION PERUANA E.I.R.L.</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>FW01-763</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="N22" s="2" t="inlineStr"/>
       <c r="O22" s="5" t="inlineStr"/>
@@ -2955,7 +3011,11 @@
           <t>INVERSIONES &amp; SERVICIOS MULTIPLES COQUITO S.A.C.</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>FA01-7588</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
@@ -2965,7 +3025,7 @@
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
@@ -3065,7 +3125,11 @@
           <t>HERNANDEZ ALMENGOR SILVIA MARLENE</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>EB01-1390</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>2026-03-23</t>
@@ -3079,7 +3143,7 @@
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
@@ -3191,7 +3255,11 @@
           <t>BRITO CAMACHO LUMBER</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>FA01-85</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
@@ -3201,7 +3269,7 @@
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix #4: fecha_emision — soportar separadores dash/punto y anio 2 digitos
_norm_date() y _fecha_moneda() en piloto_field_extract_paso4.py solo
aceptaban formato dd/mm/yyyy (slash, 4 digitos). Comprobantes reales
del piloto usan tambien:
  - Fecha: 09/03/26 (2 digitos de anio)
  - Fecha de emision : 10-03-2026 (dash como separador)

Cambios:
- _norm_date: aceptar [-/.] como separador, anios de 2 digitos (+2000)
- _fecha_moneda: buscar con [-/.] y \d{2,4} en vez de solo / y \d{4}

Resultado en el piloto DIED2026-INT-0250235:
  fecha_emision: 13/29 (44%) -> 18/29 (62%)
  +5 fechas recuperadas (p26, p30, p34, p114, p130)
  11 restantes sin fecha: OCR completamente ilegible en esas paginas
  Todos los demas campos sin cambio (0 regresiones)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/piloto_ocr/metrics/validacion_expedientes.xlsx
+++ b/data/piloto_ocr/metrics/validacion_expedientes.xlsx
@@ -1754,7 +1754,11 @@
           <t>FA01-0000007538</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
           <t>108.60</t>
@@ -1767,7 +1771,7 @@
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -1817,7 +1821,11 @@
           <t>FB02-0000007269</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
           <t>98.64</t>
@@ -1830,7 +1838,7 @@
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
@@ -1880,12 +1888,16 @@
           <t>F003-0000002453</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
@@ -3016,7 +3028,11 @@
           <t>FA01-7588</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
@@ -3025,7 +3041,7 @@
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
@@ -3260,7 +3276,11 @@
           <t>FA01-85</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
@@ -3269,7 +3289,7 @@
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix #5: monto_total — fallback desconocido intenta _factura_montos
El fallback para tipo_doc=desconocido en extract_fields_paso4 solo
extraia RUC y retornaba sin intentar montos. Paginas de comprobantes
escaneados clasificadas como desconocido tenian "Importe Total : S/109.00"
legible en el texto OCR, pero el codigo nunca llamaba a _factura_montos().

Cambio: agregar _factura_montos(text) en el fallback desconocido,
antes del return final. Si encuentra monto_total, tambien captura
monto_subtotal y monto_igv con las mismas anclas.

Resultado en el piloto DIED2026-INT-0250235:
  monto_total: 4/29 (13%) -> 8/29 (27%)
  total_detectado: S/ 467.24 -> S/ 790.53
  +4 montos: p66 (109.00), p70 (109.00), p114 (35.29), p122 (70.00)
  21 restantes sin monto: OCR ilegible o sin etiqueta reconocible
  Todos los demas campos sin cambio (0 regresiones)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/piloto_ocr/metrics/validacion_expedientes.xlsx
+++ b/data/piloto_ocr/metrics/validacion_expedientes.xlsx
@@ -2357,15 +2357,23 @@
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>109.00</t>
+        </is>
+      </c>
       <c r="K12" t="inlineStr">
         <is>
           <t>PEN</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
       <c r="M12" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -2420,15 +2428,23 @@
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>109.00</t>
+        </is>
+      </c>
       <c r="K13" t="inlineStr">
         <is>
           <t>PEN</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
       <c r="M13" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
@@ -3033,7 +3049,11 @@
           <t>2026-03-23</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>35.29</t>
+        </is>
+      </c>
       <c r="K24" t="inlineStr">
         <is>
           <t>PEN</t>
@@ -3041,7 +3061,7 @@
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
@@ -3151,15 +3171,23 @@
           <t>2026-03-23</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>70.00</t>
+        </is>
+      </c>
       <c r="K26" t="inlineStr">
         <is>
           <t>PEN</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>6.65</t>
+        </is>
+      </c>
       <c r="M26" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
housekeeping: diagnostico residual + Excel 2 expedientes + limpieza handoffs
- Agrega DIAGNOSTICO_RESIDUAL_PILOTO.txt con gaps residuales de
  fecha (11/29) y monto (21/29) clasificados por tipo de problema
- Excel regenerado con 39 comprobantes (piloto + segundo expediente)
- Elimina handoffs temporales de Cowork (ya consumidos)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/piloto_ocr/metrics/validacion_expedientes.xlsx
+++ b/data/piloto_ocr/metrics/validacion_expedientes.xlsx
@@ -13,11 +13,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="comprobantes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'documentos'!$A$1:$AG$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'expedientes'!$A$1:$I$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'documentos'!$A$1:$AG$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'expedientes'!$A$1:$I$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'errores'!$A$1:$AG$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'resolucion_ids'!$A$1:$I$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'comprobantes'!$A$1:$S$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'resolucion_ids'!$A$1:$I$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'comprobantes'!$A$1:$S$40</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG3"/>
+  <dimension ref="A1:AG6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -671,17 +671,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0250235</t>
+          <t>DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf</t>
+          <t>2026020411112511103251AMIQUERONAHUICARLOS.pdf</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>C:\Users\Hans\Proyectos\vision_rag\DIED2026-INT-0250235\20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf</t>
+          <t>C:\Users\Hans\Proyectos\vision_rag\control_previo\01_viaticos\expedientes_revision\DEBEDSAR2026-INT-0103251\2026020411112511103251AMIQUERONAHUICARLOS.pdf</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -690,16 +690,26 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.783</v>
+        <v>0.706</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>991.70</t>
+        </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2000-02-25</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>LILIANA CHAVEZ TERRONES</t>
+          <t>CARLOS FERNANDO AMIQUERO ÑAHUI</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>00242</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -709,7 +719,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sistema Integrado de Gestión Administrativa Fecha: 3/03/2026 Módulo de Tesorería Hora: 15:01 Versión 25.02.01.U1 , ágina: e PLANILLA DE VIÁTICOS N* Pagina: te UNIDAD EJECUTORA : 026 PROGRAMA EDUCACION BASICA PARA TODOS - 026 NRO. IDENTIFICACIÓN : 000081 Datos del Comisionado: Fecha: 03/03/2026 N° Exp. SIAF: N° Pedido: 572 Sr(a): LILIANA CHAVEZ TERRONES Escala: ESCALA-2 FUNCIONARIOS Y EMPLEADOS N° </t>
+          <t xml:space="preserve">Sistema Integrado de Gestión Administrativa Módulo de Tesorería Versión 25.02.00.U1 UNIDAD EJECUTORA NRO. IDENTIFICACIÓN : : 026 PROGRAMA EDUCACION BASICA PARA TODOS - 026 000081 SOLICITUD DE VIATICOS Nº : 00233 Fecha: Hora: Página: 1 de 1 Centro de Costo: Solicitante: Motivo del Viaje: APLICACIÓN DE LA I FASE - PUA 2026; AMIQUERO ÑAHUI, CARLOS FERNANDO; DNI :42192880; DIRECCIÓN: URB. LOS MÉDANOS </t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -724,17 +734,17 @@
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
-          <t>SINAD-250235</t>
+          <t>SINAD-103251</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>250235</t>
+          <t>103251</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>2603426</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -743,22 +753,22 @@
         </is>
       </c>
       <c r="W2" t="n">
-        <v>0.838</v>
+        <v>0.85</v>
       </c>
       <c r="X2" t="n">
-        <v>0.912</v>
+        <v>0.85</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.485</v>
+        <v>0.889</v>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>siaf:conflicto: top=SIAF-2603426(16.0) vs segundo=SIAF-3205(16.0)</t>
+          <t>siaf:score_max=8.0&lt;umbral_min=10.0</t>
         </is>
       </c>
       <c r="AB2" s="5" t="n"/>
@@ -771,83 +781,80 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0250235</t>
+          <t>DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+          <t>2026040910538RIDECARLOSAMIQUERO.pdf</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>C:\Users\Hans\Proyectos\vision_rag\DIED2026-INT-0250235\2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+          <t>C:\Users\Hans\Proyectos\vision_rag\control_previo\01_viaticos\expedientes_revision\DEBEDSAR2026-INT-0103251\2026040910538RIDECARLOSAMIQUERO.pdf</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>rendicion</t>
+          <t>otros</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.49</v>
+        <v>0.889</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>138.70</t>
+        </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>20380795907</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>900-4-2026</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>viaticos</t>
+          <t>desconocido</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>ANEXO N°3 Fecha : Hora : Página : 1 de 2 09/04/2026 13:01 Sistema Integrado de Gestión Módulo de Tesorería Versión 22.04.00 026 PROGRAMA EDUCACION BASICA PARA TODOS - 026 000081 Datos del CHAVEZ TERRONES LILIANA Sr(a): N° Planilla: Motivo de Salida: 00617 N° Exp SIAF: 2603426 N° Comprobante 09/03/2026 Regreso: N° Días/Horas: 11d 23h APLICACION DE INSTRUMENTOS PARA RECOJO DE INFORMACION A CARGO DEL</t>
+          <t>DIA MES UE.026 (0081) PROGRAMA EDUCACION BASICA PARA TODOS - MINEDU RUC N°: 20380795907 AMIQUERO ÑAHUI CARLOS FERNANDO DEVOLUCIÓN DE VIÁTICOS 232121 TRANSPORTE NACIONAL 232122 VIATICOS NACIONAL 2327999 OTROS RELACIONADOS A ORGANIZACIÓN DE EVENTOS 155149 REPARACION CIVIL 23271498 OTROS SERVICIOS TECNICOS Y PROFESIONALES 152211 SANCIONES ADMINISTRATIVAS 1339199 OTROS SERVICIOS DE ADMINISTRACION Y RE</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>bajo_confianza</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>override_consolidado_rendicion: top_regex=factura(45) pero filename+encabezado indican rendicion(24)</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>firmas_anexo3</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>INSUFICIENTE_EVIDENCIA</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>nombre_ilegible:comisionado:anchor=dni_sin_nombre_adyacente; nombre_ilegible:jefe_unidad:anchor=sin_anchor; rol_no_detectado:vb_coordinador</t>
-        </is>
-      </c>
-      <c r="R3" t="n">
-        <v>0.1</v>
-      </c>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
-          <t>SINAD-250235</t>
+          <t>SINAD-103251</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>250235</t>
+          <t>103251</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>2603426</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -856,22 +863,22 @@
         </is>
       </c>
       <c r="W3" t="n">
-        <v>0.838</v>
+        <v>0.85</v>
       </c>
       <c r="X3" t="n">
-        <v>0.912</v>
+        <v>0.85</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.485</v>
+        <v>0.889</v>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>siaf:conflicto: top=SIAF-2603426(16.0) vs segundo=SIAF-3205(16.0)</t>
+          <t>siaf:score_max=8.0&lt;umbral_min=10.0</t>
         </is>
       </c>
       <c r="AB3" s="5" t="n"/>
@@ -881,8 +888,334 @@
       <c r="AF3" s="5" t="n"/>
       <c r="AG3" s="5" t="n"/>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DEBEDSAR2026-INT-0103251</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>C:\Users\Hans\Proyectos\vision_rag\control_previo\01_viaticos\expedientes_revision\DEBEDSAR2026-INT-0103251\202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>rendicion</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>0.481</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>viaticos</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Sistema Integrado de Gestión Fecha : 06/04/2026 Módulo de Tesorería Hora : 17:37 Version 22.04.00 Pagina : 1 det ANEXO N*3 RENDICION DE CUENTAS POR COMISION DE SERVICIOS UNIDAD EJECUTORA : 026 PROGRAMA EDUCACION BASICA PARA TODOS - 026 NRO. IDENTIFICACIÓN : 000081 Datos del Sr(a): AMIQUERO ÑAHUI CARLOS FERNANDO N° Planilla: 00242 N° Exp SIAF: 00001792 N° Comprobante 2601620 Motivo de APLICACION DE</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>bajo_confianza</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>override_consolidado_rendicion: top_regex=factura(33) pero filename+encabezado indican rendicion(13)</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>firmas_anexo3</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>OBSERVADO</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>nombre_ilegible:jefe_unidad:anchor=sin_anchor; rol_no_detectado:vb_coordinador</t>
+        </is>
+      </c>
+      <c r="R4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>SINAD-103251</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>103251</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>1792</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="W4" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>0.889</v>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>siaf:score_max=8.0&lt;umbral_min=10.0</t>
+        </is>
+      </c>
+      <c r="AB4" s="5" t="n"/>
+      <c r="AC4" s="5" t="n"/>
+      <c r="AD4" s="5" t="n"/>
+      <c r="AE4" s="5" t="n"/>
+      <c r="AF4" s="5" t="n"/>
+      <c r="AG4" s="5" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>C:\Users\Hans\Proyectos\vision_rag\DIED2026-INT-0250235\20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>solicitud</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0.783</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>LILIANA CHAVEZ TERRONES</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>viaticos</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sistema Integrado de Gestión Administrativa Fecha: 3/03/2026 Módulo de Tesorería Hora: 15:01 Versión 25.02.01.U1 , ágina: e PLANILLA DE VIÁTICOS N* Pagina: te UNIDAD EJECUTORA : 026 PROGRAMA EDUCACION BASICA PARA TODOS - 026 NRO. IDENTIFICACIÓN : 000081 Datos del Comisionado: Fecha: 03/03/2026 N° Exp. SIAF: N° Pedido: 572 Sr(a): LILIANA CHAVEZ TERRONES Escala: ESCALA-2 FUNCIONARIOS Y EMPLEADOS N° </t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>SINAD-250235</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>250235</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>2603426</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="W5" t="n">
+        <v>0.838</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0.912</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0.485</v>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>siaf:conflicto: top=SIAF-2603426(16.0) vs segundo=SIAF-3205(16.0)</t>
+        </is>
+      </c>
+      <c r="AB5" s="5" t="n"/>
+      <c r="AC5" s="5" t="n"/>
+      <c r="AD5" s="5" t="n"/>
+      <c r="AE5" s="5" t="n"/>
+      <c r="AF5" s="5" t="n"/>
+      <c r="AG5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>C:\Users\Hans\Proyectos\vision_rag\DIED2026-INT-0250235\2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>rendicion</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>viaticos</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>ANEXO N°3 Fecha : Hora : Página : 1 de 2 09/04/2026 13:01 Sistema Integrado de Gestión Módulo de Tesorería Versión 22.04.00 026 PROGRAMA EDUCACION BASICA PARA TODOS - 026 000081 Datos del CHAVEZ TERRONES LILIANA Sr(a): N° Planilla: Motivo de Salida: 00617 N° Exp SIAF: 2603426 N° Comprobante 09/03/2026 Regreso: N° Días/Horas: 11d 23h APLICACION DE INSTRUMENTOS PARA RECOJO DE INFORMACION A CARGO DEL</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>bajo_confianza</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>override_consolidado_rendicion: top_regex=factura(45) pero filename+encabezado indican rendicion(24)</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>firmas_anexo3</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>INSUFICIENTE_EVIDENCIA</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>nombre_ilegible:comisionado:anchor=dni_sin_nombre_adyacente; nombre_ilegible:jefe_unidad:anchor=sin_anchor; rol_no_detectado:vb_coordinador</t>
+        </is>
+      </c>
+      <c r="R6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>SINAD-250235</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>250235</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>2603426</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="W6" t="n">
+        <v>0.838</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0.912</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0.485</v>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>siaf:conflicto: top=SIAF-2603426(16.0) vs segundo=SIAF-3205(16.0)</t>
+        </is>
+      </c>
+      <c r="AB6" s="5" t="n"/>
+      <c r="AC6" s="5" t="n"/>
+      <c r="AD6" s="5" t="n"/>
+      <c r="AE6" s="5" t="n"/>
+      <c r="AF6" s="5" t="n"/>
+      <c r="AG6" s="5" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AG3"/>
+  <autoFilter ref="A1:AG6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -893,7 +1226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -957,24 +1290,24 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0250235</t>
+          <t>DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>C:\Users\Hans\Proyectos\vision_rag\DIED2026-INT-0250235</t>
+          <t>C:\Users\Hans\Proyectos\vision_rag\control_previo\01_viaticos\expedientes_revision\DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>C:\Users\Hans\Proyectos\vision_rag\control_previo\procesados\DIED2026-INT-0250235</t>
+          <t>C:\Users\Hans\Proyectos\vision_rag\control_previo\procesados\DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="D2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" t="n">
         <v>2</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1</v>
       </c>
       <c r="F2" t="n">
         <v>1</v>
@@ -984,17 +1317,56 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
+          <t>otros, rendicion, solicitud</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-04-17T03:19:45-0500</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>C:\Users\Hans\Proyectos\vision_rag\DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>C:\Users\Hans\Proyectos\vision_rag\control_previo\procesados\DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>rendicion, solicitud</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>2026-04-14T16:39:29-0500</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I2"/>
+  <autoFilter ref="A1:I3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1222,7 +1594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1286,12 +1658,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0250235</t>
+          <t>DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SINAD-250235</t>
+          <t>SINAD-103251</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1300,10 +1672,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>166</v>
+        <v>91</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1317,19 +1689,19 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>CONFLICTO_EXPEDIENTE</t>
+          <t>BAJA_CONFIANZA</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1; 20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p2; 20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p3; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p1; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p2</t>
+          <t>2026020411112511103251AMIQUERONAHUICARLOS.pdf:p1; 2026020411112511103251AMIQUERONAHUICARLOS.pdf:p2; 202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf:p1; 202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf:p2; 202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf:p7</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0250235</t>
+          <t>DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1346,7 +1718,7 @@
         <v>7</v>
       </c>
       <c r="E3" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1360,36 +1732,36 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>CONFLICTO_EXPEDIENTE</t>
+          <t>BAJA_CONFIANZA</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1; 20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1; 20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p8; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p1</t>
+          <t>2026020411112511103251AMIQUERONAHUICARLOS.pdf:p1; 2026020411112511103251AMIQUERONAHUICARLOS.pdf:p1; 2026020411112511103251AMIQUERONAHUICARLOS.pdf:p1; 2026040910538RIDECARLOSAMIQUERO.pdf:p1; 202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf:p1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0250235</t>
+          <t>DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SIAF-2603426</t>
+          <t>SINAD-116260</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>siaf</t>
+          <t>sinad</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1403,24 +1775,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>CONFLICTO_EXPEDIENTE</t>
+          <t>BAJA_CONFIANZA</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p1; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p2</t>
+          <t>2026020411112511103251AMIQUERONAHUICARLOS.pdf:p7</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0250235</t>
+          <t>DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SIAF-3205</t>
+          <t>SIAF-1792</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1429,10 +1801,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1446,36 +1818,36 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>CONFLICTO_EXPEDIENTE</t>
+          <t>BAJA_CONFIANZA</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p8; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p150</t>
+          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf:p1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0250235</t>
+          <t>DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>EXP-DIED-2026-250235</t>
+          <t>PLANILLA-00242</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>exp</t>
+          <t>planilla</t>
         </is>
       </c>
       <c r="D6" t="n">
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1489,36 +1861,36 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>CONFLICTO_EXPEDIENTE</t>
+          <t>BAJA_CONFIANZA</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p8</t>
+          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf:p1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0250235</t>
+          <t>DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SINAD-112591</t>
+          <t>PEDIDO-233</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>sinad</t>
+          <t>pedido</t>
         </is>
       </c>
       <c r="D7" t="n">
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1532,12 +1904,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>CONFLICTO_EXPEDIENTE</t>
+          <t>BAJA_CONFIANZA</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p9</t>
+          <t>2026020411112511103251AMIQUERONAHUICARLOS.pdf:p2</t>
         </is>
       </c>
     </row>
@@ -1549,43 +1921,301 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>SINAD-250235</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>sinad</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E8" t="n">
+        <v>166</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>CONFLICTO_EXPEDIENTE</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1; 20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p2; 20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p3; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p1; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ANIO-2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>anio</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>7</v>
+      </c>
+      <c r="E9" t="n">
+        <v>26</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>CONFLICTO_EXPEDIENTE</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1; 20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1; 20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p8; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p1</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SIAF-2603426</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>siaf</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>16</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>CONFLICTO_EXPEDIENTE</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p1; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SIAF-3205</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>siaf</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>16</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>CONFLICTO_EXPEDIENTE</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p8; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p150</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>EXP-DIED-2026-250235</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>exp</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>16</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>CONFLICTO_EXPEDIENTE</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p8</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>SINAD-112591</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>sinad</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>15</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>CONFLICTO_EXPEDIENTE</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p9</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>PEDIDO-572</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>pedido</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D14" t="n">
         <v>2</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E14" t="n">
         <v>7</v>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>CONFLICTO_EXPEDIENTE</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf:p1; 2026041320235RENDICLILIANACHAVEZSINAD250235.pdf:p3</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I8"/>
+  <autoFilter ref="A1:I14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1596,7 +2226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S30"/>
+  <dimension ref="A1:S40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1720,19 +2350,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0250235</t>
+          <t>DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="D2" t="n">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1741,29 +2371,25 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>20477689699</t>
+          <t>20515659324</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>INVERSIONES &amp; SERVICIOS MULTIPLES COQUITO S.A.C.</t>
+          <t>TURISMO INTERNACIONAL PALOMINO S.A.C.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>FA01-0000007538</t>
+          <t>F235-0040130</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>108.60</t>
-        </is>
-      </c>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>PEN</t>
@@ -1771,11 +2397,11 @@
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>F_—-— — INVERSIONES a SERVICIOS MULTIPLES COQUITO S.A Av. America Sut 2763 Palle La Libertad *** COQUITO *** Teléfono ; 044-224451 RUC: 20477689699 L FACTURA DE VENTA ELECTRÓNICA NO: FAO1-0000007538 Mesa: A-9 Fecha: 09/03/26 01:50 PM WALTER Cliente: Teléf: - PROGRAMA EDUCACION BASICA PARA TODOS CAL.</t>
+          <t>TURISMO INTERNACIONAL PALOMINO S.A.C. AV. NICOLAS ARRIOLA NRO. 910 URB. SANTA CATALINA - LI RUC; 20515659324 FACTURA ELECTRONICA F235-0040130 RUC; 20380795907 RAZON SOC PROGRAMA EDUCACION BASICA PARA TODOS E TOTAL 1 SERVICIO DE TRANSPORTE EN LA 80.00 RUTA: ICA PUQUIO ASIENTO: 39 PASAJERO: CARLOS FER</t>
         </is>
       </c>
       <c r="O2" s="5" t="inlineStr"/>
@@ -1787,19 +2413,19 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0250235</t>
+          <t>DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="D3" t="n">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1808,27 +2434,27 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>20539971477</t>
+          <t>10288513673</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>CEBICHERIA COQUITO S.A.C.</t>
+          <t>RESTAURANT HATUN WASI</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>FB02-0000007269</t>
+          <t>F001-00001706</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>98.64</t>
+          <t>46.00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -1836,13 +2462,17 @@
           <t>PEN</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>7.02</t>
+        </is>
+      </c>
       <c r="M3" t="n">
         <v>1</v>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Cebicheria Coquito SAC. Honorio Delgado Mz Q’ Lote 2 El Bosque - Trujillo - La Ll bertad *** COQUITO *** Teléfono : 044-215511 RUC: 20539971477 — FACTURA DE VENTA ELECTRÓNICA Ne: FBO2-0000007269 Mesa: A-16 Fecha: 10/03/26 02:42 PM EDUARDO Cliente: Teléf: - PROGRAMA EDUCACION BASICA PARA TODOS CAL,DE</t>
+          <t>Representación impresa de la FACTURA ELECTRÓNICA. Esta puede ser consultada en https://hatunwasi.cpesimple.online/buscar RESTAURANT HATUN WASI De: PACHECO COYLLO GLORIA YOLANDA JR. LEONCIO PRADO N° 295 , PUQUIO , LUCANAS - AYACUCHO D. Comercial: JR. LEONCIO PRADO N° 295 935 737 974 yolandaccoyllopac</t>
         </is>
       </c>
       <c r="O3" s="5" t="inlineStr"/>
@@ -1854,19 +2484,19 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0250235</t>
+          <t>DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D4" t="n">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1875,33 +2505,45 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>20608901460</t>
+          <t>10288513673</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>LLF INVERSIONES E.I.R.L.</t>
+          <t>RESTAURANT HATUN WASI</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>F003-0000002453</t>
+          <t>F001-00001707</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>80.00</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>12.20</t>
+        </is>
+      </c>
       <c r="M4" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>DEGATTA PR¡HPNER¡¡ Le INVERSIONES É,T:R Jiron Ayacucho: 521; fry eae Peru — Trujillo. . Rue: 20608901460 FACTURA ELECTRONICA FO03-0000002483 “Orden: ov-094765 Fecha de emision : 10-03-2026 he SALON) PRINCIP AL " Rur. 2038!1 795907 Razon social - “PROGRAMA EDUCACION BASICA PARA TO Bop CALs DEL COMERC</t>
+          <t>Representación impresa de la FACTURA ELECTRÓNICA. Esta puede ser consultada en https://hatunwasi.cpesimple.online/buscar RESTAURANT HATUN WASI De: PACHECO COYLLO GLORIA YOLANDA JR. LEONCIO PRADO N° 295 , PUQUIO , LUCANAS - AYACUCHO D. Comercial: JR. LEONCIO PRADO N° 295 935 737 974 yolandaccoyllopac</t>
         </is>
       </c>
       <c r="O4" s="5" t="inlineStr"/>
@@ -1913,19 +2555,19 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0250235</t>
+          <t>DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="D5" t="n">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1934,37 +2576,45 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>10181685510</t>
+          <t>10288513673</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>JULCA ULLOA RONALD ALBERTO</t>
+          <t>RESTAURANT HATUN WASI</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>FF01-0002114</t>
+          <t>F001-00001711</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>45.00</t>
+        </is>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>PEN</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>6.86</t>
+        </is>
+      </c>
       <c r="M5" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002114 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 11/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+          <t>Representación impresa de la FACTURA ELECTRÓNICA. Esta puede ser consultada en https://hatunwasi.cpesimple.online/buscar RESTAURANT HATUN WASI De: PACHECO COYLLO GLORIA YOLANDA JR. LEONCIO PRADO N° 295 , PUQUIO , LUCANAS - AYACUCHO D. Comercial: JR. LEONCIO PRADO N° 295 935 737 974 yolandaccoyllopac</t>
         </is>
       </c>
       <c r="O5" s="5" t="inlineStr"/>
@@ -1976,19 +2626,19 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0250235</t>
+          <t>DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="D6" t="n">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1997,37 +2647,45 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>10181685510</t>
+          <t>10288019482</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>JULCA ULLOA RONALD ALBERTO</t>
+          <t>POLLOS A LA</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>FF01-0002122</t>
+          <t>F003-2106</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>50.00</t>
+        </is>
+      </c>
       <c r="K6" t="inlineStr">
         <is>
           <t>PEN</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>4.55</t>
+        </is>
+      </c>
       <c r="M6" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002122 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 11/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+          <t>POLLOS A LA BRASA RESTAURANTE EL “DORADO” De: CRUZ MURIEL DORIS R.U.C. : 10288019482 Ofrece: Pollos a La Brasa, Brosther, Salchipapas, Platos Extras, Menú Ejecutivo, Menú Económico Bebidas Calientes, Frías, Gaseosas, Licores, Vinos, Cervezas y Otros. HOSPEDAJE IMPERIAL: Habitaciones Confortables con</t>
         </is>
       </c>
       <c r="O6" s="5" t="inlineStr"/>
@@ -2039,19 +2697,19 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0250235</t>
+          <t>DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="D7" t="n">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -2060,27 +2718,47 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>20609385317</t>
+          <t>10288513673</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>AR REPRESENTACIONES GASTRONÓMICAS S.A.C .</t>
+          <t>RESTAURANT HATUN WASI</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>F006-00002488</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
+          <t>F001-00001712</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>32.00</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>4.88</t>
+        </is>
+      </c>
       <c r="M7" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N7" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>Representación impresa de la FACTURA ELECTRÓNICA. Esta puede ser consultada en https://hatunwasi.cpesimple.online/buscar RESTAURANT HATUN WASI De: PACHECO COYLLO GLORIA YOLANDA JR. LEONCIO PRADO N° 295 , PUQUIO , LUCANAS - AYACUCHO D. Comercial: JR. LEONCIO PRADO N° 295 935 737 974 yolandaccoyllopac</t>
+        </is>
+      </c>
       <c r="O7" s="5" t="inlineStr"/>
       <c r="P7" s="5" t="inlineStr"/>
       <c r="Q7" s="5" t="inlineStr"/>
@@ -2090,19 +2768,19 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0250235</t>
+          <t>DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="D8" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -2111,29 +2789,45 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>20611728159</t>
+          <t>20615320561</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>TARANTELLA TRX S.A.C</t>
+          <t>POLLOS A LA BRASA AMIGOS S.A.C.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>F001-00001460</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
+          <t>E001-27</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>35.00</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>5.34</t>
+        </is>
+      </c>
       <c r="M8" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>' - mm lt 1 ‘ E Á -¡:I;'.'. ) h — ' LF TRA.</t>
+          <t xml:space="preserve">POLLOS &amp; PARRILLAS AMIGOS POLLOS A LA BRASA AMIGOS S.A.C. JR. SAISA KM. 223 A 1 CUADRA DE LA PANAMERICANA PUQUIO - LUCANAS - AYACUCHO FACTURA ELECTRONICA RUC: 20615320561 E001-27 Fecha de Emisión : 08/02/2026 Señor(es) : PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 Dirección del Cliente : </t>
         </is>
       </c>
       <c r="O8" s="5" t="inlineStr"/>
@@ -2145,19 +2839,19 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0250235</t>
+          <t>DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="D9" t="n">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -2166,27 +2860,47 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>20608901460</t>
+          <t>20612666751</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>LLF INVERSIONES E.I.R.L.</t>
+          <t>HOTEL SUMAC SAMARI S.A.C.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>F003-2478</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
+          <t>E001-478</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>300.00</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>28.51</t>
+        </is>
+      </c>
       <c r="M9" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N9" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FACTURA ELECTRONICA RUC: 20612666751 E001-478 Sub Total Ventas : S/ 271.49 Anticipos : S/ 0.00 Descuentos : S/ 0.00 Valor Venta : S/ 271.49 ISC : S/ 0.00 IGV : S/ 28.51 ICBPER : S/ 0.00 Otros Cargos : S/ 0.00 Otros Tributos : S/ 0.00 Monto de redondeo : S/ 0.00 Importe Total : S/ 300.00 HOTEL SUMAC </t>
+        </is>
+      </c>
       <c r="O9" s="5" t="inlineStr"/>
       <c r="P9" s="5" t="inlineStr"/>
       <c r="Q9" s="5" t="inlineStr"/>
@@ -2196,19 +2910,19 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0250235</t>
+          <t>DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>58</v>
+        <v>27</v>
       </c>
       <c r="D10" t="n">
-        <v>58</v>
+        <v>27</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -2217,37 +2931,45 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10181685510</t>
+          <t>20611798637</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>JULCA ULLOA RONALD ALBERTO</t>
+          <t>E T M TOURS PUQUIO-NASCA S.A.C.</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>FF01-0002135</t>
+          <t>E001-324</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr"/>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>40.00</t>
+        </is>
+      </c>
       <c r="K10" t="inlineStr">
         <is>
           <t>PEN</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
       <c r="M10" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002135 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 15/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+          <t>E T M TOURS PUQUIO-NASCA SOCIEDAD ANONIMA CERRADA JR. OCAÑA SIN NUMERO SEGUNDA SN PUQUIO - LUCANAS - AYACUCHO FACTURA ELECTRONICA RUC: 20611798637 E001-324 Fecha de Emisión : 08/02/2026 Señor(es) : PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 Establecimiento del Emisor : JR. OCAÃ‘A SIN NUM</t>
         </is>
       </c>
       <c r="O10" s="5" t="inlineStr"/>
@@ -2259,19 +2981,19 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0250235</t>
+          <t>DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="D11" t="n">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2280,33 +3002,45 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>10181685510</t>
+          <t>20606737310</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>JULCA ULLOA RONALD ALBERTO</t>
+          <t>MULTISERVICIOS ASIEL S.A.C.</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>FF01-0002136</t>
+          <t>E001-2203</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>35.00</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>5.34</t>
+        </is>
+      </c>
       <c r="M11" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002136 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 15/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+          <t>MULTISERVICIOS ASIEL S.A.C. MULTISERVICIOS ASIEL S.A.C. C.P. SIN BARRIO COMATRANA MZA. Q LOTE. 18 CP. COMATRANA ICA - ICA - ICA FACTURA ELECTRONICA RUC: 20606737310 E001-2203 Fecha de Emisión : 08/02/2026 Señor(es) : PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 Dirección del Cliente : CAL.</t>
         </is>
       </c>
       <c r="O11" s="5" t="inlineStr"/>
@@ -2327,39 +3061,39 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>66</v>
+        <v>26</v>
       </c>
       <c r="D12" t="n">
-        <v>66</v>
+        <v>26</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>boleta_venta</t>
+          <t>factura_electronica</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>10181727883</t>
+          <t>20477689699</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>TAPIA MERINO GLADYS PATRICIA</t>
+          <t>INVERSIONES &amp; SERVICIOS MULTIPLES COQUITO S.A.C.</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>EB01-163</t>
+          <t>FA01-0000007538</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>109.00</t>
+          <t>108.60</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -2367,17 +3101,13 @@
           <t>PEN</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
+      <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
         <v>1</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>BOLETA DE VENTA ELECTRONICA RUC: 10181727883 EB01-163 TAPIA MERINO GLADYS PATRICIA JR. LOS RUBIES 383 URB. SANTA INES TRUJILLO - TRUJILLO - LA LIBERTAD Fecha de Vencimiento Fecha de Emisión : 17/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Observación : S</t>
+          <t>F_—-— — INVERSIONES a SERVICIOS MULTIPLES COQUITO S.A Av. America Sut 2763 Palle La Libertad *** COQUITO *** Teléfono ; 044-224451 RUC: 20477689699 L FACTURA DE VENTA ELECTRÓNICA NO: FAO1-0000007538 Mesa: A-9 Fecha: 09/03/26 01:50 PM WALTER Cliente: Teléf: - PROGRAMA EDUCACION BASICA PARA TODOS CAL.</t>
         </is>
       </c>
       <c r="O12" s="5" t="inlineStr"/>
@@ -2398,39 +3128,39 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="D13" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>boleta_venta</t>
+          <t>factura_electronica</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>10181727883</t>
+          <t>20539971477</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>TAPIA MERINO GLADYS PATRICIA</t>
+          <t>CEBICHERIA COQUITO S.A.C.</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>EB01-164</t>
+          <t>FB02-0000007269</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>109.00</t>
+          <t>98.64</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -2438,17 +3168,13 @@
           <t>PEN</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
+      <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
         <v>1</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>BOLETA DE VENTA ELECTRONICA RUC: 10181727883 EB01-164 TAPIA MERINO GLADYS PATRICIA JR. LOS RUBIES 383 URB. SANTA INES TRUJILLO - TRUJILLO - LA LIBERTAD Fecha de Vencimiento Fecha de Emisión : 17/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Observación : S</t>
+          <t>Cebicheria Coquito SAC. Honorio Delgado Mz Q’ Lote 2 El Bosque - Trujillo - La Ll bertad *** COQUITO *** Teléfono : 044-215511 RUC: 20539971477 — FACTURA DE VENTA ELECTRÓNICA Ne: FBO2-0000007269 Mesa: A-16 Fecha: 10/03/26 02:42 PM EDUARDO Cliente: Teléf: - PROGRAMA EDUCACION BASICA PARA TODOS CAL,DE</t>
         </is>
       </c>
       <c r="O13" s="5" t="inlineStr"/>
@@ -2469,10 +3195,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>74</v>
+        <v>34</v>
       </c>
       <c r="D14" t="n">
-        <v>74</v>
+        <v>34</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2481,29 +3207,33 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>20613429388</t>
+          <t>20608901460</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>RAFO ALFARO CAFE S.A.C.</t>
+          <t>LLF INVERSIONES E.I.R.L.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>F001-543</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr"/>
+          <t>F003-0000002453</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>16134 &lt;1 LOTE 8 URB SAN ey II ET s eet) M mta¿ — aE E 90 eo 1700 R ',frasnntaainn arte del Comprobant th e Electro) eS \Gracias Par ei preferencial h Sunwnro eRestaurant - 9764 77688</t>
+          <t>DEGATTA PR¡HPNER¡¡ Le INVERSIONES É,T:R Jiron Ayacucho: 521; fry eae Peru — Trujillo. . Rue: 20608901460 FACTURA ELECTRONICA FO03-0000002483 “Orden: ov-094765 Fecha de emision : 10-03-2026 he SALON) PRINCIP AL " Rur. 2038!1 795907 Razon social - “PROGRAMA EDUCACION BASICA PARA TO Bop CALs DEL COMERC</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr"/>
@@ -2524,10 +3254,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>78</v>
+        <v>38</v>
       </c>
       <c r="D15" t="n">
-        <v>78</v>
+        <v>38</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2546,12 +3276,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>FF01-0002139</t>
+          <t>FF01-0002114</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -2566,7 +3296,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002139 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 18/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002114 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 11/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
         </is>
       </c>
       <c r="O15" s="5" t="inlineStr"/>
@@ -2587,10 +3317,10 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>82</v>
+        <v>42</v>
       </c>
       <c r="D16" t="n">
-        <v>82</v>
+        <v>42</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2609,12 +3339,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>FF01-0002141</t>
+          <t>FF01-0002122</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -2629,7 +3359,7 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002141 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 18/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002122 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 11/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
         </is>
       </c>
       <c r="O16" s="5" t="inlineStr"/>
@@ -2650,10 +3380,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>86</v>
+        <v>46</v>
       </c>
       <c r="D17" t="n">
-        <v>86</v>
+        <v>46</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2662,17 +3392,17 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>20607776912</t>
+          <t>20609385317</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>QUE BONITA VECINDAD S.A.C.</t>
+          <t>AR REPRESENTACIONES GASTRONÓMICAS S.A.C .</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>FW01-1136</t>
+          <t>F006-00002488</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
@@ -2701,10 +3431,10 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="D18" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -2713,17 +3443,17 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>20609888769</t>
+          <t>20611728159</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>SABORES DE TRADICION PERUANA E.I.R.L.</t>
+          <t>TARANTELLA TRX S.A.C</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>FW01-759</t>
+          <t>F001-00001460</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
@@ -2733,7 +3463,11 @@
       <c r="M18" t="n">
         <v>0.5</v>
       </c>
-      <c r="N18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>' - mm lt 1 ‘ E Á -¡:I;'.'. ) h — ' LF TRA.</t>
+        </is>
+      </c>
       <c r="O18" s="5" t="inlineStr"/>
       <c r="P18" s="5" t="inlineStr"/>
       <c r="Q18" s="5" t="inlineStr"/>
@@ -2752,10 +3486,10 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>94</v>
+        <v>54</v>
       </c>
       <c r="D19" t="n">
-        <v>94</v>
+        <v>54</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -2764,35 +3498,27 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>20615160653</t>
+          <t>20608901460</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>DAMCO CAFE S.A.C.</t>
+          <t>LLF INVERSIONES E.I.R.L.</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>F001-1258</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
+          <t>F003-2478</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>u Damasco DANCO ares a; fe 20615160653 JR FRANCISCO BIZARRO ae 478 INT. 101 La Lrbenad T Ifo = Trujillo Cel 61 Tr FACTURA DE VENTA ELECTRONICA F001- 00001258 20/03/2026 - 11.06 Usuario: CARLOS VILLACORTA, ‘Ubie 004 Forma de Pago: Contado PROGRAMA. NEDUCACION. BASICA PARA TODOS 2038079590 gt CAL. DEL</t>
-        </is>
-      </c>
+        <v>0.5</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr"/>
       <c r="O19" s="5" t="inlineStr"/>
       <c r="P19" s="5" t="inlineStr"/>
       <c r="Q19" s="5" t="inlineStr"/>
@@ -2811,10 +3537,10 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>98</v>
+        <v>58</v>
       </c>
       <c r="D20" t="n">
-        <v>98</v>
+        <v>58</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -2823,27 +3549,39 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>20613176528</t>
+          <t>10181685510</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>LA ESTAMPIDA DEL MALL S.A.C.</t>
+          <t>JULCA ULLOA RONALD ALBERTO</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>F002-2057</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr"/>
+          <t>FF01-0002135</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
       <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N20" s="2" t="inlineStr"/>
+        <v>0.75</v>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002135 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 15/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+        </is>
+      </c>
       <c r="O20" s="5" t="inlineStr"/>
       <c r="P20" s="5" t="inlineStr"/>
       <c r="Q20" s="5" t="inlineStr"/>
@@ -2862,10 +3600,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>102</v>
+        <v>62</v>
       </c>
       <c r="D21" t="n">
-        <v>102</v>
+        <v>62</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -2874,27 +3612,35 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>20600593685</t>
+          <t>10181685510</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>LUCHA PARTNERS S.A.C.</t>
+          <t>JULCA ULLOA RONALD ALBERTO</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>F018-26030</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr"/>
+          <t>FF01-0002136</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N21" s="2" t="inlineStr"/>
+        <v>0.75</v>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002136 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 15/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
+        </is>
+      </c>
       <c r="O21" s="5" t="inlineStr"/>
       <c r="P21" s="5" t="inlineStr"/>
       <c r="Q21" s="5" t="inlineStr"/>
@@ -2913,39 +3659,59 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>106</v>
+        <v>66</v>
       </c>
       <c r="D22" t="n">
-        <v>106</v>
+        <v>66</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>factura_electronica</t>
+          <t>boleta_venta</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>20609888769</t>
+          <t>10181727883</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>SABORES DE TRADICION PERUANA E.I.R.L.</t>
+          <t>TAPIA MERINO GLADYS PATRICIA</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>FW01-763</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
+          <t>EB01-163</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>109.00</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
       <c r="M22" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N22" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>BOLETA DE VENTA ELECTRONICA RUC: 10181727883 EB01-163 TAPIA MERINO GLADYS PATRICIA JR. LOS RUBIES 383 URB. SANTA INES TRUJILLO - TRUJILLO - LA LIBERTAD Fecha de Vencimiento Fecha de Emisión : 17/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Observación : S</t>
+        </is>
+      </c>
       <c r="O22" s="5" t="inlineStr"/>
       <c r="P22" s="5" t="inlineStr"/>
       <c r="Q22" s="5" t="inlineStr"/>
@@ -2964,41 +3730,57 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>110</v>
+        <v>70</v>
       </c>
       <c r="D23" t="n">
-        <v>110</v>
+        <v>70</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>factura_electronica</t>
+          <t>boleta_venta</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>20601709016</t>
+          <t>10181727883</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>INVERSIONES CASA BLANCA A &amp; A S.A.C.</t>
+          <t>TAPIA MERINO GLADYS PATRICIA</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>F002-2258</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
+          <t>EB01-164</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>109.00</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
       <c r="M23" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>wa, Blanca En u?'¡ií¿ wean? &lt; euenie fowtaueann . INVERSIONES CASA BLANCA A &amp; ak RM. LA GENERAL NRO. SIN SEC, CAMPIÑA DE MOC) 20601709016 FACTURA belles Fecne: — 220V2008 — Hera, 14022 RUE - 2 30708007 - PROGRAMA EDUCACIÓN BASICA Razón Social Pana “ CA m…amaa¿ .</t>
+          <t>BOLETA DE VENTA ELECTRONICA RUC: 10181727883 EB01-164 TAPIA MERINO GLADYS PATRICIA JR. LOS RUBIES 383 URB. SANTA INES TRUJILLO - TRUJILLO - LA LIBERTAD Fecha de Vencimiento Fecha de Emisión : 17/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Observación : S</t>
         </is>
       </c>
       <c r="O23" s="5" t="inlineStr"/>
@@ -3019,10 +3801,10 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>114</v>
+        <v>74</v>
       </c>
       <c r="D24" t="n">
-        <v>114</v>
+        <v>74</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -3031,41 +3813,29 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>20380795907</t>
+          <t>20613429388</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>INVERSIONES &amp; SERVICIOS MULTIPLES COQUITO S.A.C.</t>
+          <t>RAFO ALFARO CAFE S.A.C.</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>FA01-7588</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>2026-03-23</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>35.29</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
+          <t>F001-543</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>Av. America Sur 2763 Tr N°: FA01-0000007588 Fecha: 23/03/26 10:47 AM CAL.DEL COMERCIO NRO. 193 RES. LAS TC RUC: 20380795907 01 LOMO AL JUGO | ~ 39,00 SubTotal S/ IGV.10.50% S/ICBPERS/ Total S/ 35.29 3.71 0.00 39.00 Medio Pago: Efectivo Forma de Pago: CONTADO</t>
+          <t>16134 &lt;1 LOTE 8 URB SAN ey II ET s eet) M mta¿ — aE E 90 eo 1700 R ',frasnntaainn arte del Comprobant th e Electro) eS \Gracias Par ei preferencial h Sunwnro eRestaurant - 9764 77688</t>
         </is>
       </c>
       <c r="O24" s="5" t="inlineStr"/>
@@ -3086,10 +3856,10 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>118</v>
+        <v>78</v>
       </c>
       <c r="D25" t="n">
-        <v>118</v>
+        <v>78</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -3098,29 +3868,37 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>20202961518</t>
+          <t>10181685510</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>INVERSIONES FISA S.A.</t>
+          <t>JULCA ULLOA RONALD ALBERTO</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>F219-11456</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr"/>
+          <t>FF01-0002139</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
       <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>¡ .....u¡:¿¡ux f MA |</t>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002139 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 18/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
         </is>
       </c>
       <c r="O25" s="5" t="inlineStr"/>
@@ -3141,57 +3919,49 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>122</v>
+        <v>82</v>
       </c>
       <c r="D26" t="n">
-        <v>122</v>
+        <v>82</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>boleta_venta</t>
+          <t>factura_electronica</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>20380795907</t>
+          <t>10181685510</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>HERNANDEZ ALMENGOR SILVIA MARLENE</t>
+          <t>JULCA ULLOA RONALD ALBERTO</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>EB01-1390</t>
+          <t>FF01-0002141</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>70.00</t>
-        </is>
-      </c>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
           <t>PEN</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>6.65</t>
-        </is>
-      </c>
+      <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LA ESQUINA DEL ESTUDIANTE HERNANDEZ ALMENGOR SILVIA MARLENE BOLETAR%ECY,IE¿:;;OE,II;EÍIRONICA MZA. G INT. 2 PI LOTE. 1 URB. INGENIERIA E'Bº1 1390 TRUJILLO - TRUJILLO - LA LIBERTAD - Fecha de Vencimiento Fecha de Emisión : 23/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de </t>
+          <t xml:space="preserve">RUC 10181685510 RESTAURANTE EL AMARAL RESTAURANT DE: JULCA ULLOA RONALD ALBERTO FACTURA El Amaral PRINCIPAL » PSJ. EMANUEL KANT #188 URB. LA ELECTRONICA NORIA FFO1-0002141 DOCUMENTO “ RUC 20380795907 FECHA EMISIÓN 18/03/2026 CLIENTE PROGRAMA EDUCACION BASICA PARA TODOS FECHA VENCIMIENTO - DIRECCIÓN </t>
         </is>
       </c>
       <c r="O26" s="5" t="inlineStr"/>
@@ -3212,10 +3982,10 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>126</v>
+        <v>86</v>
       </c>
       <c r="D27" t="n">
-        <v>126</v>
+        <v>86</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -3224,43 +3994,27 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>10427606037</t>
+          <t>20607776912</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>ALMANZA MALLEA EDWIN</t>
+          <t>QUE BONITA VECINDAD S.A.C.</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>E001-16</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>2026-03-09</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>80.00</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
+          <t>FW01-1136</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
-        <v>1</v>
-      </c>
-      <c r="N27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAXI ALMANZA ALMANZA MALLEA EDWIN FACTURA ELECTRONICA A.F. BELLA DURMIENTE PRIMERO MZA. Y LOTE. 11 ALT.AV. CANTO RUC: 10427606037 GRANDE CON AV. CANTO BELLO E001-16 SAN JUAN DE LURIGANCHO - LIMA - LIMA Fecha de Emisión : 09/03/2026 Forma de pago: Contado . PROGRAMA EDUCACION BASICA " PARA TODOS RUC </t>
-        </is>
-      </c>
+        <v>0.5</v>
+      </c>
+      <c r="N27" s="2" t="inlineStr"/>
       <c r="O27" s="5" t="inlineStr"/>
       <c r="P27" s="5" t="inlineStr"/>
       <c r="Q27" s="5" t="inlineStr"/>
@@ -3279,10 +4033,10 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>130</v>
+        <v>90</v>
       </c>
       <c r="D28" t="n">
-        <v>130</v>
+        <v>90</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -3291,39 +4045,27 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>10181382941</t>
+          <t>20609888769</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>BRITO CAMACHO LUMBER</t>
+          <t>SABORES DE TRADICION PERUANA E.I.R.L.</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>FA01-85</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>2026-03-09</t>
-        </is>
-      </c>
+          <t>FW01-759</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="N28" s="2" t="inlineStr">
-        <is>
-          <t>A) 10181382941 Acuario "s SUITE FACTURA ELECTRONICA HOSPEDAJE ACUARIO'S SUITE Dirección : CALLE PRIMAVERA S/N SEC.LA ENCALADA DEL GOLF LA LIBERTAD - TRUJILLO - VICTOR LARCO HERRERA FAO 1 -85 Teléfonos : 065221356 Pagina web : hospedajeacuarios.efactur.pe Razón Social : PROGRAMA EDUCACION BASICA PARA</t>
-        </is>
-      </c>
+        <v>0.5</v>
+      </c>
+      <c r="N28" s="2" t="inlineStr"/>
       <c r="O28" s="5" t="inlineStr"/>
       <c r="P28" s="5" t="inlineStr"/>
       <c r="Q28" s="5" t="inlineStr"/>
@@ -3342,10 +4084,10 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>134</v>
+        <v>94</v>
       </c>
       <c r="D29" t="n">
-        <v>134</v>
+        <v>94</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -3354,37 +4096,33 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>20131525193</t>
+          <t>20615160653</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA.</t>
+          <t>DAMCO CAFE S.A.C.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>E001-968</t>
+          <t>F001-1258</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
+      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
         <v>0.75</v>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>HOSPEDAJE EL PALACIO SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA. JR. GRAU 709 TRUJILLO - TRUJILLO - LA LIBERTAD FACTURA ELECTRONICA RUC: 20131525193 E001-968 Fecha de Emisión : 21/03/2026 Forma de pago: Contado Señor(es) . PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 . JR. GRAU 709 LA LIBERTAD</t>
+          <t>u Damasco DANCO ares a; fe 20615160653 JR FRANCISCO BIZARRO ae 478 INT. 101 La Lrbenad T Ifo = Trujillo Cel 61 Tr FACTURA DE VENTA ELECTRONICA F001- 00001258 20/03/2026 - 11.06 Usuario: CARLOS VILLACORTA, ‘Ubie 004 Forma de Pago: Contado PROGRAMA. NEDUCACION. BASICA PARA TODOS 2038079590 gt CAL. DEL</t>
         </is>
       </c>
       <c r="O29" s="5" t="inlineStr"/>
@@ -3405,10 +4143,10 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>138</v>
+        <v>98</v>
       </c>
       <c r="D30" t="n">
-        <v>138</v>
+        <v>98</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -3417,51 +4155,645 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>20131525193</t>
+          <t>20613176528</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA.</t>
+          <t>LA ESTAMPIDA DEL MALL S.A.C.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>E001-970</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>2026-03-23</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>180.00</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
+          <t>F002-2057</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
-        <v>1</v>
-      </c>
-      <c r="N30" s="2" t="inlineStr">
-        <is>
-          <t>HOSPEDAJE EL PALACIO SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA. JR. GRAU 709 TRUJILLO - TRUJILLO - LA LIBERTAD FACTURA ELECTRONICA RUC: 20131525193 E001-970 Fecha de Emisión : 23/03/2026 Forma de pago: Contado Señor(es) . PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 . JR. GRAU 709 LA LIBERTAD</t>
-        </is>
-      </c>
+        <v>0.5</v>
+      </c>
+      <c r="N30" s="2" t="inlineStr"/>
       <c r="O30" s="5" t="inlineStr"/>
       <c r="P30" s="5" t="inlineStr"/>
       <c r="Q30" s="5" t="inlineStr"/>
       <c r="R30" s="5" t="inlineStr"/>
       <c r="S30" s="5" t="inlineStr"/>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>102</v>
+      </c>
+      <c r="D31" t="n">
+        <v>102</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>20600593685</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>LUCHA PARTNERS S.A.C.</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>F018-26030</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N31" s="2" t="inlineStr"/>
+      <c r="O31" s="5" t="inlineStr"/>
+      <c r="P31" s="5" t="inlineStr"/>
+      <c r="Q31" s="5" t="inlineStr"/>
+      <c r="R31" s="5" t="inlineStr"/>
+      <c r="S31" s="5" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>106</v>
+      </c>
+      <c r="D32" t="n">
+        <v>106</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>20609888769</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>SABORES DE TRADICION PERUANA E.I.R.L.</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>FW01-763</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N32" s="2" t="inlineStr"/>
+      <c r="O32" s="5" t="inlineStr"/>
+      <c r="P32" s="5" t="inlineStr"/>
+      <c r="Q32" s="5" t="inlineStr"/>
+      <c r="R32" s="5" t="inlineStr"/>
+      <c r="S32" s="5" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>110</v>
+      </c>
+      <c r="D33" t="n">
+        <v>110</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>20601709016</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>INVERSIONES CASA BLANCA A &amp; A S.A.C.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>F002-2258</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>wa, Blanca En u?'¡ií¿ wean? &lt; euenie fowtaueann . INVERSIONES CASA BLANCA A &amp; ak RM. LA GENERAL NRO. SIN SEC, CAMPIÑA DE MOC) 20601709016 FACTURA belles Fecne: — 220V2008 — Hera, 14022 RUE - 2 30708007 - PROGRAMA EDUCACIÓN BASICA Razón Social Pana “ CA m…amaa¿ .</t>
+        </is>
+      </c>
+      <c r="O33" s="5" t="inlineStr"/>
+      <c r="P33" s="5" t="inlineStr"/>
+      <c r="Q33" s="5" t="inlineStr"/>
+      <c r="R33" s="5" t="inlineStr"/>
+      <c r="S33" s="5" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>114</v>
+      </c>
+      <c r="D34" t="n">
+        <v>114</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>20380795907</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>INVERSIONES &amp; SERVICIOS MULTIPLES COQUITO S.A.C.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>FA01-7588</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>35.29</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="n">
+        <v>1</v>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>Av. America Sur 2763 Tr N°: FA01-0000007588 Fecha: 23/03/26 10:47 AM CAL.DEL COMERCIO NRO. 193 RES. LAS TC RUC: 20380795907 01 LOMO AL JUGO | ~ 39,00 SubTotal S/ IGV.10.50% S/ICBPERS/ Total S/ 35.29 3.71 0.00 39.00 Medio Pago: Efectivo Forma de Pago: CONTADO</t>
+        </is>
+      </c>
+      <c r="O34" s="5" t="inlineStr"/>
+      <c r="P34" s="5" t="inlineStr"/>
+      <c r="Q34" s="5" t="inlineStr"/>
+      <c r="R34" s="5" t="inlineStr"/>
+      <c r="S34" s="5" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>118</v>
+      </c>
+      <c r="D35" t="n">
+        <v>118</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>20202961518</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>INVERSIONES FISA S.A.</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>F219-11456</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>¡ .....u¡:¿¡ux f MA |</t>
+        </is>
+      </c>
+      <c r="O35" s="5" t="inlineStr"/>
+      <c r="P35" s="5" t="inlineStr"/>
+      <c r="Q35" s="5" t="inlineStr"/>
+      <c r="R35" s="5" t="inlineStr"/>
+      <c r="S35" s="5" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>122</v>
+      </c>
+      <c r="D36" t="n">
+        <v>122</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>boleta_venta</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>20380795907</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>HERNANDEZ ALMENGOR SILVIA MARLENE</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>EB01-1390</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>70.00</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>6.65</t>
+        </is>
+      </c>
+      <c r="M36" t="n">
+        <v>1</v>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LA ESQUINA DEL ESTUDIANTE HERNANDEZ ALMENGOR SILVIA MARLENE BOLETAR%ECY,IE¿:;;OE,II;EÍIRONICA MZA. G INT. 2 PI LOTE. 1 URB. INGENIERIA E'Bº1 1390 TRUJILLO - TRUJILLO - LA LIBERTAD - Fecha de Vencimiento Fecha de Emisión : 23/03/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de </t>
+        </is>
+      </c>
+      <c r="O36" s="5" t="inlineStr"/>
+      <c r="P36" s="5" t="inlineStr"/>
+      <c r="Q36" s="5" t="inlineStr"/>
+      <c r="R36" s="5" t="inlineStr"/>
+      <c r="S36" s="5" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>126</v>
+      </c>
+      <c r="D37" t="n">
+        <v>126</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>10427606037</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>ALMANZA MALLEA EDWIN</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>E001-16</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>80.00</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="n">
+        <v>1</v>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAXI ALMANZA ALMANZA MALLEA EDWIN FACTURA ELECTRONICA A.F. BELLA DURMIENTE PRIMERO MZA. Y LOTE. 11 ALT.AV. CANTO RUC: 10427606037 GRANDE CON AV. CANTO BELLO E001-16 SAN JUAN DE LURIGANCHO - LIMA - LIMA Fecha de Emisión : 09/03/2026 Forma de pago: Contado . PROGRAMA EDUCACION BASICA " PARA TODOS RUC </t>
+        </is>
+      </c>
+      <c r="O37" s="5" t="inlineStr"/>
+      <c r="P37" s="5" t="inlineStr"/>
+      <c r="Q37" s="5" t="inlineStr"/>
+      <c r="R37" s="5" t="inlineStr"/>
+      <c r="S37" s="5" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>130</v>
+      </c>
+      <c r="D38" t="n">
+        <v>130</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>10181382941</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>BRITO CAMACHO LUMBER</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>FA01-85</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>A) 10181382941 Acuario "s SUITE FACTURA ELECTRONICA HOSPEDAJE ACUARIO'S SUITE Dirección : CALLE PRIMAVERA S/N SEC.LA ENCALADA DEL GOLF LA LIBERTAD - TRUJILLO - VICTOR LARCO HERRERA FAO 1 -85 Teléfonos : 065221356 Pagina web : hospedajeacuarios.efactur.pe Razón Social : PROGRAMA EDUCACION BASICA PARA</t>
+        </is>
+      </c>
+      <c r="O38" s="5" t="inlineStr"/>
+      <c r="P38" s="5" t="inlineStr"/>
+      <c r="Q38" s="5" t="inlineStr"/>
+      <c r="R38" s="5" t="inlineStr"/>
+      <c r="S38" s="5" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>134</v>
+      </c>
+      <c r="D39" t="n">
+        <v>134</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>20131525193</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA.</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>E001-968</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>HOSPEDAJE EL PALACIO SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA. JR. GRAU 709 TRUJILLO - TRUJILLO - LA LIBERTAD FACTURA ELECTRONICA RUC: 20131525193 E001-968 Fecha de Emisión : 21/03/2026 Forma de pago: Contado Señor(es) . PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 . JR. GRAU 709 LA LIBERTAD</t>
+        </is>
+      </c>
+      <c r="O39" s="5" t="inlineStr"/>
+      <c r="P39" s="5" t="inlineStr"/>
+      <c r="Q39" s="5" t="inlineStr"/>
+      <c r="R39" s="5" t="inlineStr"/>
+      <c r="S39" s="5" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0250235</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>138</v>
+      </c>
+      <c r="D40" t="n">
+        <v>138</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>20131525193</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA.</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>E001-970</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>180.00</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="n">
+        <v>1</v>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>HOSPEDAJE EL PALACIO SERV.TURIST.HOSTAL EL PALACIO S.R.LTDA. JR. GRAU 709 TRUJILLO - TRUJILLO - LA LIBERTAD FACTURA ELECTRONICA RUC: 20131525193 E001-970 Fecha de Emisión : 23/03/2026 Forma de pago: Contado Señor(es) . PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 . JR. GRAU 709 LA LIBERTAD</t>
+        </is>
+      </c>
+      <c r="O40" s="5" t="inlineStr"/>
+      <c r="P40" s="5" t="inlineStr"/>
+      <c r="Q40" s="5" t="inlineStr"/>
+      <c r="R40" s="5" t="inlineStr"/>
+      <c r="S40" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S30"/>
+  <autoFilter ref="A1:S40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: extraccion bi_gravado, op_exonerada, op_inafecta + IGV flexible
- Nueva funcion _bi_gravado con prioridad Valor Venta > Op. Gravada
  (sin leyenda $) > SUBTOTAL > Base Imponible
- Nueva funcion _grab_op para op_exonerada y op_inafecta linea por linea
  con filtro anti-leyenda ($, Sin impuestos)
- Regex monto_igv flexible: orden libre entre :, S/, paréntesis
- Campos bi_gravado, op_exonerada, op_inafecta propagados por modelo,
  consolidador, extractor, excel_export e ingest_expedientes
- Nuevas columnas de sistema en hoja comprobantes (preservan humanas)
- Validado en 3 expedientes: DIED-0344746 (32 comp), DIED-0250235 (29),
  DEBEDSAR-0103251 (10). 0 regresiones en ruc/razon/serie/fecha/monto_total
- Evidencia regenerada: validacion_expedientes.xlsx

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/piloto_ocr/metrics/validacion_expedientes.xlsx
+++ b/data/piloto_ocr/metrics/validacion_expedientes.xlsx
@@ -16,8 +16,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'documentos'!$A$1:$AG$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'expedientes'!$A$1:$I$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'errores'!$A$1:$AG$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'resolucion_ids'!$A$1:$I$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'comprobantes'!$A$1:$S$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'resolucion_ids'!$A$1:$I$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'comprobantes'!$A$1:$V$33</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -671,17 +671,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DEBEDSAR2026-INT-0103251</t>
+          <t>DIED2026-INT-0344746</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026020411112511103251AMIQUERONAHUICARLOS.pdf</t>
+          <t>20260330161326PV809VICTORCHAVEZHUANCAYOCHANCHAM.pdf</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>C:\Users\Hans\Proyectos\vision_rag\control_previo\procesados\DEBEDSAR2026-INT-0103251\source\2026020411112511103251AMIQUERONAHUICARLOS.pdf</t>
+          <t>C:\Users\Hans\Proyectos\vision_rag\DIED2026-INT-0344746_VIATICO_17_04_9.42am\20260330161326PV809VICTORCHAVEZHUANCAYOCHANCHAM.pdf</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -690,26 +690,21 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.706</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>991.70</t>
-        </is>
+        <v>0.783</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2000-02-25</t>
+          <t>2001-02-25</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>CARLOS FERNANDO AMIQUERO ÑAHUI</t>
+          <t>VICTOR MESIAS CHAVEZ ULLOA</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>00242</t>
+          <t>00809</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -719,7 +714,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sistema Integrado de Gestión Administrativa Módulo de Tesorería Versión 25.02.00.U1 UNIDAD EJECUTORA NRO. IDENTIFICACIÓN : : 026 PROGRAMA EDUCACION BASICA PARA TODOS - 026 000081 SOLICITUD DE VIATICOS Nº : 00233 Fecha: Hora: Página: 1 de 1 Centro de Costo: Solicitante: Motivo del Viaje: APLICACIÓN DE LA I FASE - PUA 2026; AMIQUERO ÑAHUI, CARLOS FERNANDO; DNI :42192880; DIRECCIÓN: URB. LOS MÉDANOS </t>
+          <t>Sistema Integrado de Gestión Administrativa Módulo de Tesorería Versión 25.02.01.U1 UNIDAD EJECUTORA NRO. IDENTIFICACIÓN : : 026 PROGRAMA EDUCACION BASICA PARA TODOS - 026 000081 00809 PLANILLA DE VIÁTICOS Nº Fecha: Hora: Página: 1 de 1 Datos del Comisionado: 17:43 26/03/2026 Nº Exp. SIAF: Nº Pedido: 751 Fecha: 26/03/2026 Sr(a): VICTOR MESIAS CHAVEZ ULLOA N° Cuenta:AHORROS-04-331-339097 Escala: ES</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -734,17 +729,17 @@
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
-          <t>SINAD-103251</t>
+          <t>SINAD-344746</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>103251</t>
+          <t>344746</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>4361</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -753,24 +748,20 @@
         </is>
       </c>
       <c r="W2" t="n">
-        <v>0.85</v>
+        <v>0.82</v>
       </c>
       <c r="X2" t="n">
-        <v>0.85</v>
+        <v>0.901</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.889</v>
+        <v>0.96</v>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>siaf:score_max=8.0&lt;umbral_min=10.0</t>
-        </is>
-      </c>
+      <c r="AA2" t="inlineStr"/>
       <c r="AB2" s="5" t="n"/>
       <c r="AC2" s="5" t="n"/>
       <c r="AD2" s="5" t="n"/>
@@ -781,80 +772,83 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DEBEDSAR2026-INT-0103251</t>
+          <t>DIED2026-INT-0344746</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026040910538RIDECARLOSAMIQUERO.pdf</t>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>C:\Users\Hans\Proyectos\vision_rag\control_previo\procesados\DEBEDSAR2026-INT-0103251\source\2026040910538RIDECARLOSAMIQUERO.pdf</t>
+          <t>C:\Users\Hans\Proyectos\vision_rag\DIED2026-INT-0344746_VIATICO_17_04_9.42am\20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>otros</t>
+          <t>rendicion</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.889</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>138.70</t>
-        </is>
+        <v>0.49</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>20380795907</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>900-4-2026</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>desconocido</t>
+          <t>viaticos</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>DIA MES UE.026 (0081) PROGRAMA EDUCACION BASICA PARA TODOS - MINEDU RUC N°: 20380795907 AMIQUERO ÑAHUI CARLOS FERNANDO DEVOLUCIÓN DE VIÁTICOS 232121 TRANSPORTE NACIONAL 232122 VIATICOS NACIONAL 2327999 OTROS RELACIONADOS A ORGANIZACIÓN DE EVENTOS 155149 REPARACION CIVIL 23271498 OTROS SERVICIOS TECNICOS Y PROFESIONALES 152211 SANCIONES ADMINISTRATIVAS 1339199 OTROS SERVICIOS DE ADMINISTRACION Y RE</t>
+          <t>Sistema Integrado de Gestión Fecha : 14/04/2026 Modulo de Tesoreria Hora : 15:02 Version 22.04.00 Pagina : 1 de2 ANEXO N°3 RENDICION DE CUENTAS POR COMISION DE SERVICIOS UNIDAD EJECUTORA =: 026 PROGRAMA EDUCACION BASICA PARA TODOS - 026 NRO. IDENTIFICACIÓN : 000081 Datos del Sr(a): CHAVEZ ULLOA VICTOR MESIAS N° Planilla: 00809 N° Exp SIAF: 00004361 N° Comprobante 2605144 Motivo de APLICACION DE IN</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
+          <t>bajo_confianza</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>override_consolidado_rendicion: top_regex=factura(45) pero filename+encabezado indican rendicion(24)</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>firmas_anexo3</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>OBSERVADO</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>nombre_ilegible:jefe_unidad:anchor=sin_anchor; rol_no_detectado:vb_coordinador</t>
+        </is>
+      </c>
+      <c r="R3" t="n">
+        <v>0.35</v>
+      </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>SINAD-103251</t>
+          <t>SINAD-344746</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>103251</t>
+          <t>344746</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>4361</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -863,24 +857,20 @@
         </is>
       </c>
       <c r="W3" t="n">
-        <v>0.85</v>
+        <v>0.82</v>
       </c>
       <c r="X3" t="n">
-        <v>0.85</v>
+        <v>0.901</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.889</v>
+        <v>0.96</v>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>siaf:score_max=8.0&lt;umbral_min=10.0</t>
-        </is>
-      </c>
+      <c r="AA3" t="inlineStr"/>
       <c r="AB3" s="5" t="n"/>
       <c r="AC3" s="5" t="n"/>
       <c r="AD3" s="5" t="n"/>
@@ -896,25 +886,40 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
+          <t>2026020411112511103251AMIQUERONAHUICARLOS.pdf</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>C:\Users\Hans\Proyectos\vision_rag\control_previo\procesados\DEBEDSAR2026-INT-0103251\source\202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
+          <t>C:\Users\Hans\Proyectos\vision_rag\control_previo\procesados\DEBEDSAR2026-INT-0103251\source\2026020411112511103251AMIQUERONAHUICARLOS.pdf</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>rendicion</t>
+          <t>solicitud</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.481</v>
+        <v>0.706</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>991.70</t>
+        </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2000-02-25</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>CARLOS FERNANDO AMIQUERO ÑAHUI</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>00242</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -924,36 +929,13 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Sistema Integrado de Gestión Fecha : 06/04/2026 Módulo de Tesorería Hora : 17:37 Version 22.04.00 Pagina : 1 det ANEXO N*3 RENDICION DE CUENTAS POR COMISION DE SERVICIOS UNIDAD EJECUTORA : 026 PROGRAMA EDUCACION BASICA PARA TODOS - 026 NRO. IDENTIFICACIÓN : 000081 Datos del Sr(a): AMIQUERO ÑAHUI CARLOS FERNANDO N° Planilla: 00242 N° Exp SIAF: 00001792 N° Comprobante 2601620 Motivo de APLICACION DE</t>
+          <t xml:space="preserve">Sistema Integrado de Gestión Administrativa Módulo de Tesorería Versión 25.02.00.U1 UNIDAD EJECUTORA NRO. IDENTIFICACIÓN : : 026 PROGRAMA EDUCACION BASICA PARA TODOS - 026 000081 SOLICITUD DE VIATICOS Nº : 00233 Fecha: Hora: Página: 1 de 1 Centro de Costo: Solicitante: Motivo del Viaje: APLICACIÓN DE LA I FASE - PUA 2026; AMIQUERO ÑAHUI, CARLOS FERNANDO; DNI :42192880; DIRECCIÓN: URB. LOS MÉDANOS </t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>bajo_confianza</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>override_consolidado_rendicion: top_regex=factura(33) pero filename+encabezado indican rendicion(13)</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>firmas_anexo3</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>OBSERVADO</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>nombre_ilegible:jefe_unidad:anchor=sin_anchor; rol_no_detectado:vb_coordinador</t>
-        </is>
-      </c>
-      <c r="R4" t="n">
-        <v>0.35</v>
+          <t>ok</t>
+        </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -1004,45 +986,55 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0250235</t>
+          <t>DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf</t>
+          <t>2026040910538RIDECARLOSAMIQUERO.pdf</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>C:\Users\Hans\Proyectos\vision_rag\control_previo\procesados\DIED2026-INT-0250235\source\20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf</t>
+          <t>C:\Users\Hans\Proyectos\vision_rag\control_previo\procesados\DEBEDSAR2026-INT-0103251\source\2026040910538RIDECARLOSAMIQUERO.pdf</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>solicitud</t>
+          <t>otros</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.783</v>
+        <v>0.889</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>138.70</t>
+        </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>LILIANA CHAVEZ TERRONES</t>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>20380795907</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>900-4-2026</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>viaticos</t>
+          <t>desconocido</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sistema Integrado de Gestión Administrativa Fecha: 3/03/2026 Módulo de Tesorería Hora: 15:01 Versión 25.02.01.U1 , ágina: e PLANILLA DE VIÁTICOS N* Pagina: te UNIDAD EJECUTORA : 026 PROGRAMA EDUCACION BASICA PARA TODOS - 026 NRO. IDENTIFICACIÓN : 000081 Datos del Comisionado: Fecha: 03/03/2026 N° Exp. SIAF: N° Pedido: 572 Sr(a): LILIANA CHAVEZ TERRONES Escala: ESCALA-2 FUNCIONARIOS Y EMPLEADOS N° </t>
+          <t>DIA MES UE.026 (0081) PROGRAMA EDUCACION BASICA PARA TODOS - MINEDU RUC N°: 20380795907 AMIQUERO ÑAHUI CARLOS FERNANDO DEVOLUCIÓN DE VIÁTICOS 232121 TRANSPORTE NACIONAL 232122 VIATICOS NACIONAL 2327999 OTROS RELACIONADOS A ORGANIZACIÓN DE EVENTOS 155149 REPARACION CIVIL 23271498 OTROS SERVICIOS TECNICOS Y PROFESIONALES 152211 SANCIONES ADMINISTRATIVAS 1339199 OTROS SERVICIOS DE ADMINISTRACION Y RE</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -1052,17 +1044,17 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>SINAD-250235</t>
+          <t>SINAD-103251</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>250235</t>
+          <t>103251</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>2603426</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -1071,22 +1063,22 @@
         </is>
       </c>
       <c r="W5" t="n">
-        <v>0.838</v>
+        <v>0.85</v>
       </c>
       <c r="X5" t="n">
-        <v>0.912</v>
+        <v>0.85</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.485</v>
+        <v>0.889</v>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>siaf:conflicto: top=SIAF-2603426(16.0) vs segundo=SIAF-3205(16.0)</t>
+          <t>siaf:score_max=8.0&lt;umbral_min=10.0</t>
         </is>
       </c>
       <c r="AB5" s="5" t="n"/>
@@ -1099,17 +1091,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0250235</t>
+          <t>DEBEDSAR2026-INT-0103251</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>C:\Users\Hans\Proyectos\vision_rag\control_previo\procesados\DIED2026-INT-0250235\source\2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
+          <t>C:\Users\Hans\Proyectos\vision_rag\control_previo\procesados\DEBEDSAR2026-INT-0103251\source\202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1118,11 +1110,11 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.49</v>
+        <v>0.481</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1132,7 +1124,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>ANEXO N°3 Fecha : Hora : Página : 1 de 2 09/04/2026 13:01 Sistema Integrado de Gestión Módulo de Tesorería Versión 22.04.00 026 PROGRAMA EDUCACION BASICA PARA TODOS - 026 000081 Datos del CHAVEZ TERRONES LILIANA Sr(a): N° Planilla: Motivo de Salida: 00617 N° Exp SIAF: 2603426 N° Comprobante 09/03/2026 Regreso: N° Días/Horas: 11d 23h APLICACION DE INSTRUMENTOS PARA RECOJO DE INFORMACION A CARGO DEL</t>
+          <t>Sistema Integrado de Gestión Fecha : 06/04/2026 Módulo de Tesorería Hora : 17:37 Version 22.04.00 Pagina : 1 det ANEXO N*3 RENDICION DE CUENTAS POR COMISION DE SERVICIOS UNIDAD EJECUTORA : 026 PROGRAMA EDUCACION BASICA PARA TODOS - 026 NRO. IDENTIFICACIÓN : 000081 Datos del Sr(a): AMIQUERO ÑAHUI CARLOS FERNANDO N° Planilla: 00242 N° Exp SIAF: 00001792 N° Comprobante 2601620 Motivo de APLICACION DE</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1142,7 +1134,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>override_consolidado_rendicion: top_regex=factura(45) pero filename+encabezado indican rendicion(24)</t>
+          <t>override_consolidado_rendicion: top_regex=factura(33) pero filename+encabezado indican rendicion(13)</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -1152,30 +1144,30 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>INSUFICIENTE_EVIDENCIA</t>
+          <t>OBSERVADO</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>nombre_ilegible:comisionado:anchor=dni_sin_nombre_adyacente; nombre_ilegible:jefe_unidad:anchor=sin_anchor; rol_no_detectado:vb_coordinador</t>
+          <t>nombre_ilegible:jefe_unidad:anchor=sin_anchor; rol_no_detectado:vb_coordinador</t>
         </is>
       </c>
       <c r="R6" t="n">
-        <v>0.1</v>
+        <v>0.35</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>SINAD-250235</t>
+          <t>SINAD-103251</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>250235</t>
+          <t>103251</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>2603426</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1184,22 +1176,22 @@
         </is>
       </c>
       <c r="W6" t="n">
-        <v>0.838</v>
+        <v>0.85</v>
       </c>
       <c r="X6" t="n">
-        <v>0.912</v>
+        <v>0.85</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.485</v>
+        <v>0.889</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>siaf:conflicto: top=SIAF-2603426(16.0) vs segundo=SIAF-3205(16.0)</t>
+          <t>siaf:score_max=8.0&lt;umbral_min=10.0</t>
         </is>
       </c>
       <c r="AB6" s="5" t="n"/>
@@ -1212,17 +1204,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0344746</t>
+          <t>DIED2026-INT-0250235</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>20260330161326PV809VICTORCHAVEZHUANCAYOCHANCHAM.pdf</t>
+          <t>20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>C:\Users\Hans\Proyectos\vision_rag\DIED2026-INT-0344746_VIATICO_17_04_9.42am\20260330161326PV809VICTORCHAVEZHUANCAYOCHANCHAM.pdf</t>
+          <t>C:\Users\Hans\Proyectos\vision_rag\control_previo\procesados\DIED2026-INT-0250235\source\20260306953PV617LILIANACHAVEZTRUJILLOJULCAN.pdf</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1235,17 +1227,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2001-02-25</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>VICTOR MESIAS CHAVEZ ULLOA</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>00809</t>
+          <t>LILIANA CHAVEZ TERRONES</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1255,7 +1242,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Sistema Integrado de Gestión Administrativa Módulo de Tesorería Versión 25.02.01.U1 UNIDAD EJECUTORA NRO. IDENTIFICACIÓN : : 026 PROGRAMA EDUCACION BASICA PARA TODOS - 026 000081 00809 PLANILLA DE VIÁTICOS Nº Fecha: Hora: Página: 1 de 1 Datos del Comisionado: 17:43 26/03/2026 Nº Exp. SIAF: Nº Pedido: 751 Fecha: 26/03/2026 Sr(a): VICTOR MESIAS CHAVEZ ULLOA N° Cuenta:AHORROS-04-331-339097 Escala: ES</t>
+          <t xml:space="preserve">Sistema Integrado de Gestión Administrativa Fecha: 3/03/2026 Módulo de Tesorería Hora: 15:01 Versión 25.02.01.U1 , ágina: e PLANILLA DE VIÁTICOS N* Pagina: te UNIDAD EJECUTORA : 026 PROGRAMA EDUCACION BASICA PARA TODOS - 026 NRO. IDENTIFICACIÓN : 000081 Datos del Comisionado: Fecha: 03/03/2026 N° Exp. SIAF: N° Pedido: 572 Sr(a): LILIANA CHAVEZ TERRONES Escala: ESCALA-2 FUNCIONARIOS Y EMPLEADOS N° </t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1265,17 +1252,17 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>SINAD-344746</t>
+          <t>SINAD-250235</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>344746</t>
+          <t>250235</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>4361</t>
+          <t>2603426</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1284,17 +1271,22 @@
         </is>
       </c>
       <c r="W7" t="n">
-        <v>0.82</v>
+        <v>0.838</v>
       </c>
       <c r="X7" t="n">
-        <v>0.901</v>
+        <v>0.912</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.96</v>
+        <v>0.485</v>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>siaf:conflicto: top=SIAF-2603426(16.0) vs segundo=SIAF-3205(16.0)</t>
         </is>
       </c>
       <c r="AB7" s="5" t="n"/>
@@ -1307,17 +1299,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DIED2026-INT-0344746</t>
+          <t>DIED2026-INT-0250235</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+          <t>2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>C:\Users\Hans\Proyectos\vision_rag\DIED2026-INT-0344746_VIATICO_17_04_9.42am\20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+          <t>C:\Users\Hans\Proyectos\vision_rag\control_previo\procesados\DIED2026-INT-0250235\source\2026041320235RENDICLILIANACHAVEZSINAD250235.pdf</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1330,7 +1322,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1340,7 +1332,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Sistema Integrado de Gestión Fecha : 14/04/2026 Modulo de Tesoreria Hora : 15:02 Version 22.04.00 Pagina : 1 de2 ANEXO N°3 RENDICION DE CUENTAS POR COMISION DE SERVICIOS UNIDAD EJECUTORA =: 026 PROGRAMA EDUCACION BASICA PARA TODOS - 026 NRO. IDENTIFICACIÓN : 000081 Datos del Sr(a): CHAVEZ ULLOA VICTOR MESIAS N° Planilla: 00809 N° Exp SIAF: 00004361 N° Comprobante 2605144 Motivo de APLICACION DE IN</t>
+          <t>ANEXO N°3 Fecha : Hora : Página : 1 de 2 09/04/2026 13:01 Sistema Integrado de Gestión Módulo de Tesorería Versión 22.04.00 026 PROGRAMA EDUCACION BASICA PARA TODOS - 026 000081 Datos del CHAVEZ TERRONES LILIANA Sr(a): N° Planilla: Motivo de Salida: 00617 N° Exp SIAF: 2603426 N° Comprobante 09/03/2026 Regreso: N° Días/Horas: 11d 23h APLICACION DE INSTRUMENTOS PARA RECOJO DE INFORMACION A CARGO DEL</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1360,30 +1352,30 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>OBSERVADO</t>
+          <t>INSUFICIENTE_EVIDENCIA</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>nombre_ilegible:jefe_unidad:anchor=sin_anchor; rol_no_detectado:vb_coordinador</t>
+          <t>nombre_ilegible:comisionado:anchor=dni_sin_nombre_adyacente; nombre_ilegible:jefe_unidad:anchor=sin_anchor; rol_no_detectado:vb_coordinador</t>
         </is>
       </c>
       <c r="R8" t="n">
-        <v>0.35</v>
+        <v>0.1</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>SINAD-344746</t>
+          <t>SINAD-250235</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>344746</t>
+          <t>250235</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>4361</t>
+          <t>2603426</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1392,17 +1384,22 @@
         </is>
       </c>
       <c r="W8" t="n">
-        <v>0.82</v>
+        <v>0.838</v>
       </c>
       <c r="X8" t="n">
-        <v>0.901</v>
+        <v>0.912</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.96</v>
+        <v>0.485</v>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>siaf:conflicto: top=SIAF-2603426(16.0) vs segundo=SIAF-3205(16.0)</t>
         </is>
       </c>
       <c r="AB8" s="5" t="n"/>
@@ -1488,24 +1485,24 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DEBEDSAR2026-INT-0103251</t>
+          <t>DIED2026-INT-0344746</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>C:\Users\Hans\Proyectos\vision_rag\control_previo\procesados\DEBEDSAR2026-INT-0103251\source</t>
+          <t>C:\Users\Hans\Proyectos\vision_rag\DIED2026-INT-0344746_VIATICO_17_04_9.42am</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>C:\Users\Hans\Proyectos\vision_rag\control_previo\procesados\DEBEDSAR2026-INT-0103251</t>
+          <t>C:\Users\Hans\Proyectos\vision_rag\control_previo\procesados\DIED2026-INT-0344746</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
         <v>1</v>
@@ -1515,12 +1512,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>otros, rendicion, solicitud</t>
+          <t>rendicion, solicitud</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-04-17T12:20:23-0500</t>
+          <t>2026-04-17T23:30:29-0500</t>
         </is>
       </c>
     </row>
@@ -1753,7 +1750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1817,12 +1814,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DEBEDSAR2026-INT-0103251</t>
+          <t>DIED2026-INT-0344746</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SINAD-103251</t>
+          <t>SINAD-344746</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1831,10 +1828,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E2" t="n">
-        <v>91</v>
+        <v>146</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1848,19 +1845,19 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>BAJA_CONFIANZA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026020411112511103251AMIQUERONAHUICARLOS.pdf:p1; 2026020411112511103251AMIQUERONAHUICARLOS.pdf:p2; 202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf:p1; 202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf:p2; 202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf:p7</t>
+          <t>20260330161326PV809VICTORCHAVEZHUANCAYOCHANCHAM.pdf:p1; 20260330161326PV809VICTORCHAVEZHUANCAYOCHANCHAM.pdf:p2; 20260330161326PV809VICTORCHAVEZHUANCAYOCHANCHAM.pdf:p3; 20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf:p1; 20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf:p2</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DEBEDSAR2026-INT-0103251</t>
+          <t>DIED2026-INT-0344746</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1877,7 +1874,7 @@
         <v>7</v>
       </c>
       <c r="E3" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1891,36 +1888,36 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>BAJA_CONFIANZA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026020411112511103251AMIQUERONAHUICARLOS.pdf:p1; 2026020411112511103251AMIQUERONAHUICARLOS.pdf:p1; 2026020411112511103251AMIQUERONAHUICARLOS.pdf:p1; 2026040910538RIDECARLOSAMIQUERO.pdf:p1; 202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf:p1</t>
+          <t>20260330161326PV809VICTORCHAVEZHUANCAYOCHANCHAM.pdf:p1; 20260330161326PV809VICTORCHAVEZHUANCAYOCHANCHAM.pdf:p1; 20260330161326PV809VICTORCHAVEZHUANCAYOCHANCHAM.pdf:p1; 20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf:p9; 20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf:p1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DEBEDSAR2026-INT-0103251</t>
+          <t>DIED2026-INT-0344746</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SINAD-116260</t>
+          <t>SIAF-4361</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>sinad</t>
+          <t>siaf</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1934,36 +1931,36 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>BAJA_CONFIANZA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026020411112511103251AMIQUERONAHUICARLOS.pdf:p7</t>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf:p1; 20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf:p2; 20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf:p9</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DEBEDSAR2026-INT-0103251</t>
+          <t>DIED2026-INT-0344746</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SIAF-1792</t>
+          <t>EXP-DIED-2026-344746</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>siaf</t>
+          <t>exp</t>
         </is>
       </c>
       <c r="D5" t="n">
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1977,36 +1974,36 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>BAJA_CONFIANZA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf:p1</t>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf:p9</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DEBEDSAR2026-INT-0103251</t>
+          <t>DIED2026-INT-0344746</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PLANILLA-00242</t>
+          <t>SINAD-112591</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>planilla</t>
+          <t>sinad</t>
         </is>
       </c>
       <c r="D6" t="n">
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -2020,60 +2017,103 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>BAJA_CONFIANZA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf:p1</t>
+          <t>20260330161326PV809VICTORCHAVEZHUANCAYOCHANCHAM.pdf:p9</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DEBEDSAR2026-INT-0103251</t>
+          <t>DIED2026-INT-0344746</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PEDIDO-233</t>
+          <t>PLANILLA-00809</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>planilla</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>8</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf:p1; 20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf:p2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>PEDIDO-751</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>pedido</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F7" t="inlineStr">
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>7</v>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>BAJA_CONFIANZA</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>2026020411112511103251AMIQUERONAHUICARLOS.pdf:p2</t>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>20260330161326PV809VICTORCHAVEZHUANCAYOCHANCHAM.pdf:p1; 20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf:p3</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I7"/>
+  <autoFilter ref="A1:I8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2084,7 +2124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S11"/>
+  <dimension ref="A1:V33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2099,13 +2139,16 @@
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="8" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="28" customWidth="1" min="17" max="17"/>
-    <col width="40" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="28" customWidth="1" min="20" max="20"/>
+    <col width="40" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2171,35 +2214,50 @@
       </c>
       <c r="M1" s="4" t="inlineStr">
         <is>
+          <t>bi_gravado</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>op_exonerada</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>op_inafecta</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
           <t>confianza</t>
         </is>
       </c>
-      <c r="N1" s="4" t="inlineStr">
+      <c r="Q1" s="4" t="inlineStr">
         <is>
           <t>texto_resumen</t>
         </is>
       </c>
-      <c r="O1" s="4" t="inlineStr">
+      <c r="R1" s="4" t="inlineStr">
         <is>
           <t>monto_correcto</t>
         </is>
       </c>
-      <c r="P1" s="4" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
         <is>
           <t>ruc_correcto</t>
         </is>
       </c>
-      <c r="Q1" s="4" t="inlineStr">
+      <c r="T1" s="4" t="inlineStr">
         <is>
           <t>proveedor_correcto</t>
         </is>
       </c>
-      <c r="R1" s="4" t="inlineStr">
+      <c r="U1" s="4" t="inlineStr">
         <is>
           <t>observaciones</t>
         </is>
       </c>
-      <c r="S1" s="4" t="inlineStr">
+      <c r="V1" s="4" t="inlineStr">
         <is>
           <t>validacion_final</t>
         </is>
@@ -2208,19 +2266,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DEBEDSAR2026-INT-0103251</t>
+          <t>DIED2026-INT-0344746</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="D2" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -2229,27 +2287,27 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>20515659324</t>
+          <t>20380795907</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>TURISMO INTERNACIONAL PALOMINO S.A.C.</t>
+          <t>ANFLOR SERVICE S.A.C.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>F235-0040130</t>
+          <t>F001-00000737</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>80.00</t>
+          <t>90.00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -2258,36 +2316,43 @@
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
-      <c r="M2" t="n">
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>90.00</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="n">
         <v>1</v>
       </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>TURISMO INTERNACIONAL PALOMINO S.A.C. AV. NICOLAS ARRIOLA NRO. 910 URB. SANTA CATALINA - LI RUC; 20515659324 FACTURA ELECTRONICA F235-0040130 RUC; 20380795907 RAZON SOC PROGRAMA EDUCACION BASICA PARA TODOS E TOTAL 1 SERVICIO DE TRANSPORTE EN LA 80.00 RUTA: ICA PUQUIO ASIENTO: 39 PASAJERO: CARLOS FER</t>
-        </is>
-      </c>
-      <c r="O2" s="5" t="inlineStr"/>
-      <c r="P2" s="5" t="inlineStr"/>
-      <c r="Q2" s="5" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R.U.C. N° 20613343700 ANFLOR SERVICE S.A.C. JR. ALFONSO UGARTE MZ. 2G LT. 24 P.J. JOSE OLAYA FACTURA ELECTRONICA CALLAO PROV. CONST. DEL CALLAO PROV. CONST. DEL CALLAO A Oo i= mee F001-00000737 RAZÓN SOCIAL: PROGRAMA EDUCACION BASICA PARA TODOS RUC: 20380795907 DIRECCION: CAL. DEL COMERCIO NRO. 193 </t>
+        </is>
+      </c>
       <c r="R2" s="5" t="inlineStr"/>
       <c r="S2" s="5" t="inlineStr"/>
+      <c r="T2" s="5" t="inlineStr"/>
+      <c r="U2" s="5" t="inlineStr"/>
+      <c r="V2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DEBEDSAR2026-INT-0103251</t>
+          <t>DIED2026-INT-0344746</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="D3" t="n">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -2296,69 +2361,72 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>10288513673</t>
+          <t>10425467188</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>RESTAURANT HATUN WASI</t>
+          <t>ROJAS CHUQUILLANQUI JESUS MAEL</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>F001-00001706</t>
+          <t>E001-2601</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>46.00</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
+          <t>60.00</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>7.02</t>
-        </is>
-      </c>
-      <c r="M3" t="n">
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>60.00</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="n">
         <v>1</v>
       </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>Representación impresa de la FACTURA ELECTRÓNICA. Esta puede ser consultada en https://hatunwasi.cpesimple.online/buscar RESTAURANT HATUN WASI De: PACHECO COYLLO GLORIA YOLANDA JR. LEONCIO PRADO N° 295 , PUQUIO , LUCANAS - AYACUCHO D. Comercial: JR. LEONCIO PRADO N° 295 935 737 974 yolandaccoyllopac</t>
-        </is>
-      </c>
-      <c r="O3" s="5" t="inlineStr"/>
-      <c r="P3" s="5" t="inlineStr"/>
-      <c r="Q3" s="5" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>ROJAS CHUQUILLANQUI JESUS MAEL FACTU RA ELECTRONICA ROJAS CHUQUILLANQUI JESUS MAEL . RUC:10425467188 JR. PUCATEA 904 C.P.M UNAS 2 CDR ANT D PLANTA D TRATAMIENT D SEDAM E001 -2601 HUANCAYO - HUANCAYO - JUNIN Formato de Pago’: Al Contado Fecha de Emisión :05/04/2026 Señor (es) ‘PROGRAMA EDUCACION BASI</t>
+        </is>
+      </c>
       <c r="R3" s="5" t="inlineStr"/>
       <c r="S3" s="5" t="inlineStr"/>
+      <c r="T3" s="5" t="inlineStr"/>
+      <c r="U3" s="5" t="inlineStr"/>
+      <c r="V3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DEBEDSAR2026-INT-0103251</t>
+          <t>DIED2026-INT-0344746</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="D4" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -2367,27 +2435,27 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>10288513673</t>
+          <t>20140249212</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>RESTAURANT HATUN WASI</t>
+          <t>RESTAURANTE OLIMPICO SAC</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>F001-00001707</t>
+          <t>F001-00056333</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>80.00</t>
+          <t>44.90</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -2395,41 +2463,44 @@
           <t>PEN</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>12.20</t>
-        </is>
-      </c>
-      <c r="M4" t="n">
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>40.63</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="n">
         <v>1</v>
       </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>Representación impresa de la FACTURA ELECTRÓNICA. Esta puede ser consultada en https://hatunwasi.cpesimple.online/buscar RESTAURANT HATUN WASI De: PACHECO COYLLO GLORIA YOLANDA JR. LEONCIO PRADO N° 295 , PUQUIO , LUCANAS - AYACUCHO D. Comercial: JR. LEONCIO PRADO N° 295 935 737 974 yolandaccoyllopac</t>
-        </is>
-      </c>
-      <c r="O4" s="5" t="inlineStr"/>
-      <c r="P4" s="5" t="inlineStr"/>
-      <c r="Q4" s="5" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>RESTAURANTE OLIMPICO RESTAURANTE OLIMPICO S.A.C. AV. GIRALDEZ NRO. 199 - HUANCAYO - JUNIN RUC 20140249212 FACTURA ELECTRONICA F001-00056333 CLIENTE: PROGRAMA EDUCACION BASICA PARA TODOS : 20380795907 DIRECCION: CAL. DEL COMERCIO NRO. 193 RES, LAS T URRES DE SAN BORJA FECHA DE EMISION: 05-04-2026 HOR</t>
+        </is>
+      </c>
       <c r="R4" s="5" t="inlineStr"/>
       <c r="S4" s="5" t="inlineStr"/>
+      <c r="T4" s="5" t="inlineStr"/>
+      <c r="U4" s="5" t="inlineStr"/>
+      <c r="V4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DEBEDSAR2026-INT-0103251</t>
+          <t>DIED2026-INT-0344746</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="D5" t="n">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -2438,27 +2509,27 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>10288513673</t>
+          <t>20607154521</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>RESTAURANT HATUN WASI</t>
+          <t>FT CHINA SOCIEDAD ANONIMA CERRADA</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>F001-00001711</t>
+          <t>F001-00014469</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>45.00</t>
+          <t>27.00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -2466,70 +2537,69 @@
           <t>PEN</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>6.86</t>
-        </is>
-      </c>
-      <c r="M5" t="n">
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="n">
         <v>1</v>
       </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>Representación impresa de la FACTURA ELECTRÓNICA. Esta puede ser consultada en https://hatunwasi.cpesimple.online/buscar RESTAURANT HATUN WASI De: PACHECO COYLLO GLORIA YOLANDA JR. LEONCIO PRADO N° 295 , PUQUIO , LUCANAS - AYACUCHO D. Comercial: JR. LEONCIO PRADO N° 295 935 737 974 yolandaccoyllopac</t>
-        </is>
-      </c>
-      <c r="O5" s="5" t="inlineStr"/>
-      <c r="P5" s="5" t="inlineStr"/>
-      <c r="Q5" s="5" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>CHIFA YUFU FT CHINA S.A.C 20607154521 AV. GIRALDEZ NRO. 208 HUANCAYO CERCADO JUNIN - HUANCAYO - HUANCAYO .................................................................... F001-00014469 05-04-2026 18:33:48 .................................................................... PARA TODOS RUC/DNI: 203</t>
+        </is>
+      </c>
       <c r="R5" s="5" t="inlineStr"/>
       <c r="S5" s="5" t="inlineStr"/>
+      <c r="T5" s="5" t="inlineStr"/>
+      <c r="U5" s="5" t="inlineStr"/>
+      <c r="V5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DEBEDSAR2026-INT-0103251</t>
+          <t>DIED2026-INT-0344746</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="D6" t="n">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>factura_electronica</t>
+          <t>boleta_venta</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>10288019482</t>
+          <t>10715562681</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>POLLOS A LA</t>
+          <t>SORIANO ACLARI DIANA</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>F003-2106</t>
+          <t>EB01-2294</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>50.00</t>
+          <t>60.00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -2539,68 +2609,79 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>4.55</t>
-        </is>
-      </c>
-      <c r="M6" t="n">
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
         <v>1</v>
       </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>POLLOS A LA BRASA RESTAURANTE EL “DORADO” De: CRUZ MURIEL DORIS R.U.C. : 10288019482 Ofrece: Pollos a La Brasa, Brosther, Salchipapas, Platos Extras, Menú Ejecutivo, Menú Económico Bebidas Calientes, Frías, Gaseosas, Licores, Vinos, Cervezas y Otros. HOSPEDAJE IMPERIAL: Habitaciones Confortables con</t>
-        </is>
-      </c>
-      <c r="O6" s="5" t="inlineStr"/>
-      <c r="P6" s="5" t="inlineStr"/>
-      <c r="Q6" s="5" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>BOLETA DE VENTA ELECTRONICA RUC: 10715562681 EB01-2294 SORIANO ACLARI DIANA AV. AV.HUAYTAPALLANA 1201 AL FRENTE DE UNA LOZA DEPORTIVA EL TAMBO - HUANCAYO - JUNIN Fecha de Vencimiento Fecha de Emisión : 06/04/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Obser</t>
+        </is>
+      </c>
       <c r="R6" s="5" t="inlineStr"/>
       <c r="S6" s="5" t="inlineStr"/>
+      <c r="T6" s="5" t="inlineStr"/>
+      <c r="U6" s="5" t="inlineStr"/>
+      <c r="V6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DEBEDSAR2026-INT-0103251</t>
+          <t>DIED2026-INT-0344746</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="D7" t="n">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>factura_electronica</t>
+          <t>boleta_venta</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>10288513673</t>
+          <t>10715562681</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>RESTAURANT HATUN WASI</t>
+          <t>SORIANO ACLARI DIANA</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>F001-00001712</t>
+          <t>EB01-2296</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>32.00</t>
+          <t>40.00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -2610,68 +2691,79 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>4.88</t>
-        </is>
-      </c>
-      <c r="M7" t="n">
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
         <v>1</v>
       </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>Representación impresa de la FACTURA ELECTRÓNICA. Esta puede ser consultada en https://hatunwasi.cpesimple.online/buscar RESTAURANT HATUN WASI De: PACHECO COYLLO GLORIA YOLANDA JR. LEONCIO PRADO N° 295 , PUQUIO , LUCANAS - AYACUCHO D. Comercial: JR. LEONCIO PRADO N° 295 935 737 974 yolandaccoyllopac</t>
-        </is>
-      </c>
-      <c r="O7" s="5" t="inlineStr"/>
-      <c r="P7" s="5" t="inlineStr"/>
-      <c r="Q7" s="5" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>BOLETA DE VENTA ELECTRONICA RUC: 10715562681 EB01-2296 SORIANO ACLARI DIANA AV. AV.HUAYTAPALLANA 1201 AL FRENTE DE UNA LOZA DEPORTIVA EL TAMBO - HUANCAYO - JUNIN Fecha de Vencimiento Fecha de Emisión : 06/04/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Obser</t>
+        </is>
+      </c>
       <c r="R7" s="5" t="inlineStr"/>
       <c r="S7" s="5" t="inlineStr"/>
+      <c r="T7" s="5" t="inlineStr"/>
+      <c r="U7" s="5" t="inlineStr"/>
+      <c r="V7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DEBEDSAR2026-INT-0103251</t>
+          <t>DIED2026-INT-0344746</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="D8" t="n">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>factura_electronica</t>
+          <t>boleta_venta</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>20615320561</t>
+          <t>10427147491</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>POLLOS A LA BRASA AMIGOS S.A.C.</t>
+          <t>HILARIO FLORES JORGE LUIS</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>E001-27</t>
+          <t>EB01-1416</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>35.00</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -2681,68 +2773,79 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>5.34</t>
-        </is>
-      </c>
-      <c r="M8" t="n">
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
         <v>1</v>
       </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">POLLOS &amp; PARRILLAS AMIGOS POLLOS A LA BRASA AMIGOS S.A.C. JR. SAISA KM. 223 A 1 CUADRA DE LA PANAMERICANA PUQUIO - LUCANAS - AYACUCHO FACTURA ELECTRONICA RUC: 20615320561 E001-27 Fecha de Emisión : 08/02/2026 Señor(es) : PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 Dirección del Cliente : </t>
-        </is>
-      </c>
-      <c r="O8" s="5" t="inlineStr"/>
-      <c r="P8" s="5" t="inlineStr"/>
-      <c r="Q8" s="5" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BOLETA DE VENTA ELECTRONICA HILARIO FLORES JORGE LUIS RUC: 10427147491 JR. PARAMONGA 121 ENTRE INTIHUATANA Y AV.CIRCUNVALACION EB01-1416 EL TAMBO - HUANCAYO - JUNIN - Fecha de Vencimiento Fecha de Emisión : 06/04/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES </t>
+        </is>
+      </c>
       <c r="R8" s="5" t="inlineStr"/>
       <c r="S8" s="5" t="inlineStr"/>
+      <c r="T8" s="5" t="inlineStr"/>
+      <c r="U8" s="5" t="inlineStr"/>
+      <c r="V8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DEBEDSAR2026-INT-0103251</t>
+          <t>DIED2026-INT-0344746</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="D9" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>factura_electronica</t>
+          <t>boleta_venta</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>20612666751</t>
+          <t>10715562681</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>HOTEL SUMAC SAMARI S.A.C.</t>
+          <t>SORIANO ACLARI DIANA</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>E001-478</t>
+          <t>EB01-2317</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>300.00</t>
+          <t>60.00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -2752,63 +2855,74 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>28.51</t>
-        </is>
-      </c>
-      <c r="M9" t="n">
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
         <v>1</v>
       </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FACTURA ELECTRONICA RUC: 20612666751 E001-478 Sub Total Ventas : S/ 271.49 Anticipos : S/ 0.00 Descuentos : S/ 0.00 Valor Venta : S/ 271.49 ISC : S/ 0.00 IGV : S/ 28.51 ICBPER : S/ 0.00 Otros Cargos : S/ 0.00 Otros Tributos : S/ 0.00 Monto de redondeo : S/ 0.00 Importe Total : S/ 300.00 HOTEL SUMAC </t>
-        </is>
-      </c>
-      <c r="O9" s="5" t="inlineStr"/>
-      <c r="P9" s="5" t="inlineStr"/>
-      <c r="Q9" s="5" t="inlineStr"/>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>BOLETA DE VENTA ELECTRONICA RUC: 10715562681 EB01-2317 SORIANO ACLARI DIANA AV. AV.HUAYTAPALLANA 1201 AL FRENTE DE UNA LOZA DEPORTIVA EL TAMBO - HUANCAYO - JUNIN Fecha de Vencimiento Fecha de Emisión : 07/04/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Obser</t>
+        </is>
+      </c>
       <c r="R9" s="5" t="inlineStr"/>
       <c r="S9" s="5" t="inlineStr"/>
+      <c r="T9" s="5" t="inlineStr"/>
+      <c r="U9" s="5" t="inlineStr"/>
+      <c r="V9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DEBEDSAR2026-INT-0103251</t>
+          <t>DIED2026-INT-0344746</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>27</v>
+        <v>54</v>
       </c>
       <c r="D10" t="n">
-        <v>27</v>
+        <v>54</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>factura_electronica</t>
+          <t>boleta_venta</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>20611798637</t>
+          <t>10449028673</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>E T M TOURS PUQUIO-NASCA S.A.C.</t>
+          <t>MANZANARES NUÑEZ EDUARD ADOLFO</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>E001-324</t>
+          <t>EB01-1277</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -2826,65 +2940,76 @@
           <t>0.00</t>
         </is>
       </c>
-      <c r="M10" t="n">
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
         <v>1</v>
       </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>E T M TOURS PUQUIO-NASCA SOCIEDAD ANONIMA CERRADA JR. OCAÑA SIN NUMERO SEGUNDA SN PUQUIO - LUCANAS - AYACUCHO FACTURA ELECTRONICA RUC: 20611798637 E001-324 Fecha de Emisión : 08/02/2026 Señor(es) : PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 Establecimiento del Emisor : JR. OCAÃ‘A SIN NUM</t>
-        </is>
-      </c>
-      <c r="O10" s="5" t="inlineStr"/>
-      <c r="P10" s="5" t="inlineStr"/>
-      <c r="Q10" s="5" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>HEM - BOLETA DE VENTA ELECTRONICA MANZANARES NUNEZ EDUARD ADOLFO RUC: 10449028673 AV. PALIAN 545 HUANCAYO - HUANCAYO - JUNIN EB01-1277 Fecha de Vencimiento Fecha de Emisión : 07/04/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Observación : Señor(es) Cantidad</t>
+        </is>
+      </c>
       <c r="R10" s="5" t="inlineStr"/>
       <c r="S10" s="5" t="inlineStr"/>
+      <c r="T10" s="5" t="inlineStr"/>
+      <c r="U10" s="5" t="inlineStr"/>
+      <c r="V10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DEBEDSAR2026-INT-0103251</t>
+          <t>DIED2026-INT-0344746</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>202604101137186103251RENDICIONCORREGIDADECARLOSA.pdf</t>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="D11" t="n">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>factura_electronica</t>
+          <t>boleta_venta</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>20606737310</t>
+          <t>10427147491</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>MULTISERVICIOS ASIEL S.A.C.</t>
+          <t>HILARIO FLORES JORGE LUIS</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>E001-2203</t>
+          <t>EB01-1428</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>35.00</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -2894,25 +3019,1632 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>5.34</t>
-        </is>
-      </c>
-      <c r="M11" t="n">
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
         <v>1</v>
       </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>MULTISERVICIOS ASIEL S.A.C. MULTISERVICIOS ASIEL S.A.C. C.P. SIN BARRIO COMATRANA MZA. Q LOTE. 18 CP. COMATRANA ICA - ICA - ICA FACTURA ELECTRONICA RUC: 20606737310 E001-2203 Fecha de Emisión : 08/02/2026 Señor(es) : PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 Dirección del Cliente : CAL.</t>
-        </is>
-      </c>
-      <c r="O11" s="5" t="inlineStr"/>
-      <c r="P11" s="5" t="inlineStr"/>
-      <c r="Q11" s="5" t="inlineStr"/>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BOLETA DE VENTA ELECTRONICA HILARIO FLORES JORGE LUIS RUC: 10427147491 JR. PARAMONGA 121 ENTRE INTIHUATANA Y AV.CIRCUNVALACION EB01-1428 EL TAMBO - HUANCAYO - JUNIN - Fecha de Vencimiento Fecha de Emisión : 07/04/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES </t>
+        </is>
+      </c>
       <c r="R11" s="5" t="inlineStr"/>
       <c r="S11" s="5" t="inlineStr"/>
+      <c r="T11" s="5" t="inlineStr"/>
+      <c r="U11" s="5" t="inlineStr"/>
+      <c r="V11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>62</v>
+      </c>
+      <c r="D12" t="n">
+        <v>62</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>10200513237</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>PUCUHUANCA HUAMAN AGAPITO E</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>FP01-390</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>200.00</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>181.00</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>* HOTEL* ROGGER De : PUCUHUANCA HUAMAN AGAPITO E JR ANCASH N* 460 HUANCAYO - HUANCAYO - JUNIN RUC:10200513237 TELF: 07/04/2026 07:54:57 FACTURA ELECTRONICA FP01 0000000390 TIPO DE PAGO: CONTADO RUC: 20380795907 NOMBRE: PROGRAMA EDUCACION BASICA PARA TODOS DIRECCION: CAL. DEL COMERCIO NRO. 193 RES. L</t>
+        </is>
+      </c>
+      <c r="R12" s="5" t="inlineStr"/>
+      <c r="S12" s="5" t="inlineStr"/>
+      <c r="T12" s="5" t="inlineStr"/>
+      <c r="U12" s="5" t="inlineStr"/>
+      <c r="V12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>66</v>
+      </c>
+      <c r="D13" t="n">
+        <v>66</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>10200513237</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>PUCUHUANCA HUAMAN AGAPITO E</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>FP01-391</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>100.00</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>90.50</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">* HOTEL* ROGGER De : PUCUHUANCA HUAMAN AGAPITO E JR ANCASH N* 460 HUANCAYO - HUANCAYO - JUNIN RUC:10200513237 TELF: 08/04/2026 10:28:35 FACTURA ELECTRONICA FP0O1 0000000391 TIPO DE PAGO: CONTADO RUC: 20380795907 NOMBRE: PROGRAMA EDUCACION BASICA PARA TODOS DIRECCION: CAL. DEL COMERCIO NRO. 193 RES. </t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="inlineStr"/>
+      <c r="S13" s="5" t="inlineStr"/>
+      <c r="T13" s="5" t="inlineStr"/>
+      <c r="U13" s="5" t="inlineStr"/>
+      <c r="V13" s="5" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>70</v>
+      </c>
+      <c r="D14" t="n">
+        <v>70</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>20380795907</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>BALTAZAR GALLARDO MARIA ELENA</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>E001-40</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>BALTAZAR GALLARDO MARIA ELENA BALTAZAR GALLARDO MARIA ELENA AV. MARGINAL SN URB. MIRAFORES S81451524 COST LLANTERIA EL APOLO SAN RAMON - CHANCHAMAYO - JUNIN Formato de Pago’: Al Contado Fecha de Emisión :08/04/2026 Señor (es) ‘PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380795907 Tipo de Moneda FAC</t>
+        </is>
+      </c>
+      <c r="R14" s="5" t="inlineStr"/>
+      <c r="S14" s="5" t="inlineStr"/>
+      <c r="T14" s="5" t="inlineStr"/>
+      <c r="U14" s="5" t="inlineStr"/>
+      <c r="V14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>74</v>
+      </c>
+      <c r="D15" t="n">
+        <v>74</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>20610937471</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>AISHALE SOCIEDAD ANONIMA CERRADA</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>FF02-1001</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>AISHALE SOCIEDAD ANONIMA RUC N*: 20610937471 CERRADA FACTURA ELECTRONICA CAL.SANTO TOMAS NRO. 359 URB. SANTO TOMAS FF02-00001001 (S.72406163) JUNIN - CHANCHAMAYO - CHANCHAMAYO 000000000 F. EMISIÓN: 8/04/2026 19:29:33 SEÑOR (ES): PROGRAMA EDUCACION BASICA PARA TODOS R.U.C./D.N.I.: 20380795907 CAL. DE</t>
+        </is>
+      </c>
+      <c r="R15" s="5" t="inlineStr"/>
+      <c r="S15" s="5" t="inlineStr"/>
+      <c r="T15" s="5" t="inlineStr"/>
+      <c r="U15" s="5" t="inlineStr"/>
+      <c r="V15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>78</v>
+      </c>
+      <c r="D16" t="n">
+        <v>78</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>10207416067</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>BALTAZAR GALLARDO MARIA ELENA</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>E001-38</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>BALTAZAR GALLARDO MARIA ELENA BALTAZAR GALLARDO MARIA ELENA AV. MARGINAL SN URB. MIRAFORES S81451524 COST LLANTERIA EL APOLO SAN RAMON - CHANCHAMAYO - JUNIN Formato de Pago’: Al Contado Fecha de Emisión :08/04/2026 FACTURA ELECTRÓNICA RUC:10207416067 E001-38 :SOLES Valor Unitario 20.00 10.00 Señor (</t>
+        </is>
+      </c>
+      <c r="R16" s="5" t="inlineStr"/>
+      <c r="S16" s="5" t="inlineStr"/>
+      <c r="T16" s="5" t="inlineStr"/>
+      <c r="U16" s="5" t="inlineStr"/>
+      <c r="V16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>82</v>
+      </c>
+      <c r="D17" t="n">
+        <v>82</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>20380795907</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>MACASSI FRANCIA TALIA ABIGAID</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>E001-1273</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>ALTAÑA GRILL MACASSI FRANCIA TALIA ABIGAID raat panned pia JR. AREQUIPA S/N URB. LA MERCED ESQ. CON JR 2 DE MAYO E001 1273 CHANCHAMAYO - CHANCHAMAYO - JUNIN - Fecha de Emisión : 08/04/2026 Forma de pago: Contado . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 CAL. DEL COMERCIO 193 RES. LA</t>
+        </is>
+      </c>
+      <c r="R17" s="5" t="inlineStr"/>
+      <c r="S17" s="5" t="inlineStr"/>
+      <c r="T17" s="5" t="inlineStr"/>
+      <c r="U17" s="5" t="inlineStr"/>
+      <c r="V17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>86</v>
+      </c>
+      <c r="D18" t="n">
+        <v>86</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>10407833037</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>ESPIRITU VALENTIN ELIZABETH KEYLI</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>EB01-712</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>40.00</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>40.00</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>ESPIRITU VALENTIN ELIZABETH KEYLI BOLETA ELECTRÓNICA ESPIRITU VALENTIN ELIZABETH KEYLI RUC :10407833037 EB01 - 712 CAL. DARIO LEON 175 SEC. OROYA — ANTIGUA COSTADO DE I.E. NTRA SENORA LA OROYA - YAULI - JUNIN Fecha de Emisión : 09/04/2026 Señor (es) : PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380</t>
+        </is>
+      </c>
+      <c r="R18" s="5" t="inlineStr"/>
+      <c r="S18" s="5" t="inlineStr"/>
+      <c r="T18" s="5" t="inlineStr"/>
+      <c r="U18" s="5" t="inlineStr"/>
+      <c r="V18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>90</v>
+      </c>
+      <c r="D19" t="n">
+        <v>90</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>20402248824</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>RESTAURANT MARISQUERIA MICHELIN SA</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>F001-35094</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-64-09</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="Q19" s="2" t="inlineStr">
+        <is>
+          <t>RESTAURANT MICHELIN SA RESTAURANT MARTSQUERTA MICHELIN SA AV. MIGUEL NRO. 1027 CHUCCHTS (COSTADO D E RES CTAL) JUNIN - VAULT - SANTA ROSA D E SACCO RUC: 20402248824 TELE: (064)391627 CAJA: DESKTOP-8TL21UH FACTURA DE VENTA ELECTRONICA £001-35094 09/64/2026 02:54:39 PM MESA: 19 MOZO: ISABEL PERS: 1 PT</t>
+        </is>
+      </c>
+      <c r="R19" s="5" t="inlineStr"/>
+      <c r="S19" s="5" t="inlineStr"/>
+      <c r="T19" s="5" t="inlineStr"/>
+      <c r="U19" s="5" t="inlineStr"/>
+      <c r="V19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>94</v>
+      </c>
+      <c r="D20" t="n">
+        <v>94</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>20607154521</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>FT CHINA SOCIEDAD ANONIMA CERRADA</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>F001-00014500</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>19.00</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>CHIFA YUFU FT CHINA S.A.C 20607154521 AV. GIRALDEZ NRO. 208 HUANCAYO CERCADO JUNIN - HUANCAYO - HUANCAYO .................................................................... FACTURA ELECTRONICA F001-00014500 09-04-2026 19'38'07 PARA TODOS RUC/DNI: 20380795907 DIRE.: CAL.DELCOMERCIONRO.193RES. LASTOR</t>
+        </is>
+      </c>
+      <c r="R20" s="5" t="inlineStr"/>
+      <c r="S20" s="5" t="inlineStr"/>
+      <c r="T20" s="5" t="inlineStr"/>
+      <c r="U20" s="5" t="inlineStr"/>
+      <c r="V20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>98</v>
+      </c>
+      <c r="D21" t="n">
+        <v>98</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>10407833037</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>ESPIRITU VALENTIN ELIZABETH KEYLI</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>EB01-711</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>60.00</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>60.00</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q21" s="2" t="inlineStr">
+        <is>
+          <t>ESPIRITU VALENTIN ELIZABETH KEYLI BOLETA ELECTRÓNICA ESPIRITU VALENTIN ELIZABETH KEYLI RUC :10407833037 EB01 - 711 CAL. DARIO LEON 175 SEC. OROYA — ANTIGUA COSTADO DE I.E. NTRA SENORA LA OROYA - YAULI - JUNIN Fecha de Emisión : 09/04/2026 Señor (es) : PROGRAMA EDUCACION BASICA PARA TODOS RUC : 20380</t>
+        </is>
+      </c>
+      <c r="R21" s="5" t="inlineStr"/>
+      <c r="S21" s="5" t="inlineStr"/>
+      <c r="T21" s="5" t="inlineStr"/>
+      <c r="U21" s="5" t="inlineStr"/>
+      <c r="V21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>102</v>
+      </c>
+      <c r="D22" t="n">
+        <v>102</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>20487317242</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>LAS BRASAS D´MICHELINN SOCIEDAD ANONIMA CERRADA-</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>E001-7319</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>110.00</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>99.55</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9/4/26, 0:12 .:: Factura Electronica - Impresion ::. FACTURA ELECTRONICA RUC: 20487317242 E001-7319 LAS BRASAS D ' MICHELINN SOCIEDAD ANONIMA CERRADA-LAS BRASAS D “ MICHELINN S.A.C. AV. MIGUEL GRAU 1029 SEC. SANTA ROSA DE SACCO SANTA ROSA DE SACCO - YAULI - JUNIN Fecha de Emisión : 09/04/2026 Forma </t>
+        </is>
+      </c>
+      <c r="R22" s="5" t="inlineStr"/>
+      <c r="S22" s="5" t="inlineStr"/>
+      <c r="T22" s="5" t="inlineStr"/>
+      <c r="U22" s="5" t="inlineStr"/>
+      <c r="V22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>106</v>
+      </c>
+      <c r="D23" t="n">
+        <v>106</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>boleta_venta</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>10715562681</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>SORIANO ACLARI DIANA</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>EB01-2355</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>60.00</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q23" s="2" t="inlineStr">
+        <is>
+          <t>BOLETA DE VENTA ELECTRONICA RUC: 10715562681 EB01-2355 SORIANO ACLARI DIANA AV. AV.HUAYTAPALLANA 1201 AL FRENTE DE UNA LOZA DEPORTIVA EL TAMBO - HUANCAYO - JUNIN Fecha de Vencimiento Fecha de Emisión : 10/04/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Obser</t>
+        </is>
+      </c>
+      <c r="R23" s="5" t="inlineStr"/>
+      <c r="S23" s="5" t="inlineStr"/>
+      <c r="T23" s="5" t="inlineStr"/>
+      <c r="U23" s="5" t="inlineStr"/>
+      <c r="V23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>110</v>
+      </c>
+      <c r="D24" t="n">
+        <v>110</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>boleta_venta</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>10449028673</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>MANZANARES NUÑEZ EDUARD ADOLFO</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>EB01-1305</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>40.00</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>HEM - BOLETA DE VENTA ELECTRONICA MANZANARES NUNEZ EDUARD ADOLFO RUC: 10449028673 AV. PALIAN 545 HUANCAYO - HUANCAYO - JUNIN EB01-1305 Fecha de Vencimiento Fecha de Emisión : 10/04/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Observación : POR ALIMENTOS Cant</t>
+        </is>
+      </c>
+      <c r="R24" s="5" t="inlineStr"/>
+      <c r="S24" s="5" t="inlineStr"/>
+      <c r="T24" s="5" t="inlineStr"/>
+      <c r="U24" s="5" t="inlineStr"/>
+      <c r="V24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>114</v>
+      </c>
+      <c r="D25" t="n">
+        <v>114</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>boleta_venta</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>10427147491</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>HILARIO FLORES JORGE LUIS</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>EB01-1452</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>20.00</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>70.00</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q25" s="2" t="inlineStr">
+        <is>
+          <t>BOLETA DE VENTA ELECTRONICA RUC: 10427147491 EB01-1452 HILARIO FLORES JORGE LUIS JR. PARAMONGA 121 ENTRE INTIHUATANA Y AV.CIRCUNVALACION EL TAMBO - HUANCAYO - JUNIN Fecha de Vencimiento Fecha de Emisión : 10/04/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Ob</t>
+        </is>
+      </c>
+      <c r="R25" s="5" t="inlineStr"/>
+      <c r="S25" s="5" t="inlineStr"/>
+      <c r="T25" s="5" t="inlineStr"/>
+      <c r="U25" s="5" t="inlineStr"/>
+      <c r="V25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>118</v>
+      </c>
+      <c r="D26" t="n">
+        <v>118</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>boleta_venta</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>10722590428</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>GRANADOS RAMOS INGRID MARGOT</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>EB01-49</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>13.00</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>PINKI SWEET PASTRIES GRANADOS RAMOS INGRID MARGOT JR. AYACUCHO 288 COSTADO DE IE SEBASTIAN LORENTE HUANCAYO - HUANCAYO - JUNIN BOLETA DE VENTA ELECTRONICA RUC: 10722590428 EB01-49 Fecha de Vencimiento Fecha de Emisión : 10/04/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Mo</t>
+        </is>
+      </c>
+      <c r="R26" s="5" t="inlineStr"/>
+      <c r="S26" s="5" t="inlineStr"/>
+      <c r="T26" s="5" t="inlineStr"/>
+      <c r="U26" s="5" t="inlineStr"/>
+      <c r="V26" s="5" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>122</v>
+      </c>
+      <c r="D27" t="n">
+        <v>122</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>boleta_venta</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>10715562681</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>SORIANO ACLARI DIANA</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>EB01-2358</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>65.00</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q27" s="2" t="inlineStr">
+        <is>
+          <t>BOLETA DE VENTA ELECTRONICA SORIANO ACLARI DIANA RUC: 10715562681 AV. AV.HUAYTAPALLANA 1201 AL FRENTE DE UNA LOZA DEPORTIVA EL TAMBO - HUANCAYO - JUNIN EB01-2358 Fecha de Vencimiento Fecha de Emisión : 11/04/2026 . PROGRAMA EDUCACION BASICA " PARA TODOS RUC : 20380795907 Tipo de Moneda : SOLES Obser</t>
+        </is>
+      </c>
+      <c r="R27" s="5" t="inlineStr"/>
+      <c r="S27" s="5" t="inlineStr"/>
+      <c r="T27" s="5" t="inlineStr"/>
+      <c r="U27" s="5" t="inlineStr"/>
+      <c r="V27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>126</v>
+      </c>
+      <c r="D28" t="n">
+        <v>126</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>20380795907</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>ANFLOR SERVICE S.A.C.</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>F001-00000767</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>100.00</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>100.00</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q28" s="2" t="inlineStr">
+        <is>
+          <t>R.U.C. N° 20613343700 ANFLOR SERVICE S.A.C. a JR. ALFONSO UGARTE MZ. 2G LT. 24 P.J. JOSE OLAYA FACTURA ELECTRONICA FLOR SERVICE 5. 5.7 CALLAO PROV. CONST. DEL CALLAO PROV, CONST. DEL ili F001-00000767 RAZÓN SOCIAL: PROGRAMA EDUCACION BASICA PARA TODOS RUC: 20380795907 DIRECCION: CAL. DEL COMERCIO NR</t>
+        </is>
+      </c>
+      <c r="R28" s="5" t="inlineStr"/>
+      <c r="S28" s="5" t="inlineStr"/>
+      <c r="T28" s="5" t="inlineStr"/>
+      <c r="U28" s="5" t="inlineStr"/>
+      <c r="V28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>130</v>
+      </c>
+      <c r="D29" t="n">
+        <v>130</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>10425467188</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>ROJAS CHUQUILLANQUI JESUS MAEL</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>E001-2634</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>60.00</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>60.00</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q29" s="2" t="inlineStr">
+        <is>
+          <t>ROJAS CHUQUILLANQUI JESUS MAEL FACTU RA ELECTRONICA ROJAS CHUQUILLANQUI JESUS MAEL . RUC:10425467188 JR. PUCATEA 904 C.P.M UNAS 2 CDR ANT D PLANTA D TRATAMIENT D SEDAM E001 -2634 HUANCAYO - HUANCAYO - JUNIN Formato de Pago’: Al Contado Fecha de Emisión § : 11/04/2026 Señor (es) ‘PROGRAMA EDUCACION B</t>
+        </is>
+      </c>
+      <c r="R29" s="5" t="inlineStr"/>
+      <c r="S29" s="5" t="inlineStr"/>
+      <c r="T29" s="5" t="inlineStr"/>
+      <c r="U29" s="5" t="inlineStr"/>
+      <c r="V29" s="5" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>134</v>
+      </c>
+      <c r="D30" t="n">
+        <v>134</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>10200513237</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>PUCUHUANCA HUAMAN AGAPITO E</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>FP01-395</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>200.00</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q30" s="2" t="inlineStr">
+        <is>
+          <t>+ HOTEL+ ROGGER De : PUCUHUANCA HUAMAN AGAPITO E JR ANCASH N* 460 HUANCAYO HUANCAYO - JUNIN RUC:10200513237 TELT: 11/04/2026 10:43:08 FACTURA ELECTRONICA TIPO DE PAGO: CONTADO RUC: 20380795907 NOMBRE: PROGRAMA EDUCACION BASICA PARA TODOS DIRECCION: CAL. DEL COMERCIO NRO. 193 RES. LAS TORRES DE SAN B</t>
+        </is>
+      </c>
+      <c r="R30" s="5" t="inlineStr"/>
+      <c r="S30" s="5" t="inlineStr"/>
+      <c r="T30" s="5" t="inlineStr"/>
+      <c r="U30" s="5" t="inlineStr"/>
+      <c r="V30" s="5" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>138</v>
+      </c>
+      <c r="D31" t="n">
+        <v>138</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>20486048035</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>EMPRESA DE TRANSPORTES CRUZ MORADO SCRL</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>FF01-5730</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="Q31" s="2" t="inlineStr">
+        <is>
+          <t>~~ EMPRESA DE TRANSPORTES CRUZ MORADO SRL RUC 20486048035 PRINCIPAL » JR. BOLOGNESI NRO. 1942 - JUNIN FACTURA HUANCAYO EL TAMBO SUCURSAL TERMINAL LOS ñ Ne ELECTRONICA Empresa de transportes Cruz Morado scrl - = Cel: 965668080 FFO1-0005730 DOCUMENTO RUC 20380795907 FECHA EMISION 09/04/2026 CLIENTE PR</t>
+        </is>
+      </c>
+      <c r="R31" s="5" t="inlineStr"/>
+      <c r="S31" s="5" t="inlineStr"/>
+      <c r="T31" s="5" t="inlineStr"/>
+      <c r="U31" s="5" t="inlineStr"/>
+      <c r="V31" s="5" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>142</v>
+      </c>
+      <c r="D32" t="n">
+        <v>142</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>20486048035</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>EMPRESA DE TRANSPORTES CRUZ MORADO SCRL</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>FF02-46</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="Q32" s="2" t="inlineStr">
+        <is>
+          <t>~~ EMPRESA DE TRANSPORTES RUC 20486048035 CRUZ MORADO » JR. BOLOGNESI NRO. 1942 - FACTURA JUNIN HUANCAYO EL TAMBO SUCURSAL TERMINAL á NN EA ELECTRÓNICA Empresa de transportes Cruz Morado scrl - = Cel: 965668080 FF02-0000046 DOCUMENTO RUC 20380795907 FECHA EMISIÓN 08/04/2026 CLIENTE PROGRAMA EDUCACIO</t>
+        </is>
+      </c>
+      <c r="R32" s="5" t="inlineStr"/>
+      <c r="S32" s="5" t="inlineStr"/>
+      <c r="T32" s="5" t="inlineStr"/>
+      <c r="U32" s="5" t="inlineStr"/>
+      <c r="V32" s="5" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>DIED2026-INT-0344746</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>20260416143823RENDICIONVICTORCHAVEZJUNINSINAD.pdf</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>146</v>
+      </c>
+      <c r="D33" t="n">
+        <v>146</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>factura_electronica</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>20486048035</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>EMPRESA DE TRANSPORTES CRUZ MORADO SCRL</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>FF01-5711</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="Q33" s="2" t="inlineStr">
+        <is>
+          <t>~~ EMPRESA DE TRANSPORTES CRUZ MORADO SRL RUC 20486048035 PRINCIPAL » JR. BOLOGNESI NRO. 1942 - JUNIN FACTURA HUANCAYO EL TAMBO SUCURSAL TERMINAL LOS ñ Ne ELECTRONICA Empresa de transportes Cruz Morado scrl - = Cel: 965668080 FFO1-0005711 DOCUMENTO RUC 20380795907 FECHA EMISION 08/04/2026 CLIENTE PR</t>
+        </is>
+      </c>
+      <c r="R33" s="5" t="inlineStr"/>
+      <c r="S33" s="5" t="inlineStr"/>
+      <c r="T33" s="5" t="inlineStr"/>
+      <c r="U33" s="5" t="inlineStr"/>
+      <c r="V33" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S11"/>
+  <autoFilter ref="A1:V33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>